<commit_message>
JO: restore the underline rules (keep underscore rows overflowing)
The prior exceljs re-save centered the underscore 'line' rows, so they no
longer overflowed into a rule. Revert to the pristine template and redo
concat+centre in one pass that explicitly left-aligns the underscore rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HNv2pt2j3pqxEC7sBHUC3k
</commit_message>
<xml_diff>
--- a/public/templates/fans-jo-template.xlsx
+++ b/public/templates/fans-jo-template.xlsx
@@ -856,7 +856,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -888,6 +888,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="12" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1517,7 +1520,7 @@
         <v>4</v>
       </c>
       <c r="D14" s="6"/>
-      <c r="R14" t="s">
+      <c r="R14" s="5" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1552,7 +1555,7 @@
       <c r="V15" s="7"/>
     </row>
     <row r="16" ht="5" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C16" t="s">
+      <c r="C16" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1660,7 +1663,7 @@
         <v>19</v>
       </c>
       <c r="P36" s="3"/>
-      <c r="Q36" s="3" t="s">
+      <c r="Q36" s="13" t="s">
         <v>2</v>
       </c>
       <c r="R36" s="3" t="str">
@@ -1672,40 +1675,40 @@
       <c r="U36" s="6"/>
       <c r="V36" s="6"/>
       <c r="W36" s="6"/>
-      <c r="X36" s="3"/>
+      <c r="X36" s="13"/>
     </row>
     <row r="37" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="3" t="s">
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
-      <c r="J37" s="3"/>
-      <c r="K37" s="3"/>
-      <c r="L37" s="3"/>
-      <c r="M37" s="3"/>
-      <c r="N37" s="3"/>
-      <c r="O37" s="3"/>
-      <c r="P37" s="3"/>
-      <c r="Q37" s="3"/>
-      <c r="R37" s="3" t="s">
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
+      <c r="G37" s="13"/>
+      <c r="H37" s="13"/>
+      <c r="I37" s="13"/>
+      <c r="J37" s="13"/>
+      <c r="K37" s="13"/>
+      <c r="L37" s="13"/>
+      <c r="M37" s="13"/>
+      <c r="N37" s="13"/>
+      <c r="O37" s="13"/>
+      <c r="P37" s="13"/>
+      <c r="Q37" s="13"/>
+      <c r="R37" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="S37" s="3"/>
-      <c r="T37" s="3"/>
-      <c r="U37" s="3"/>
-      <c r="V37" s="3"/>
-      <c r="W37" s="3"/>
-      <c r="X37" s="3"/>
+      <c r="S37" s="13"/>
+      <c r="T37" s="13"/>
+      <c r="U37" s="13"/>
+      <c r="V37" s="13"/>
+      <c r="W37" s="13"/>
+      <c r="X37" s="13"/>
     </row>
     <row r="38" ht="18" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A38" s="13" t="s">
+      <c r="A38" s="14" t="s">
         <v>22</v>
       </c>
       <c r="B38" s="12" t="s">
@@ -1730,7 +1733,7 @@
         <v>23</v>
       </c>
       <c r="P38" s="3"/>
-      <c r="Q38" s="3" t="s">
+      <c r="Q38" s="13" t="s">
         <v>2</v>
       </c>
       <c r="R38" s="3" t="str">
@@ -1742,40 +1745,40 @@
       <c r="U38" s="6"/>
       <c r="V38" s="6"/>
       <c r="W38" s="6"/>
-      <c r="X38" s="3"/>
+      <c r="X38" s="13"/>
     </row>
     <row r="39" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A39" s="13"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="3" t="s">
+      <c r="A39" s="14"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
-      <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
-      <c r="K39" s="3"/>
-      <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
-      <c r="N39" s="3"/>
-      <c r="O39" s="3"/>
-      <c r="P39" s="3"/>
-      <c r="Q39" s="3"/>
-      <c r="R39" s="3" t="s">
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="13"/>
+      <c r="H39" s="13"/>
+      <c r="I39" s="13"/>
+      <c r="J39" s="13"/>
+      <c r="K39" s="13"/>
+      <c r="L39" s="13"/>
+      <c r="M39" s="13"/>
+      <c r="N39" s="13"/>
+      <c r="O39" s="13"/>
+      <c r="P39" s="13"/>
+      <c r="Q39" s="13"/>
+      <c r="R39" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="S39" s="3"/>
-      <c r="T39" s="3"/>
-      <c r="U39" s="3"/>
-      <c r="V39" s="3"/>
-      <c r="W39" s="3"/>
-      <c r="X39" s="3"/>
+      <c r="S39" s="13"/>
+      <c r="T39" s="13"/>
+      <c r="U39" s="13"/>
+      <c r="V39" s="13"/>
+      <c r="W39" s="13"/>
+      <c r="X39" s="13"/>
     </row>
     <row r="40" ht="18" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A40" s="13" t="s">
+      <c r="A40" s="14" t="s">
         <v>24</v>
       </c>
       <c r="B40" s="12" t="s">
@@ -1803,39 +1806,39 @@
       <c r="T40" s="3"/>
       <c r="U40" s="3"/>
       <c r="V40" s="3"/>
-      <c r="W40" s="3"/>
-      <c r="X40" s="3"/>
+      <c r="W40" s="13"/>
+      <c r="X40" s="13"/>
     </row>
     <row r="41" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A41" s="13"/>
-      <c r="B41" s="13"/>
-      <c r="C41" s="3" t="s">
+      <c r="A41" s="14"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
-      <c r="F41" s="3"/>
-      <c r="G41" s="3"/>
-      <c r="H41" s="3"/>
-      <c r="I41" s="3"/>
-      <c r="J41" s="3"/>
-      <c r="K41" s="3"/>
-      <c r="L41" s="3"/>
-      <c r="M41" s="3"/>
-      <c r="N41" s="3"/>
-      <c r="O41" s="3"/>
-      <c r="P41" s="3"/>
-      <c r="Q41" s="3"/>
-      <c r="R41" s="3"/>
-      <c r="S41" s="3"/>
-      <c r="T41" s="3"/>
-      <c r="U41" s="3"/>
-      <c r="V41" s="3"/>
-      <c r="W41" s="3"/>
-      <c r="X41" s="3"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="13"/>
+      <c r="J41" s="13"/>
+      <c r="K41" s="13"/>
+      <c r="L41" s="13"/>
+      <c r="M41" s="13"/>
+      <c r="N41" s="13"/>
+      <c r="O41" s="13"/>
+      <c r="P41" s="13"/>
+      <c r="Q41" s="13"/>
+      <c r="R41" s="13"/>
+      <c r="S41" s="13"/>
+      <c r="T41" s="13"/>
+      <c r="U41" s="13"/>
+      <c r="V41" s="13"/>
+      <c r="W41" s="13"/>
+      <c r="X41" s="13"/>
     </row>
     <row r="42" ht="18" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="14" t="s">
         <v>26</v>
       </c>
       <c r="B42" s="12" t="s">
@@ -1863,216 +1866,216 @@
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
       <c r="V42" s="3"/>
-      <c r="W42" s="3"/>
-      <c r="X42" s="3"/>
+      <c r="W42" s="13"/>
+      <c r="X42" s="13"/>
     </row>
     <row r="43" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A43" s="13"/>
-      <c r="B43" s="13"/>
-      <c r="C43" s="3" t="s">
+      <c r="A43" s="14"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
-      <c r="F43" s="3"/>
-      <c r="G43" s="3"/>
-      <c r="H43" s="3"/>
-      <c r="I43" s="3"/>
-      <c r="J43" s="3"/>
-      <c r="K43" s="3"/>
-      <c r="L43" s="3"/>
-      <c r="M43" s="3"/>
-      <c r="N43" s="3"/>
-      <c r="O43" s="3"/>
-      <c r="P43" s="3"/>
-      <c r="Q43" s="3"/>
-      <c r="R43" s="3"/>
-      <c r="S43" s="3"/>
-      <c r="T43" s="3"/>
-      <c r="U43" s="3"/>
-      <c r="V43" s="3"/>
-      <c r="W43" s="3"/>
-      <c r="X43" s="3"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
+      <c r="H43" s="13"/>
+      <c r="I43" s="13"/>
+      <c r="J43" s="13"/>
+      <c r="K43" s="13"/>
+      <c r="L43" s="13"/>
+      <c r="M43" s="13"/>
+      <c r="N43" s="13"/>
+      <c r="O43" s="13"/>
+      <c r="P43" s="13"/>
+      <c r="Q43" s="13"/>
+      <c r="R43" s="13"/>
+      <c r="S43" s="13"/>
+      <c r="T43" s="13"/>
+      <c r="U43" s="13"/>
+      <c r="V43" s="13"/>
+      <c r="W43" s="13"/>
+      <c r="X43" s="13"/>
     </row>
     <row r="44" ht="18" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A44" s="13" t="s">
+      <c r="A44" s="14" t="s">
         <v>27</v>
       </c>
       <c r="B44" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C44" s="14">
+      <c r="C44" s="15">
         <f>TRIM(TEXT(Source!D87,"# ?/?"))&amp;" HP,  "&amp;Source!D88&amp;" PH,  "&amp;Source!B90&amp;" V,  "&amp;Source!B91&amp;" Hz,  "&amp;Source!D90&amp;" pole,  "&amp;Source!D89&amp;" rpm,  "&amp;Source!B92&amp;",  "&amp;Source!B87&amp;",  "&amp;Source!B93</f>
       </c>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
-      <c r="H44" s="14"/>
-      <c r="I44" s="14"/>
-      <c r="J44" s="14"/>
-      <c r="K44" s="14"/>
-      <c r="L44" s="14"/>
-      <c r="M44" s="14"/>
-      <c r="N44" s="14"/>
-      <c r="O44" s="14"/>
-      <c r="P44" s="14"/>
-      <c r="Q44" s="14"/>
-      <c r="R44" s="14"/>
-      <c r="S44" s="14"/>
-      <c r="T44" s="14"/>
-      <c r="U44" s="14"/>
-      <c r="V44" s="14"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="15"/>
+      <c r="I44" s="15"/>
+      <c r="J44" s="15"/>
+      <c r="K44" s="15"/>
+      <c r="L44" s="15"/>
+      <c r="M44" s="15"/>
+      <c r="N44" s="15"/>
+      <c r="O44" s="15"/>
+      <c r="P44" s="15"/>
+      <c r="Q44" s="15"/>
+      <c r="R44" s="15"/>
+      <c r="S44" s="15"/>
+      <c r="T44" s="15"/>
+      <c r="U44" s="15"/>
+      <c r="V44" s="15"/>
     </row>
     <row r="45" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A45" s="13"/>
-      <c r="B45" s="13"/>
-      <c r="C45" s="3" t="s">
+      <c r="A45" s="14"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-      <c r="F45" s="3"/>
-      <c r="G45" s="3"/>
-      <c r="H45" s="3"/>
-      <c r="I45" s="3"/>
-      <c r="J45" s="3"/>
-      <c r="K45" s="3"/>
-      <c r="L45" s="3"/>
-      <c r="M45" s="3"/>
-      <c r="N45" s="3"/>
-      <c r="O45" s="3"/>
-      <c r="P45" s="3"/>
-      <c r="Q45" s="3"/>
-      <c r="R45" s="3"/>
-      <c r="S45" s="3"/>
-      <c r="T45" s="3"/>
-      <c r="U45" s="3"/>
-      <c r="V45" s="3"/>
-      <c r="W45" s="3"/>
-      <c r="X45" s="3"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="13"/>
+      <c r="F45" s="13"/>
+      <c r="G45" s="13"/>
+      <c r="H45" s="13"/>
+      <c r="I45" s="13"/>
+      <c r="J45" s="13"/>
+      <c r="K45" s="13"/>
+      <c r="L45" s="13"/>
+      <c r="M45" s="13"/>
+      <c r="N45" s="13"/>
+      <c r="O45" s="13"/>
+      <c r="P45" s="13"/>
+      <c r="Q45" s="13"/>
+      <c r="R45" s="13"/>
+      <c r="S45" s="13"/>
+      <c r="T45" s="13"/>
+      <c r="U45" s="13"/>
+      <c r="V45" s="13"/>
+      <c r="W45" s="13"/>
+      <c r="X45" s="13"/>
     </row>
     <row r="46" ht="18" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A46" s="13" t="s">
+      <c r="A46" s="14" t="s">
         <v>28</v>
       </c>
       <c r="B46" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C46" s="14">
+      <c r="C46" s="15">
         <f>TRIM(TEXT(Source!B96,"# ?/?"))&amp;""" Ø x "&amp;Source!D93&amp;" x "&amp;Source!D91&amp;" mm Ø bore x "&amp;Source!D92&amp;" mm keyway        "&amp;Source!D94&amp;" mm Ø Hub"</f>
       </c>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="14"/>
-      <c r="J46" s="14"/>
-      <c r="K46" s="14"/>
-      <c r="L46" s="14"/>
-      <c r="M46" s="14"/>
-      <c r="N46" s="14"/>
-      <c r="O46" s="14"/>
-      <c r="P46" s="14"/>
-      <c r="Q46" s="14"/>
-      <c r="R46" s="14"/>
-      <c r="S46" s="14"/>
-      <c r="T46" s="14"/>
-      <c r="U46" s="14"/>
-      <c r="V46" s="14"/>
-      <c r="X46" s="3"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="15"/>
+      <c r="I46" s="15"/>
+      <c r="J46" s="15"/>
+      <c r="K46" s="15"/>
+      <c r="L46" s="15"/>
+      <c r="M46" s="15"/>
+      <c r="N46" s="15"/>
+      <c r="O46" s="15"/>
+      <c r="P46" s="15"/>
+      <c r="Q46" s="15"/>
+      <c r="R46" s="15"/>
+      <c r="S46" s="15"/>
+      <c r="T46" s="15"/>
+      <c r="U46" s="15"/>
+      <c r="V46" s="15"/>
+      <c r="X46" s="13"/>
     </row>
     <row r="47" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A47" s="13"/>
-      <c r="B47" s="13"/>
-      <c r="C47" s="3" t="s">
+      <c r="A47" s="14"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
-      <c r="I47" s="3"/>
-      <c r="J47" s="3"/>
-      <c r="K47" s="3"/>
-      <c r="L47" s="3"/>
-      <c r="M47" s="3"/>
-      <c r="N47" s="3"/>
-      <c r="O47" s="3"/>
-      <c r="P47" s="3"/>
-      <c r="Q47" s="3"/>
-      <c r="R47" s="3"/>
-      <c r="S47" s="3"/>
-      <c r="T47" s="3"/>
-      <c r="U47" s="3"/>
-      <c r="V47" s="3"/>
-      <c r="W47" s="3"/>
-      <c r="X47" s="3"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="13"/>
+      <c r="F47" s="13"/>
+      <c r="G47" s="13"/>
+      <c r="H47" s="13"/>
+      <c r="I47" s="13"/>
+      <c r="J47" s="13"/>
+      <c r="K47" s="13"/>
+      <c r="L47" s="13"/>
+      <c r="M47" s="13"/>
+      <c r="N47" s="13"/>
+      <c r="O47" s="13"/>
+      <c r="P47" s="13"/>
+      <c r="Q47" s="13"/>
+      <c r="R47" s="13"/>
+      <c r="S47" s="13"/>
+      <c r="T47" s="13"/>
+      <c r="U47" s="13"/>
+      <c r="V47" s="13"/>
+      <c r="W47" s="13"/>
+      <c r="X47" s="13"/>
     </row>
     <row r="48" ht="18" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A48" s="13" t="s">
+      <c r="A48" s="14" t="s">
         <v>29</v>
       </c>
       <c r="B48" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C48" s="14">
+      <c r="C48" s="15">
         <f>TRIM(TEXT(Source!B97,"# ?/?"))&amp;""" Ø x "&amp;Source!D93&amp;" x "&amp;Source!D80&amp;"        "&amp;Source!D95&amp;" mm Ø Hub"</f>
       </c>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="14"/>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
-      <c r="L48" s="14"/>
-      <c r="M48" s="14"/>
-      <c r="N48" s="14"/>
-      <c r="O48" s="14"/>
-      <c r="P48" s="14"/>
-      <c r="Q48" s="14"/>
-      <c r="R48" s="14"/>
-      <c r="S48" s="14"/>
-      <c r="T48" s="14"/>
-      <c r="U48" s="14"/>
-      <c r="V48" s="14"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
+      <c r="I48" s="15"/>
+      <c r="J48" s="15"/>
+      <c r="K48" s="15"/>
+      <c r="L48" s="15"/>
+      <c r="M48" s="15"/>
+      <c r="N48" s="15"/>
+      <c r="O48" s="15"/>
+      <c r="P48" s="15"/>
+      <c r="Q48" s="15"/>
+      <c r="R48" s="15"/>
+      <c r="S48" s="15"/>
+      <c r="T48" s="15"/>
+      <c r="U48" s="15"/>
+      <c r="V48" s="15"/>
       <c r="W48" s="5"/>
-      <c r="X48" s="3"/>
+      <c r="X48" s="13"/>
     </row>
     <row r="49" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A49" s="13"/>
-      <c r="B49" s="13"/>
-      <c r="C49" s="3" t="s">
+      <c r="A49" s="14"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
-      <c r="J49" s="3"/>
-      <c r="K49" s="3"/>
-      <c r="L49" s="3"/>
-      <c r="M49" s="3"/>
-      <c r="N49" s="3"/>
-      <c r="O49" s="3"/>
-      <c r="P49" s="3"/>
-      <c r="Q49" s="3"/>
-      <c r="R49" s="3"/>
-      <c r="S49" s="3"/>
-      <c r="T49" s="3"/>
-      <c r="U49" s="3"/>
-      <c r="V49" s="3"/>
-      <c r="W49" s="3"/>
-      <c r="X49" s="3"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
+      <c r="H49" s="13"/>
+      <c r="I49" s="13"/>
+      <c r="J49" s="13"/>
+      <c r="K49" s="13"/>
+      <c r="L49" s="13"/>
+      <c r="M49" s="13"/>
+      <c r="N49" s="13"/>
+      <c r="O49" s="13"/>
+      <c r="P49" s="13"/>
+      <c r="Q49" s="13"/>
+      <c r="R49" s="13"/>
+      <c r="S49" s="13"/>
+      <c r="T49" s="13"/>
+      <c r="U49" s="13"/>
+      <c r="V49" s="13"/>
+      <c r="W49" s="13"/>
+      <c r="X49" s="13"/>
     </row>
     <row r="50" ht="18" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A50" s="13" t="s">
+      <c r="A50" s="14" t="s">
         <v>30</v>
       </c>
       <c r="B50" s="12" t="s">
@@ -2095,45 +2098,45 @@
       <c r="N50" s="3"/>
       <c r="O50" s="3"/>
       <c r="P50" s="3"/>
-      <c r="Q50" s="15"/>
-      <c r="R50" s="15"/>
-      <c r="S50" s="15"/>
-      <c r="T50" s="15"/>
-      <c r="U50" s="15"/>
-      <c r="V50" s="15"/>
-      <c r="W50" s="15"/>
-      <c r="X50" s="3"/>
+      <c r="Q50" s="16"/>
+      <c r="R50" s="16"/>
+      <c r="S50" s="16"/>
+      <c r="T50" s="16"/>
+      <c r="U50" s="16"/>
+      <c r="V50" s="16"/>
+      <c r="W50" s="16"/>
+      <c r="X50" s="13"/>
     </row>
     <row r="51" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A51" s="13"/>
-      <c r="B51" s="13"/>
-      <c r="C51" s="3" t="s">
+      <c r="A51" s="14"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
-      <c r="F51" s="3"/>
-      <c r="G51" s="3"/>
-      <c r="H51" s="3"/>
-      <c r="I51" s="3"/>
-      <c r="J51" s="3"/>
-      <c r="K51" s="3"/>
-      <c r="L51" s="3"/>
-      <c r="M51" s="3"/>
-      <c r="N51" s="3"/>
-      <c r="O51" s="3"/>
-      <c r="P51" s="3"/>
-      <c r="Q51" s="3"/>
-      <c r="R51" s="3"/>
-      <c r="S51" s="3"/>
-      <c r="T51" s="3"/>
-      <c r="U51" s="3"/>
-      <c r="V51" s="3"/>
-      <c r="W51" s="3"/>
-      <c r="X51" s="3"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="13"/>
+      <c r="F51" s="13"/>
+      <c r="G51" s="13"/>
+      <c r="H51" s="13"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="13"/>
+      <c r="K51" s="13"/>
+      <c r="L51" s="13"/>
+      <c r="M51" s="13"/>
+      <c r="N51" s="13"/>
+      <c r="O51" s="13"/>
+      <c r="P51" s="13"/>
+      <c r="Q51" s="13"/>
+      <c r="R51" s="13"/>
+      <c r="S51" s="13"/>
+      <c r="T51" s="13"/>
+      <c r="U51" s="13"/>
+      <c r="V51" s="13"/>
+      <c r="W51" s="13"/>
+      <c r="X51" s="13"/>
     </row>
     <row r="52" ht="18" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A52" s="13" t="s">
+      <c r="A52" s="14" t="s">
         <v>31</v>
       </c>
       <c r="B52" s="12" t="s">
@@ -2152,48 +2155,48 @@
       <c r="K52" s="5"/>
       <c r="L52" s="5"/>
       <c r="M52" s="5"/>
-      <c r="N52" s="3"/>
-      <c r="O52" s="3"/>
-      <c r="P52" s="3"/>
-      <c r="Q52" s="3"/>
-      <c r="R52" s="3"/>
-      <c r="S52" s="3"/>
-      <c r="T52" s="3"/>
-      <c r="U52" s="3"/>
-      <c r="V52" s="3"/>
-      <c r="W52" s="3"/>
-      <c r="X52" s="3"/>
+      <c r="N52" s="13"/>
+      <c r="O52" s="13"/>
+      <c r="P52" s="13"/>
+      <c r="Q52" s="13"/>
+      <c r="R52" s="13"/>
+      <c r="S52" s="13"/>
+      <c r="T52" s="13"/>
+      <c r="U52" s="13"/>
+      <c r="V52" s="13"/>
+      <c r="W52" s="13"/>
+      <c r="X52" s="13"/>
     </row>
     <row r="53" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A53" s="13"/>
-      <c r="B53" s="13"/>
-      <c r="C53" s="3" t="s">
+      <c r="A53" s="14"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="3"/>
-      <c r="H53" s="3"/>
-      <c r="I53" s="3"/>
-      <c r="J53" s="3"/>
-      <c r="K53" s="3"/>
-      <c r="L53" s="3"/>
-      <c r="M53" s="3"/>
-      <c r="N53" s="3"/>
-      <c r="O53" s="3"/>
-      <c r="P53" s="3"/>
-      <c r="Q53" s="3"/>
-      <c r="R53" s="3"/>
-      <c r="S53" s="3"/>
-      <c r="T53" s="3"/>
-      <c r="U53" s="3"/>
-      <c r="V53" s="3"/>
-      <c r="W53" s="3"/>
-      <c r="X53" s="3"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="13"/>
+      <c r="F53" s="13"/>
+      <c r="G53" s="13"/>
+      <c r="H53" s="13"/>
+      <c r="I53" s="13"/>
+      <c r="J53" s="13"/>
+      <c r="K53" s="13"/>
+      <c r="L53" s="13"/>
+      <c r="M53" s="13"/>
+      <c r="N53" s="13"/>
+      <c r="O53" s="13"/>
+      <c r="P53" s="13"/>
+      <c r="Q53" s="13"/>
+      <c r="R53" s="13"/>
+      <c r="S53" s="13"/>
+      <c r="T53" s="13"/>
+      <c r="U53" s="13"/>
+      <c r="V53" s="13"/>
+      <c r="W53" s="13"/>
+      <c r="X53" s="13"/>
     </row>
     <row r="54" ht="18" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A54" s="13" t="s">
+      <c r="A54" s="14" t="s">
         <v>32</v>
       </c>
       <c r="B54" s="12" t="s">
@@ -2206,52 +2209,52 @@
       <c r="G54"/>
       <c r="H54"/>
       <c r="I54"/>
-      <c r="J54" s="3"/>
-      <c r="K54" s="3"/>
-      <c r="L54" s="3"/>
-      <c r="M54" s="3"/>
-      <c r="N54" s="3"/>
-      <c r="O54" s="3"/>
-      <c r="P54" s="3"/>
-      <c r="Q54" s="3"/>
-      <c r="R54" s="3"/>
-      <c r="S54" s="3"/>
-      <c r="T54" s="3"/>
-      <c r="U54" s="3"/>
-      <c r="V54" s="3"/>
-      <c r="W54" s="3"/>
-      <c r="X54" s="3"/>
+      <c r="J54" s="13"/>
+      <c r="K54" s="13"/>
+      <c r="L54" s="13"/>
+      <c r="M54" s="13"/>
+      <c r="N54" s="13"/>
+      <c r="O54" s="13"/>
+      <c r="P54" s="13"/>
+      <c r="Q54" s="13"/>
+      <c r="R54" s="13"/>
+      <c r="S54" s="13"/>
+      <c r="T54" s="13"/>
+      <c r="U54" s="13"/>
+      <c r="V54" s="13"/>
+      <c r="W54" s="13"/>
+      <c r="X54" s="13"/>
     </row>
     <row r="55" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A55" s="13"/>
-      <c r="B55" s="13"/>
-      <c r="C55" s="3" t="s">
+      <c r="A55" s="14"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D55" s="3"/>
-      <c r="E55" s="3"/>
-      <c r="F55" s="3"/>
-      <c r="G55" s="3"/>
-      <c r="H55" s="3"/>
-      <c r="I55" s="3"/>
-      <c r="J55" s="3"/>
-      <c r="K55" s="3"/>
-      <c r="L55" s="3"/>
-      <c r="M55" s="3"/>
-      <c r="N55" s="3"/>
-      <c r="O55" s="3"/>
-      <c r="P55" s="3"/>
-      <c r="Q55" s="3"/>
-      <c r="R55" s="3"/>
-      <c r="S55" s="3"/>
-      <c r="T55" s="3"/>
-      <c r="U55" s="3"/>
-      <c r="V55" s="3"/>
-      <c r="W55" s="3"/>
-      <c r="X55" s="3"/>
+      <c r="D55" s="13"/>
+      <c r="E55" s="13"/>
+      <c r="F55" s="13"/>
+      <c r="G55" s="13"/>
+      <c r="H55" s="13"/>
+      <c r="I55" s="13"/>
+      <c r="J55" s="13"/>
+      <c r="K55" s="13"/>
+      <c r="L55" s="13"/>
+      <c r="M55" s="13"/>
+      <c r="N55" s="13"/>
+      <c r="O55" s="13"/>
+      <c r="P55" s="13"/>
+      <c r="Q55" s="13"/>
+      <c r="R55" s="13"/>
+      <c r="S55" s="13"/>
+      <c r="T55" s="13"/>
+      <c r="U55" s="13"/>
+      <c r="V55" s="13"/>
+      <c r="W55" s="13"/>
+      <c r="X55" s="13"/>
     </row>
     <row r="56" ht="18" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A56" s="13" t="s">
+      <c r="A56" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B56" s="12" t="s">
@@ -2279,45 +2282,45 @@
       <c r="T56" s="3"/>
       <c r="U56" s="3"/>
       <c r="V56" s="3"/>
-      <c r="W56" s="3"/>
-      <c r="X56" s="3"/>
+      <c r="W56" s="13"/>
+      <c r="X56" s="13"/>
     </row>
     <row r="57" ht="5" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A57" s="13"/>
-      <c r="B57" s="13"/>
-      <c r="C57" s="3" t="s">
+      <c r="A57" s="14"/>
+      <c r="B57" s="14"/>
+      <c r="C57" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D57" s="3"/>
-      <c r="E57" s="3"/>
-      <c r="F57" s="3"/>
-      <c r="G57" s="3"/>
-      <c r="H57" s="3"/>
-      <c r="I57" s="3"/>
-      <c r="J57" s="3"/>
-      <c r="K57" s="3"/>
-      <c r="L57" s="3"/>
-      <c r="M57" s="3"/>
-      <c r="N57" s="3"/>
-      <c r="O57" s="3"/>
-      <c r="P57" s="3"/>
-      <c r="Q57" s="3"/>
-      <c r="R57" s="3"/>
-      <c r="S57" s="3"/>
-      <c r="T57" s="3"/>
-      <c r="U57" s="3"/>
-      <c r="V57" s="3"/>
-      <c r="W57" s="3"/>
-      <c r="X57" s="3"/>
+      <c r="D57" s="13"/>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+      <c r="H57" s="13"/>
+      <c r="I57" s="13"/>
+      <c r="J57" s="13"/>
+      <c r="K57" s="13"/>
+      <c r="L57" s="13"/>
+      <c r="M57" s="13"/>
+      <c r="N57" s="13"/>
+      <c r="O57" s="13"/>
+      <c r="P57" s="13"/>
+      <c r="Q57" s="13"/>
+      <c r="R57" s="13"/>
+      <c r="S57" s="13"/>
+      <c r="T57" s="13"/>
+      <c r="U57" s="13"/>
+      <c r="V57" s="13"/>
+      <c r="W57" s="13"/>
+      <c r="X57" s="13"/>
     </row>
     <row r="58" spans="19:23" x14ac:dyDescent="0.25">
-      <c r="S58" s="16" t="s">
+      <c r="S58" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="T58" s="16"/>
-      <c r="U58" s="16"/>
-      <c r="V58" s="16"/>
-      <c r="W58" s="16"/>
+      <c r="T58" s="17"/>
+      <c r="U58" s="17"/>
+      <c r="V58" s="17"/>
+      <c r="W58" s="17"/>
     </row>
     <row r="59" spans="23:23" x14ac:dyDescent="0.25">
       <c r="W59" s="7"/>
@@ -2362,11 +2365,11 @@
   <dimension ref="A2:X98"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.81640625" style="15" customWidth="1"/>
-    <col min="2" max="2" width="42.81640625" style="15" customWidth="1"/>
-    <col min="3" max="3" width="42.26953125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="42.81640625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="14.54296875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="27.81640625" style="16" customWidth="1"/>
+    <col min="2" max="2" width="42.81640625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="42.26953125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="42.81640625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="14.54296875" style="13" customWidth="1"/>
     <col min="6" max="6" width="10.90625" customWidth="1"/>
     <col min="8" max="10" width="16.08984375" customWidth="1"/>
     <col min="11" max="11" width="19.90625" customWidth="1"/>
@@ -2381,13 +2384,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
       <c r="H2" s="6" t="s">
         <v>36</v>
       </c>
@@ -2406,54 +2409,54 @@
       <c r="M2" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="O2" s="15" t="s">
+      <c r="O2" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="P2" s="15" t="s">
+      <c r="P2" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="Q2" s="15" t="s">
+      <c r="Q2" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="R2" s="15" t="s">
+      <c r="R2" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="S2" s="15" t="s">
+      <c r="S2" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="T2" s="15" t="s">
+      <c r="T2" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="U2" s="15" t="s">
+      <c r="U2" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="V2" s="15" t="s">
+      <c r="V2" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="W2" s="15" t="s">
+      <c r="W2" s="16" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="16" t="s">
         <v>37</v>
       </c>
       <c r="I3" s="6" t="s">
@@ -2462,34 +2465,34 @@
       <c r="J3" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="K3" s="19" t="s">
+      <c r="K3" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="L3" s="19" t="s">
+      <c r="L3" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="M3" s="19" t="s">
+      <c r="M3" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="P3" s="19" t="s">
+      <c r="P3" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="Q3" s="15">
+      <c r="Q3" s="16">
         <v>1715</v>
       </c>
-      <c r="R3" s="15">
+      <c r="R3" s="16">
         <v>14</v>
       </c>
-      <c r="S3" s="15">
+      <c r="S3" s="16">
         <v>5</v>
       </c>
-      <c r="T3" s="20">
+      <c r="T3" s="21">
         <v>0.25</v>
       </c>
-      <c r="U3" s="15">
+      <c r="U3" s="16">
         <v>1</v>
       </c>
-      <c r="V3" s="15">
+      <c r="V3" s="16">
         <v>4</v>
       </c>
       <c r="W3" s="6" t="s">
@@ -2497,59 +2500,59 @@
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
+      <c r="A4" s="16">
         <v>9</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>62</v>
       </c>
       <c r="F4" s="6">
         <v>1</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="16" t="s">
         <v>38</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="J4" s="15"/>
-      <c r="K4" s="21" t="s">
+      <c r="J4" s="16"/>
+      <c r="K4" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="L4" s="21" t="s">
+      <c r="L4" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="M4" s="21" t="s">
+      <c r="M4" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="P4" s="21" t="s">
+      <c r="P4" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="Q4" s="15">
+      <c r="Q4" s="16">
         <v>1750</v>
       </c>
-      <c r="R4" s="15">
+      <c r="R4" s="16">
         <v>19</v>
       </c>
-      <c r="S4" s="15">
+      <c r="S4" s="16">
         <v>6</v>
       </c>
-      <c r="T4" s="20">
+      <c r="T4" s="21">
         <v>0.5</v>
       </c>
-      <c r="U4" s="15">
+      <c r="U4" s="16">
         <v>1</v>
       </c>
-      <c r="V4" s="15">
+      <c r="V4" s="16">
         <v>4</v>
       </c>
       <c r="W4" s="6" t="s">
@@ -2557,55 +2560,55 @@
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A5" s="15">
+      <c r="A5" s="16">
         <v>10.5</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="16" t="s">
         <v>62</v>
       </c>
       <c r="F5" s="6">
         <v>1</v>
       </c>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="21" t="s">
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="L5" s="21" t="s">
+      <c r="L5" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="M5" s="21" t="s">
+      <c r="M5" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="P5" s="21" t="s">
+      <c r="P5" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="Q5" s="15">
+      <c r="Q5" s="16">
         <v>1750</v>
       </c>
-      <c r="R5" s="15">
+      <c r="R5" s="16">
         <v>19</v>
       </c>
-      <c r="S5" s="15">
+      <c r="S5" s="16">
         <v>6</v>
       </c>
-      <c r="T5" s="20">
+      <c r="T5" s="21">
         <v>0.75</v>
       </c>
-      <c r="U5" s="15">
+      <c r="U5" s="16">
         <v>1</v>
       </c>
-      <c r="V5" s="15">
+      <c r="V5" s="16">
         <v>4</v>
       </c>
       <c r="W5" s="6" t="s">
@@ -2613,55 +2616,55 @@
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A6" s="15">
+      <c r="A6" s="16">
         <v>12.25</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="24">
+      <c r="F6" s="25">
         <v>1.25</v>
       </c>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="21" t="s">
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="L6" s="21" t="s">
+      <c r="L6" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="M6" s="21" t="s">
+      <c r="M6" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="P6" s="21" t="s">
+      <c r="P6" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="Q6" s="15">
+      <c r="Q6" s="16">
         <v>1750</v>
       </c>
-      <c r="R6" s="15">
+      <c r="R6" s="16">
         <v>24</v>
       </c>
-      <c r="S6" s="15">
+      <c r="S6" s="16">
         <v>8</v>
       </c>
-      <c r="T6" s="25">
+      <c r="T6" s="26">
         <v>1</v>
       </c>
-      <c r="U6" s="15">
+      <c r="U6" s="16">
         <v>1</v>
       </c>
-      <c r="V6" s="15">
+      <c r="V6" s="16">
         <v>4</v>
       </c>
       <c r="W6" s="6" t="s">
@@ -2669,55 +2672,55 @@
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A7" s="15">
+      <c r="A7" s="16">
         <v>13.5</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F7" s="24">
+      <c r="F7" s="25">
         <v>1.25</v>
       </c>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="21" t="s">
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="L7" s="21" t="s">
+      <c r="L7" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="M7" s="21" t="s">
+      <c r="M7" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="P7" s="21" t="s">
+      <c r="P7" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="Q7" s="15">
+      <c r="Q7" s="16">
         <v>1750</v>
       </c>
-      <c r="R7" s="15">
+      <c r="R7" s="16">
         <v>24</v>
       </c>
-      <c r="S7" s="15">
+      <c r="S7" s="16">
         <v>8</v>
       </c>
-      <c r="T7" s="20">
+      <c r="T7" s="21">
         <v>1.5</v>
       </c>
-      <c r="U7" s="15">
+      <c r="U7" s="16">
         <v>1</v>
       </c>
-      <c r="V7" s="15">
+      <c r="V7" s="16">
         <v>4</v>
       </c>
       <c r="W7" s="6" t="s">
@@ -2725,55 +2728,55 @@
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A8" s="15">
+      <c r="A8" s="16">
         <v>15</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E8" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="25">
         <v>1.25</v>
       </c>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="21" t="s">
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="L8" s="21" t="s">
+      <c r="L8" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="M8" s="21" t="s">
+      <c r="M8" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="P8" s="21" t="s">
+      <c r="P8" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="Q8" s="15">
+      <c r="Q8" s="16">
         <v>1750</v>
       </c>
-      <c r="R8" s="15">
+      <c r="R8" s="16">
         <v>28</v>
       </c>
-      <c r="S8" s="15">
+      <c r="S8" s="16">
         <v>8</v>
       </c>
-      <c r="T8" s="20">
+      <c r="T8" s="21">
         <v>2</v>
       </c>
-      <c r="U8" s="15">
+      <c r="U8" s="16">
         <v>1</v>
       </c>
-      <c r="V8" s="15">
+      <c r="V8" s="16">
         <v>4</v>
       </c>
       <c r="W8" s="6" t="s">
@@ -2781,55 +2784,55 @@
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A9" s="15">
+      <c r="A9" s="16">
         <v>16.5</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="24">
+      <c r="F9" s="25">
         <v>1.25</v>
       </c>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="21" t="s">
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="L9" s="21" t="s">
+      <c r="L9" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="M9" s="21" t="s">
+      <c r="M9" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="P9" s="21" t="s">
+      <c r="P9" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="Q9" s="15">
+      <c r="Q9" s="16">
         <v>1750</v>
       </c>
-      <c r="R9" s="15">
+      <c r="R9" s="16">
         <v>28</v>
       </c>
-      <c r="S9" s="15">
+      <c r="S9" s="16">
         <v>8</v>
       </c>
-      <c r="T9" s="20">
-        <v>3</v>
-      </c>
-      <c r="U9" s="15">
+      <c r="T9" s="21">
+        <v>3</v>
+      </c>
+      <c r="U9" s="16">
         <v>1</v>
       </c>
-      <c r="V9" s="15">
+      <c r="V9" s="16">
         <v>4</v>
       </c>
       <c r="W9" s="6" t="s">
@@ -2837,55 +2840,55 @@
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
+      <c r="A10" s="16">
         <v>18.25</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="24">
+      <c r="F10" s="25">
         <v>1.25</v>
       </c>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
-      <c r="J10" s="15"/>
-      <c r="K10" s="21" t="s">
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="L10" s="21" t="s">
+      <c r="L10" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="M10" s="21" t="s">
+      <c r="M10" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="P10" s="21" t="s">
+      <c r="P10" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="Q10" s="15">
+      <c r="Q10" s="16">
         <v>1750</v>
       </c>
-      <c r="R10" s="15">
+      <c r="R10" s="16">
         <v>28</v>
       </c>
-      <c r="S10" s="15">
+      <c r="S10" s="16">
         <v>8</v>
       </c>
-      <c r="T10" s="20">
+      <c r="T10" s="21">
         <v>5</v>
       </c>
-      <c r="U10" s="15">
+      <c r="U10" s="16">
         <v>1</v>
       </c>
-      <c r="V10" s="15">
+      <c r="V10" s="16">
         <v>4</v>
       </c>
       <c r="W10" s="6" t="s">
@@ -2893,56 +2896,56 @@
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+      <c r="A11" s="16">
         <v>20</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="24">
+      <c r="F11" s="25">
         <v>1.25</v>
       </c>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="21" t="s">
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="M11" s="21" t="s">
+      <c r="M11" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="O11" s="15" t="s">
+      <c r="O11" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="P11" s="19" t="s">
+      <c r="P11" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="Q11" s="15">
+      <c r="Q11" s="16">
         <v>1680</v>
       </c>
-      <c r="R11" s="15">
+      <c r="R11" s="16">
         <v>14</v>
       </c>
-      <c r="S11" s="15">
+      <c r="S11" s="16">
         <v>5</v>
       </c>
-      <c r="T11" s="20">
+      <c r="T11" s="21">
         <v>0.5</v>
       </c>
-      <c r="U11" s="15">
-        <v>3</v>
-      </c>
-      <c r="V11" s="15">
+      <c r="U11" s="16">
+        <v>3</v>
+      </c>
+      <c r="V11" s="16">
         <v>4</v>
       </c>
       <c r="W11" s="6" t="s">
@@ -2950,53 +2953,53 @@
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" s="15">
+      <c r="A12" s="16">
         <v>22.25</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F12" s="24">
+      <c r="F12" s="25">
         <v>1.25</v>
       </c>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="15"/>
-      <c r="L12" s="21" t="s">
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="M12" s="21" t="s">
+      <c r="M12" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="P12" s="21" t="s">
+      <c r="P12" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="Q12" s="15">
+      <c r="Q12" s="16">
         <v>1710</v>
       </c>
-      <c r="R12" s="15">
+      <c r="R12" s="16">
         <v>19</v>
       </c>
-      <c r="S12" s="15">
+      <c r="S12" s="16">
         <v>6</v>
       </c>
-      <c r="T12" s="20">
+      <c r="T12" s="21">
         <v>1</v>
       </c>
-      <c r="U12" s="15">
-        <v>3</v>
-      </c>
-      <c r="V12" s="15">
+      <c r="U12" s="16">
+        <v>3</v>
+      </c>
+      <c r="V12" s="16">
         <v>4</v>
       </c>
       <c r="W12" s="6" t="s">
@@ -3004,53 +3007,53 @@
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A13" s="15">
+      <c r="A13" s="16">
         <v>24.5</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E13" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="25">
         <v>1.5</v>
       </c>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="21" t="s">
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="M13" s="21" t="s">
+      <c r="M13" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="P13" s="21" t="s">
+      <c r="P13" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="Q13" s="15">
+      <c r="Q13" s="16">
         <v>1720</v>
       </c>
-      <c r="R13" s="15">
+      <c r="R13" s="16">
         <v>24</v>
       </c>
-      <c r="S13" s="15">
+      <c r="S13" s="16">
         <v>8</v>
       </c>
-      <c r="T13" s="20">
+      <c r="T13" s="21">
         <v>1.5</v>
       </c>
-      <c r="U13" s="15">
-        <v>3</v>
-      </c>
-      <c r="V13" s="15">
+      <c r="U13" s="16">
+        <v>3</v>
+      </c>
+      <c r="V13" s="16">
         <v>4</v>
       </c>
       <c r="W13" s="6" t="s">
@@ -3058,53 +3061,53 @@
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
+      <c r="A14" s="16">
         <v>27</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="F14" s="24">
+      <c r="F14" s="25">
         <v>1.5</v>
       </c>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15"/>
-      <c r="L14" s="21" t="s">
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="M14" s="21" t="s">
+      <c r="M14" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="P14" s="21" t="s">
+      <c r="P14" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="Q14" s="15">
+      <c r="Q14" s="16">
         <v>1715</v>
       </c>
-      <c r="R14" s="15">
+      <c r="R14" s="16">
         <v>24</v>
       </c>
-      <c r="S14" s="15">
+      <c r="S14" s="16">
         <v>8</v>
       </c>
-      <c r="T14" s="20">
+      <c r="T14" s="21">
         <v>2</v>
       </c>
-      <c r="U14" s="15">
-        <v>3</v>
-      </c>
-      <c r="V14" s="15">
+      <c r="U14" s="16">
+        <v>3</v>
+      </c>
+      <c r="V14" s="16">
         <v>4</v>
       </c>
       <c r="W14" s="6" t="s">
@@ -3112,53 +3115,53 @@
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A15" s="15">
+      <c r="A15" s="16">
         <v>30</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="F15" s="24">
+      <c r="F15" s="25">
         <v>1.75</v>
       </c>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="21" t="s">
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="M15" s="21" t="s">
+      <c r="M15" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="P15" s="21" t="s">
+      <c r="P15" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="Q15" s="15">
+      <c r="Q15" s="16">
         <v>1735</v>
       </c>
-      <c r="R15" s="15">
+      <c r="R15" s="16">
         <v>28</v>
       </c>
-      <c r="S15" s="15">
+      <c r="S15" s="16">
         <v>8</v>
       </c>
-      <c r="T15" s="20">
-        <v>3</v>
-      </c>
-      <c r="U15" s="15">
-        <v>3</v>
-      </c>
-      <c r="V15" s="15">
+      <c r="T15" s="21">
+        <v>3</v>
+      </c>
+      <c r="U15" s="16">
+        <v>3</v>
+      </c>
+      <c r="V15" s="16">
         <v>4</v>
       </c>
       <c r="W15" s="6" t="s">
@@ -3166,53 +3169,53 @@
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
+      <c r="A16" s="16">
         <v>33</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="F16" s="24">
+      <c r="F16" s="25">
         <v>2</v>
       </c>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="21" t="s">
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="M16" s="21" t="s">
+      <c r="M16" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="P16" s="21" t="s">
+      <c r="P16" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="Q16" s="15">
+      <c r="Q16" s="16">
         <v>1745</v>
       </c>
-      <c r="R16" s="15">
+      <c r="R16" s="16">
         <v>28</v>
       </c>
-      <c r="S16" s="15">
+      <c r="S16" s="16">
         <v>8</v>
       </c>
-      <c r="T16" s="20">
+      <c r="T16" s="21">
         <v>5</v>
       </c>
-      <c r="U16" s="15">
-        <v>3</v>
-      </c>
-      <c r="V16" s="15">
+      <c r="U16" s="16">
+        <v>3</v>
+      </c>
+      <c r="V16" s="16">
         <v>4</v>
       </c>
       <c r="W16" s="6" t="s">
@@ -3220,53 +3223,53 @@
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
+      <c r="A17" s="16">
         <v>36.5</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E17" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="25">
         <v>2</v>
       </c>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="21" t="s">
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="M17" s="21" t="s">
+      <c r="M17" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="P17" s="21" t="s">
+      <c r="P17" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="Q17" s="15">
+      <c r="Q17" s="16">
         <v>1750</v>
       </c>
-      <c r="R17" s="15">
+      <c r="R17" s="16">
         <v>38</v>
       </c>
-      <c r="S17" s="15">
+      <c r="S17" s="16">
         <v>10</v>
       </c>
-      <c r="T17" s="20">
+      <c r="T17" s="21">
         <v>7.5</v>
       </c>
-      <c r="U17" s="15">
-        <v>3</v>
-      </c>
-      <c r="V17" s="15">
+      <c r="U17" s="16">
+        <v>3</v>
+      </c>
+      <c r="V17" s="16">
         <v>4</v>
       </c>
       <c r="W17" s="6" t="s">
@@ -3274,53 +3277,53 @@
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
+      <c r="A18" s="16">
         <v>40.25</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="E18" s="15" t="s">
+      <c r="E18" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="25">
         <v>2.25</v>
       </c>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="21" t="s">
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="M18" s="21" t="s">
+      <c r="M18" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="P18" s="21" t="s">
+      <c r="P18" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="Q18" s="15">
+      <c r="Q18" s="16">
         <v>1750</v>
       </c>
-      <c r="R18" s="15">
+      <c r="R18" s="16">
         <v>38</v>
       </c>
-      <c r="S18" s="15">
+      <c r="S18" s="16">
         <v>10</v>
       </c>
-      <c r="T18" s="20">
+      <c r="T18" s="21">
         <v>10</v>
       </c>
-      <c r="U18" s="15">
-        <v>3</v>
-      </c>
-      <c r="V18" s="15">
+      <c r="U18" s="16">
+        <v>3</v>
+      </c>
+      <c r="V18" s="16">
         <v>4</v>
       </c>
       <c r="W18" s="6" t="s">
@@ -3328,53 +3331,53 @@
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
+      <c r="A19" s="16">
         <v>44.5</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="E19" s="15" t="s">
+      <c r="E19" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="F19" s="24">
+      <c r="F19" s="25">
         <v>2.25</v>
       </c>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="21" t="s">
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="M19" s="21" t="s">
+      <c r="M19" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="P19" s="21" t="s">
+      <c r="P19" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="Q19" s="15">
+      <c r="Q19" s="16">
         <v>1760</v>
       </c>
-      <c r="R19" s="15">
+      <c r="R19" s="16">
         <v>42</v>
       </c>
-      <c r="S19" s="15">
+      <c r="S19" s="16">
         <v>12</v>
       </c>
-      <c r="T19" s="20">
+      <c r="T19" s="21">
         <v>15</v>
       </c>
-      <c r="U19" s="15">
-        <v>3</v>
-      </c>
-      <c r="V19" s="15">
+      <c r="U19" s="16">
+        <v>3</v>
+      </c>
+      <c r="V19" s="16">
         <v>4</v>
       </c>
       <c r="W19" s="6" t="s">
@@ -3382,53 +3385,53 @@
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
+      <c r="A20" s="16">
         <v>49</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E20" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="25">
         <v>2.5</v>
       </c>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="21" t="s">
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="M20" s="21" t="s">
+      <c r="M20" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="P20" s="21" t="s">
+      <c r="P20" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="Q20" s="15">
+      <c r="Q20" s="16">
         <v>1760</v>
       </c>
-      <c r="R20" s="15">
+      <c r="R20" s="16">
         <v>42</v>
       </c>
-      <c r="S20" s="15">
+      <c r="S20" s="16">
         <v>12</v>
       </c>
-      <c r="T20" s="20">
+      <c r="T20" s="21">
         <v>20</v>
       </c>
-      <c r="U20" s="15">
-        <v>3</v>
-      </c>
-      <c r="V20" s="15">
+      <c r="U20" s="16">
+        <v>3</v>
+      </c>
+      <c r="V20" s="16">
         <v>4</v>
       </c>
       <c r="W20" s="6" t="s">
@@ -3436,53 +3439,53 @@
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
+      <c r="A21" s="16">
         <v>54.5</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F21" s="24">
+      <c r="F21" s="25">
         <v>2.5</v>
       </c>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="15"/>
-      <c r="L21" s="21" t="s">
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="M21" s="21" t="s">
+      <c r="M21" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="P21" s="21" t="s">
+      <c r="P21" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="Q21" s="15">
+      <c r="Q21" s="16">
         <v>1760</v>
       </c>
-      <c r="R21" s="15">
+      <c r="R21" s="16">
         <v>48</v>
       </c>
-      <c r="S21" s="15">
+      <c r="S21" s="16">
         <v>14</v>
       </c>
-      <c r="T21" s="20">
+      <c r="T21" s="21">
         <v>25</v>
       </c>
-      <c r="U21" s="15">
-        <v>3</v>
-      </c>
-      <c r="V21" s="15">
+      <c r="U21" s="16">
+        <v>3</v>
+      </c>
+      <c r="V21" s="16">
         <v>4</v>
       </c>
       <c r="W21" s="6" t="s">
@@ -3490,53 +3493,53 @@
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A22" s="15">
+      <c r="A22" s="16">
         <v>60</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F22" s="24">
-        <v>3</v>
-      </c>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="21" t="s">
+      <c r="F22" s="25">
+        <v>3</v>
+      </c>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="M22" s="21" t="s">
+      <c r="M22" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="P22" s="21" t="s">
+      <c r="P22" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="Q22" s="15">
+      <c r="Q22" s="16">
         <v>1765</v>
       </c>
-      <c r="R22" s="15">
+      <c r="R22" s="16">
         <v>48</v>
       </c>
-      <c r="S22" s="15">
+      <c r="S22" s="16">
         <v>14</v>
       </c>
-      <c r="T22" s="20">
+      <c r="T22" s="21">
         <v>30</v>
       </c>
-      <c r="U22" s="15">
-        <v>3</v>
-      </c>
-      <c r="V22" s="15">
+      <c r="U22" s="16">
+        <v>3</v>
+      </c>
+      <c r="V22" s="16">
         <v>4</v>
       </c>
       <c r="W22" s="6" t="s">
@@ -3544,53 +3547,53 @@
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
+      <c r="A23" s="16">
         <v>66</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="E23" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F23" s="24">
-        <v>3</v>
-      </c>
-      <c r="H23" s="15"/>
-      <c r="I23" s="15"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="15"/>
-      <c r="L23" s="21" t="s">
+      <c r="F23" s="25">
+        <v>3</v>
+      </c>
+      <c r="H23" s="16"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="M23" s="21" t="s">
+      <c r="M23" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="P23" s="21" t="s">
+      <c r="P23" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="Q23" s="15">
+      <c r="Q23" s="16">
         <v>1760</v>
       </c>
-      <c r="R23" s="15">
+      <c r="R23" s="16">
         <v>55</v>
       </c>
-      <c r="S23" s="15">
+      <c r="S23" s="16">
         <v>16</v>
       </c>
-      <c r="T23" s="20">
+      <c r="T23" s="21">
         <v>40</v>
       </c>
-      <c r="U23" s="15">
-        <v>3</v>
-      </c>
-      <c r="V23" s="15">
+      <c r="U23" s="16">
+        <v>3</v>
+      </c>
+      <c r="V23" s="16">
         <v>4</v>
       </c>
       <c r="W23" s="6" t="s">
@@ -3598,53 +3601,53 @@
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
+      <c r="A24" s="16">
         <v>73</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F24" s="24">
-        <v>3</v>
-      </c>
-      <c r="H24" s="15"/>
-      <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="15"/>
-      <c r="L24" s="21" t="s">
+      <c r="F24" s="25">
+        <v>3</v>
+      </c>
+      <c r="H24" s="16"/>
+      <c r="I24" s="16"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="16"/>
+      <c r="L24" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="M24" s="21" t="s">
+      <c r="M24" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="P24" s="21" t="s">
+      <c r="P24" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="Q24" s="15">
+      <c r="Q24" s="16">
         <v>1770</v>
       </c>
-      <c r="R24" s="15">
+      <c r="R24" s="16">
         <v>60</v>
       </c>
-      <c r="S24" s="15">
+      <c r="S24" s="16">
         <v>18</v>
       </c>
-      <c r="T24" s="20">
+      <c r="T24" s="21">
         <v>50</v>
       </c>
-      <c r="U24" s="15">
-        <v>3</v>
-      </c>
-      <c r="V24" s="15">
+      <c r="U24" s="16">
+        <v>3</v>
+      </c>
+      <c r="V24" s="16">
         <v>4</v>
       </c>
       <c r="W24" s="6" t="s">
@@ -3652,53 +3655,53 @@
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
+      <c r="A25" s="16">
         <v>83</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F25" s="24">
-        <v>3</v>
-      </c>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="15"/>
-      <c r="L25" s="21" t="s">
+      <c r="F25" s="25">
+        <v>3</v>
+      </c>
+      <c r="H25" s="16"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="M25" s="21" t="s">
+      <c r="M25" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="P25" s="21" t="s">
+      <c r="P25" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="Q25" s="15">
+      <c r="Q25" s="16">
         <v>1765</v>
       </c>
-      <c r="R25" s="15">
+      <c r="R25" s="16">
         <v>60</v>
       </c>
-      <c r="S25" s="15">
+      <c r="S25" s="16">
         <v>18</v>
       </c>
-      <c r="T25" s="20">
+      <c r="T25" s="21">
         <v>60</v>
       </c>
-      <c r="U25" s="15">
-        <v>3</v>
-      </c>
-      <c r="V25" s="15">
+      <c r="U25" s="16">
+        <v>3</v>
+      </c>
+      <c r="V25" s="16">
         <v>4</v>
       </c>
       <c r="W25" s="6" t="s">
@@ -3706,31 +3709,31 @@
       </c>
     </row>
     <row r="26" spans="8:23" x14ac:dyDescent="0.25">
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="15"/>
-      <c r="K26" s="15"/>
-      <c r="L26" s="15"/>
-      <c r="M26" s="21"/>
-      <c r="P26" s="21" t="s">
+      <c r="H26" s="16"/>
+      <c r="I26" s="16"/>
+      <c r="J26" s="16"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="16"/>
+      <c r="M26" s="22"/>
+      <c r="P26" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="Q26" s="15">
+      <c r="Q26" s="16">
         <v>1775</v>
       </c>
-      <c r="R26" s="15">
+      <c r="R26" s="16">
         <v>65</v>
       </c>
-      <c r="S26" s="15">
+      <c r="S26" s="16">
         <v>18</v>
       </c>
-      <c r="T26" s="20">
+      <c r="T26" s="21">
         <v>75</v>
       </c>
-      <c r="U26" s="15">
-        <v>3</v>
-      </c>
-      <c r="V26" s="15">
+      <c r="U26" s="16">
+        <v>3</v>
+      </c>
+      <c r="V26" s="16">
         <v>4</v>
       </c>
       <c r="W26" s="6" t="s">
@@ -3738,31 +3741,31 @@
       </c>
     </row>
     <row r="27" spans="8:23" x14ac:dyDescent="0.25">
-      <c r="H27" s="15"/>
-      <c r="I27" s="15"/>
-      <c r="J27" s="15"/>
-      <c r="K27" s="15"/>
-      <c r="L27" s="15"/>
-      <c r="M27" s="15"/>
-      <c r="P27" s="21" t="s">
+      <c r="H27" s="16"/>
+      <c r="I27" s="16"/>
+      <c r="J27" s="16"/>
+      <c r="K27" s="16"/>
+      <c r="L27" s="16"/>
+      <c r="M27" s="16"/>
+      <c r="P27" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="Q27" s="15">
+      <c r="Q27" s="16">
         <v>1775</v>
       </c>
-      <c r="R27" s="15">
+      <c r="R27" s="16">
         <v>75</v>
       </c>
-      <c r="S27" s="15">
+      <c r="S27" s="16">
         <v>20</v>
       </c>
-      <c r="T27" s="20">
+      <c r="T27" s="21">
         <v>100</v>
       </c>
-      <c r="U27" s="15">
-        <v>3</v>
-      </c>
-      <c r="V27" s="15">
+      <c r="U27" s="16">
+        <v>3</v>
+      </c>
+      <c r="V27" s="16">
         <v>4</v>
       </c>
       <c r="W27" s="6" t="s">
@@ -3770,37 +3773,37 @@
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="B28" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
-      <c r="K28" s="15"/>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
-      <c r="P28" s="21" t="s">
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
+      <c r="M28" s="16"/>
+      <c r="P28" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="Q28" s="15">
+      <c r="Q28" s="16">
         <v>1770</v>
       </c>
-      <c r="R28" s="15">
+      <c r="R28" s="16">
         <v>75</v>
       </c>
-      <c r="S28" s="15">
+      <c r="S28" s="16">
         <v>20</v>
       </c>
-      <c r="T28" s="20">
+      <c r="T28" s="21">
         <v>125</v>
       </c>
-      <c r="U28" s="15">
-        <v>3</v>
-      </c>
-      <c r="V28" s="15">
+      <c r="U28" s="16">
+        <v>3</v>
+      </c>
+      <c r="V28" s="16">
         <v>4</v>
       </c>
       <c r="W28" s="6" t="s">
@@ -3808,37 +3811,37 @@
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B29" s="15" t="s">
+      <c r="B29" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
-      <c r="J29" s="15"/>
-      <c r="K29" s="15"/>
-      <c r="L29" s="15"/>
-      <c r="M29" s="15"/>
-      <c r="P29" s="21" t="s">
+      <c r="H29" s="16"/>
+      <c r="I29" s="16"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="16"/>
+      <c r="P29" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="Q29" s="15">
+      <c r="Q29" s="16">
         <v>1770</v>
       </c>
-      <c r="R29" s="15">
+      <c r="R29" s="16">
         <v>85</v>
       </c>
-      <c r="S29" s="15">
+      <c r="S29" s="16">
         <v>22</v>
       </c>
-      <c r="T29" s="20">
+      <c r="T29" s="21">
         <v>150</v>
       </c>
-      <c r="U29" s="15">
-        <v>3</v>
-      </c>
-      <c r="V29" s="15">
+      <c r="U29" s="16">
+        <v>3</v>
+      </c>
+      <c r="V29" s="16">
         <v>4</v>
       </c>
       <c r="W29" s="6" t="s">
@@ -3846,37 +3849,37 @@
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="B30" s="15" t="s">
+      <c r="B30" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="H30" s="15"/>
-      <c r="I30" s="15"/>
-      <c r="J30" s="15"/>
-      <c r="K30" s="15"/>
-      <c r="L30" s="15"/>
-      <c r="M30" s="15"/>
-      <c r="P30" s="21" t="s">
+      <c r="H30" s="16"/>
+      <c r="I30" s="16"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
+      <c r="M30" s="16"/>
+      <c r="P30" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="Q30" s="15">
+      <c r="Q30" s="16">
         <v>1770</v>
       </c>
-      <c r="R30" s="15">
+      <c r="R30" s="16">
         <v>85</v>
       </c>
-      <c r="S30" s="15">
+      <c r="S30" s="16">
         <v>22</v>
       </c>
-      <c r="T30" s="20">
+      <c r="T30" s="21">
         <v>175</v>
       </c>
-      <c r="U30" s="15">
-        <v>3</v>
-      </c>
-      <c r="V30" s="15">
+      <c r="U30" s="16">
+        <v>3</v>
+      </c>
+      <c r="V30" s="16">
         <v>4</v>
       </c>
       <c r="W30" s="6" t="s">
@@ -3884,37 +3887,37 @@
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A31" s="15" t="s">
+      <c r="A31" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="B31" s="15" t="s">
+      <c r="B31" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="H31" s="15"/>
-      <c r="I31" s="15"/>
-      <c r="J31" s="15"/>
-      <c r="K31" s="15"/>
-      <c r="L31" s="15"/>
-      <c r="M31" s="15"/>
-      <c r="P31" s="21" t="s">
+      <c r="H31" s="16"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="16"/>
+      <c r="M31" s="16"/>
+      <c r="P31" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="Q31" s="15">
+      <c r="Q31" s="16">
         <v>1775</v>
       </c>
-      <c r="R31" s="15">
+      <c r="R31" s="16">
         <v>95</v>
       </c>
-      <c r="S31" s="15">
+      <c r="S31" s="16">
         <v>25</v>
       </c>
-      <c r="T31" s="20">
+      <c r="T31" s="21">
         <v>200</v>
       </c>
-      <c r="U31" s="15">
-        <v>3</v>
-      </c>
-      <c r="V31" s="15">
+      <c r="U31" s="16">
+        <v>3</v>
+      </c>
+      <c r="V31" s="16">
         <v>4</v>
       </c>
       <c r="W31" s="6" t="s">
@@ -3922,31 +3925,31 @@
       </c>
     </row>
     <row r="32" spans="8:23" x14ac:dyDescent="0.25">
-      <c r="H32" s="15"/>
-      <c r="I32" s="15"/>
-      <c r="J32" s="15"/>
-      <c r="K32" s="15"/>
-      <c r="L32" s="15"/>
-      <c r="M32" s="15"/>
-      <c r="P32" s="21" t="s">
+      <c r="H32" s="16"/>
+      <c r="I32" s="16"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="16"/>
+      <c r="L32" s="16"/>
+      <c r="M32" s="16"/>
+      <c r="P32" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="Q32" s="15">
+      <c r="Q32" s="16">
         <v>1775</v>
       </c>
-      <c r="R32" s="15">
+      <c r="R32" s="16">
         <v>95</v>
       </c>
-      <c r="S32" s="15">
+      <c r="S32" s="16">
         <v>25</v>
       </c>
-      <c r="T32" s="20">
+      <c r="T32" s="21">
         <v>250</v>
       </c>
-      <c r="U32" s="15">
-        <v>3</v>
-      </c>
-      <c r="V32" s="15">
+      <c r="U32" s="16">
+        <v>3</v>
+      </c>
+      <c r="V32" s="16">
         <v>4</v>
       </c>
       <c r="W32" s="6" t="s">
@@ -3954,31 +3957,31 @@
       </c>
     </row>
     <row r="33" spans="8:23" x14ac:dyDescent="0.25">
-      <c r="H33" s="15"/>
-      <c r="I33" s="15"/>
-      <c r="J33" s="15"/>
-      <c r="K33" s="15"/>
-      <c r="L33" s="15"/>
-      <c r="M33" s="15"/>
-      <c r="P33" s="21" t="s">
+      <c r="H33" s="16"/>
+      <c r="I33" s="16"/>
+      <c r="J33" s="16"/>
+      <c r="K33" s="16"/>
+      <c r="L33" s="16"/>
+      <c r="M33" s="16"/>
+      <c r="P33" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="Q33" s="15">
+      <c r="Q33" s="16">
         <v>1775</v>
       </c>
-      <c r="R33" s="15">
+      <c r="R33" s="16">
         <v>95</v>
       </c>
-      <c r="S33" s="15">
+      <c r="S33" s="16">
         <v>25</v>
       </c>
-      <c r="T33" s="20">
+      <c r="T33" s="21">
         <v>300</v>
       </c>
-      <c r="U33" s="15">
-        <v>3</v>
-      </c>
-      <c r="V33" s="15">
+      <c r="U33" s="16">
+        <v>3</v>
+      </c>
+      <c r="V33" s="16">
         <v>4</v>
       </c>
       <c r="W33" s="6" t="s">
@@ -3986,37 +3989,37 @@
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="H34" s="15"/>
-      <c r="I34" s="15"/>
-      <c r="J34" s="15"/>
-      <c r="K34" s="15"/>
-      <c r="L34" s="15"/>
-      <c r="M34" s="15"/>
-      <c r="O34" s="15" t="s">
+      <c r="H34" s="16"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="16"/>
+      <c r="K34" s="16"/>
+      <c r="L34" s="16"/>
+      <c r="M34" s="16"/>
+      <c r="O34" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="P34" s="19" t="s">
+      <c r="P34" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="Q34" s="15">
+      <c r="Q34" s="16">
         <v>1660</v>
       </c>
-      <c r="R34" s="15">
+      <c r="R34" s="16">
         <v>14</v>
       </c>
-      <c r="S34" s="15">
+      <c r="S34" s="16">
         <v>5</v>
       </c>
-      <c r="T34" s="20">
+      <c r="T34" s="21">
         <v>0.5</v>
       </c>
-      <c r="U34" s="15">
-        <v>3</v>
-      </c>
-      <c r="V34" s="15">
+      <c r="U34" s="16">
+        <v>3</v>
+      </c>
+      <c r="V34" s="16">
         <v>4</v>
       </c>
       <c r="W34" s="6" t="s">
@@ -4024,34 +4027,34 @@
       </c>
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A35" s="15" t="s">
+      <c r="A35" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="H35" s="15"/>
-      <c r="I35" s="15"/>
-      <c r="J35" s="15"/>
-      <c r="K35" s="15"/>
-      <c r="L35" s="15"/>
-      <c r="M35" s="15"/>
-      <c r="P35" s="21" t="s">
+      <c r="H35" s="16"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="16"/>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16"/>
+      <c r="M35" s="16"/>
+      <c r="P35" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="Q35" s="15">
+      <c r="Q35" s="16">
         <v>1668</v>
       </c>
-      <c r="R35" s="15">
+      <c r="R35" s="16">
         <v>19</v>
       </c>
-      <c r="S35" s="15">
+      <c r="S35" s="16">
         <v>6</v>
       </c>
-      <c r="T35" s="20">
+      <c r="T35" s="21">
         <v>1</v>
       </c>
-      <c r="U35" s="15">
-        <v>3</v>
-      </c>
-      <c r="V35" s="15">
+      <c r="U35" s="16">
+        <v>3</v>
+      </c>
+      <c r="V35" s="16">
         <v>4</v>
       </c>
       <c r="W35" s="6" t="s">
@@ -4059,34 +4062,34 @@
       </c>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A36" s="15" t="s">
+      <c r="A36" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="H36" s="15"/>
-      <c r="I36" s="15"/>
-      <c r="J36" s="15"/>
-      <c r="K36" s="15"/>
-      <c r="L36" s="15"/>
-      <c r="M36" s="15"/>
-      <c r="P36" s="21" t="s">
+      <c r="H36" s="16"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="16"/>
+      <c r="K36" s="16"/>
+      <c r="L36" s="16"/>
+      <c r="M36" s="16"/>
+      <c r="P36" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="Q36" s="15">
+      <c r="Q36" s="16">
         <v>1680</v>
       </c>
-      <c r="R36" s="15">
+      <c r="R36" s="16">
         <v>24</v>
       </c>
-      <c r="S36" s="15">
+      <c r="S36" s="16">
         <v>8</v>
       </c>
-      <c r="T36" s="20">
+      <c r="T36" s="21">
         <v>1.5</v>
       </c>
-      <c r="U36" s="15">
-        <v>3</v>
-      </c>
-      <c r="V36" s="15">
+      <c r="U36" s="16">
+        <v>3</v>
+      </c>
+      <c r="V36" s="16">
         <v>4</v>
       </c>
       <c r="W36" s="6" t="s">
@@ -4094,34 +4097,34 @@
       </c>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A37" s="15" t="s">
+      <c r="A37" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
-      <c r="J37" s="27"/>
-      <c r="K37" s="27"/>
-      <c r="L37" s="27"/>
-      <c r="M37" s="27"/>
-      <c r="P37" s="21" t="s">
+      <c r="H37" s="28"/>
+      <c r="I37" s="28"/>
+      <c r="J37" s="28"/>
+      <c r="K37" s="28"/>
+      <c r="L37" s="28"/>
+      <c r="M37" s="28"/>
+      <c r="P37" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="Q37" s="15">
+      <c r="Q37" s="16">
         <v>1680</v>
       </c>
-      <c r="R37" s="15">
+      <c r="R37" s="16">
         <v>24</v>
       </c>
-      <c r="S37" s="15">
+      <c r="S37" s="16">
         <v>8</v>
       </c>
-      <c r="T37" s="20">
+      <c r="T37" s="21">
         <v>2</v>
       </c>
-      <c r="U37" s="15">
-        <v>3</v>
-      </c>
-      <c r="V37" s="15">
+      <c r="U37" s="16">
+        <v>3</v>
+      </c>
+      <c r="V37" s="16">
         <v>4</v>
       </c>
       <c r="W37" s="6" t="s">
@@ -4129,31 +4132,31 @@
       </c>
     </row>
     <row r="38" spans="8:23" x14ac:dyDescent="0.25">
-      <c r="H38" s="15"/>
-      <c r="I38" s="15"/>
-      <c r="J38" s="15"/>
-      <c r="K38" s="15"/>
-      <c r="L38" s="15"/>
-      <c r="M38" s="15"/>
-      <c r="P38" s="21" t="s">
+      <c r="H38" s="16"/>
+      <c r="I38" s="16"/>
+      <c r="J38" s="16"/>
+      <c r="K38" s="16"/>
+      <c r="L38" s="16"/>
+      <c r="M38" s="16"/>
+      <c r="P38" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="Q38" s="15">
+      <c r="Q38" s="16">
         <v>1716</v>
       </c>
-      <c r="R38" s="15">
+      <c r="R38" s="16">
         <v>28</v>
       </c>
-      <c r="S38" s="15">
+      <c r="S38" s="16">
         <v>8</v>
       </c>
-      <c r="T38" s="20">
-        <v>3</v>
-      </c>
-      <c r="U38" s="15">
-        <v>3</v>
-      </c>
-      <c r="V38" s="15">
+      <c r="T38" s="21">
+        <v>3</v>
+      </c>
+      <c r="U38" s="16">
+        <v>3</v>
+      </c>
+      <c r="V38" s="16">
         <v>4</v>
       </c>
       <c r="W38" s="6" t="s">
@@ -4161,31 +4164,31 @@
       </c>
     </row>
     <row r="39" spans="8:23" x14ac:dyDescent="0.25">
-      <c r="H39" s="15"/>
-      <c r="I39" s="15"/>
-      <c r="J39" s="15"/>
-      <c r="K39" s="15"/>
-      <c r="L39" s="15"/>
-      <c r="M39" s="15"/>
-      <c r="P39" s="21" t="s">
+      <c r="H39" s="16"/>
+      <c r="I39" s="16"/>
+      <c r="J39" s="16"/>
+      <c r="K39" s="16"/>
+      <c r="L39" s="16"/>
+      <c r="M39" s="16"/>
+      <c r="P39" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="Q39" s="15">
+      <c r="Q39" s="16">
         <v>1728</v>
       </c>
-      <c r="R39" s="15">
+      <c r="R39" s="16">
         <v>28</v>
       </c>
-      <c r="S39" s="15">
+      <c r="S39" s="16">
         <v>8</v>
       </c>
-      <c r="T39" s="20">
+      <c r="T39" s="21">
         <v>5.5</v>
       </c>
-      <c r="U39" s="15">
-        <v>3</v>
-      </c>
-      <c r="V39" s="15">
+      <c r="U39" s="16">
+        <v>3</v>
+      </c>
+      <c r="V39" s="16">
         <v>4</v>
       </c>
       <c r="W39" s="6" t="s">
@@ -4193,49 +4196,49 @@
       </c>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B40" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="C40" s="17" t="s">
+      <c r="C40" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="D40" s="17" t="s">
+      <c r="D40" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E40" s="17" t="s">
+      <c r="E40" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="F40" s="17" t="s">
+      <c r="F40" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="H40" s="15"/>
-      <c r="I40" s="15"/>
-      <c r="J40" s="15"/>
-      <c r="K40" s="15"/>
-      <c r="L40" s="15"/>
-      <c r="M40" s="15"/>
-      <c r="P40" s="21" t="s">
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="16"/>
+      <c r="L40" s="16"/>
+      <c r="M40" s="16"/>
+      <c r="P40" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="Q40" s="15">
+      <c r="Q40" s="16">
         <v>1728</v>
       </c>
-      <c r="R40" s="15">
+      <c r="R40" s="16">
         <v>38</v>
       </c>
-      <c r="S40" s="15">
+      <c r="S40" s="16">
         <v>10</v>
       </c>
-      <c r="T40" s="20">
+      <c r="T40" s="21">
         <v>7.5</v>
       </c>
-      <c r="U40" s="15">
-        <v>3</v>
-      </c>
-      <c r="V40" s="15">
+      <c r="U40" s="16">
+        <v>3</v>
+      </c>
+      <c r="V40" s="16">
         <v>4</v>
       </c>
       <c r="W40" s="6" t="s">
@@ -4243,49 +4246,49 @@
       </c>
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A41" s="15">
+      <c r="A41" s="16">
         <v>1</v>
       </c>
-      <c r="B41" s="15">
+      <c r="B41" s="16">
         <v>220</v>
       </c>
-      <c r="C41" s="15">
+      <c r="C41" s="16">
         <v>60</v>
       </c>
-      <c r="D41" s="15">
+      <c r="D41" s="16">
         <v>2</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="F41" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="H41" s="15"/>
-      <c r="I41" s="15"/>
-      <c r="J41" s="15"/>
-      <c r="K41" s="15"/>
-      <c r="L41" s="15"/>
-      <c r="M41" s="15"/>
-      <c r="P41" s="21" t="s">
+      <c r="H41" s="16"/>
+      <c r="I41" s="16"/>
+      <c r="J41" s="16"/>
+      <c r="K41" s="16"/>
+      <c r="L41" s="16"/>
+      <c r="M41" s="16"/>
+      <c r="P41" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="Q41" s="15">
+      <c r="Q41" s="16">
         <v>1728</v>
       </c>
-      <c r="R41" s="15">
+      <c r="R41" s="16">
         <v>38</v>
       </c>
-      <c r="S41" s="15">
+      <c r="S41" s="16">
         <v>10</v>
       </c>
-      <c r="T41" s="20">
+      <c r="T41" s="21">
         <v>10</v>
       </c>
-      <c r="U41" s="15">
-        <v>3</v>
-      </c>
-      <c r="V41" s="15">
+      <c r="U41" s="16">
+        <v>3</v>
+      </c>
+      <c r="V41" s="16">
         <v>4</v>
       </c>
       <c r="W41" s="6" t="s">
@@ -4293,49 +4296,49 @@
       </c>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A42" s="15">
-        <v>3</v>
-      </c>
-      <c r="B42" s="15">
+      <c r="A42" s="16">
+        <v>3</v>
+      </c>
+      <c r="B42" s="16">
         <v>380</v>
       </c>
-      <c r="C42" s="15">
+      <c r="C42" s="16">
         <v>50</v>
       </c>
-      <c r="D42" s="15">
-        <v>4</v>
-      </c>
-      <c r="E42" s="3" t="s">
+      <c r="D42" s="16">
+        <v>4</v>
+      </c>
+      <c r="E42" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="F42" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="H42" s="15"/>
-      <c r="I42" s="15"/>
-      <c r="J42" s="15"/>
-      <c r="K42" s="15"/>
-      <c r="L42" s="15"/>
-      <c r="M42" s="15"/>
-      <c r="P42" s="21" t="s">
+      <c r="H42" s="16"/>
+      <c r="I42" s="16"/>
+      <c r="J42" s="16"/>
+      <c r="K42" s="16"/>
+      <c r="L42" s="16"/>
+      <c r="M42" s="16"/>
+      <c r="P42" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="Q42" s="15">
+      <c r="Q42" s="16">
         <v>1728</v>
       </c>
-      <c r="R42" s="15">
+      <c r="R42" s="16">
         <v>42</v>
       </c>
-      <c r="S42" s="15">
+      <c r="S42" s="16">
         <v>12</v>
       </c>
-      <c r="T42" s="20">
+      <c r="T42" s="21">
         <v>15</v>
       </c>
-      <c r="U42" s="15">
-        <v>3</v>
-      </c>
-      <c r="V42" s="15">
+      <c r="U42" s="16">
+        <v>3</v>
+      </c>
+      <c r="V42" s="16">
         <v>4</v>
       </c>
       <c r="W42" s="6" t="s">
@@ -4343,38 +4346,38 @@
       </c>
     </row>
     <row r="43" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B43" s="15">
+      <c r="B43" s="16">
         <v>440</v>
       </c>
-      <c r="D43" s="15">
+      <c r="D43" s="16">
         <v>6</v>
       </c>
-      <c r="F43" s="3"/>
-      <c r="H43" s="15"/>
-      <c r="I43" s="15"/>
-      <c r="J43" s="15"/>
-      <c r="K43" s="15"/>
-      <c r="L43" s="15"/>
-      <c r="M43" s="15"/>
-      <c r="P43" s="21" t="s">
+      <c r="F43" s="13"/>
+      <c r="H43" s="16"/>
+      <c r="I43" s="16"/>
+      <c r="J43" s="16"/>
+      <c r="K43" s="16"/>
+      <c r="L43" s="16"/>
+      <c r="M43" s="16"/>
+      <c r="P43" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="Q43" s="15">
+      <c r="Q43" s="16">
         <v>1752</v>
       </c>
-      <c r="R43" s="15">
+      <c r="R43" s="16">
         <v>42</v>
       </c>
-      <c r="S43" s="15">
+      <c r="S43" s="16">
         <v>12</v>
       </c>
-      <c r="T43" s="20">
+      <c r="T43" s="21">
         <v>20</v>
       </c>
-      <c r="U43" s="15">
-        <v>3</v>
-      </c>
-      <c r="V43" s="15">
+      <c r="U43" s="16">
+        <v>3</v>
+      </c>
+      <c r="V43" s="16">
         <v>4</v>
       </c>
       <c r="W43" s="6" t="s">
@@ -4382,35 +4385,35 @@
       </c>
     </row>
     <row r="44" spans="4:23" x14ac:dyDescent="0.25">
-      <c r="D44" s="15">
+      <c r="D44" s="16">
         <v>8</v>
       </c>
-      <c r="F44" s="3"/>
-      <c r="H44" s="3"/>
-      <c r="I44" s="3"/>
-      <c r="J44" s="3"/>
-      <c r="K44" s="3"/>
-      <c r="L44" s="3"/>
-      <c r="M44" s="3"/>
-      <c r="P44" s="21" t="s">
+      <c r="F44" s="13"/>
+      <c r="H44" s="13"/>
+      <c r="I44" s="13"/>
+      <c r="J44" s="13"/>
+      <c r="K44" s="13"/>
+      <c r="L44" s="13"/>
+      <c r="M44" s="13"/>
+      <c r="P44" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="Q44" s="15">
+      <c r="Q44" s="16">
         <v>1752</v>
       </c>
-      <c r="R44" s="15">
+      <c r="R44" s="16">
         <v>48</v>
       </c>
-      <c r="S44" s="15">
+      <c r="S44" s="16">
         <v>14</v>
       </c>
-      <c r="T44" s="20">
+      <c r="T44" s="21">
         <v>25</v>
       </c>
-      <c r="U44" s="15">
-        <v>3</v>
-      </c>
-      <c r="V44" s="15">
+      <c r="U44" s="16">
+        <v>3</v>
+      </c>
+      <c r="V44" s="16">
         <v>4</v>
       </c>
       <c r="W44" s="6" t="s">
@@ -4418,27 +4421,27 @@
       </c>
     </row>
     <row r="45" spans="4:23" x14ac:dyDescent="0.25">
-      <c r="D45" s="15"/>
-      <c r="F45" s="3"/>
-      <c r="P45" s="21" t="s">
+      <c r="D45" s="16"/>
+      <c r="F45" s="13"/>
+      <c r="P45" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="Q45" s="15">
+      <c r="Q45" s="16">
         <v>1764</v>
       </c>
-      <c r="R45" s="15">
+      <c r="R45" s="16">
         <v>48</v>
       </c>
-      <c r="S45" s="15">
+      <c r="S45" s="16">
         <v>14</v>
       </c>
-      <c r="T45" s="20">
+      <c r="T45" s="21">
         <v>30</v>
       </c>
-      <c r="U45" s="15">
-        <v>3</v>
-      </c>
-      <c r="V45" s="15">
+      <c r="U45" s="16">
+        <v>3</v>
+      </c>
+      <c r="V45" s="16">
         <v>4</v>
       </c>
       <c r="W45" s="6" t="s">
@@ -4446,31 +4449,31 @@
       </c>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A46" s="27"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="15"/>
-      <c r="D46" s="15"/>
-      <c r="E46" s="15"/>
-      <c r="F46" s="3"/>
-      <c r="P46" s="21" t="s">
+      <c r="A46" s="28"/>
+      <c r="B46" s="15"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
+      <c r="F46" s="13"/>
+      <c r="P46" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="Q46" s="15">
+      <c r="Q46" s="16">
         <v>1764</v>
       </c>
-      <c r="R46" s="15">
+      <c r="R46" s="16">
         <v>55</v>
       </c>
-      <c r="S46" s="15">
+      <c r="S46" s="16">
         <v>16</v>
       </c>
-      <c r="T46" s="20">
+      <c r="T46" s="21">
         <v>40</v>
       </c>
-      <c r="U46" s="15">
-        <v>3</v>
-      </c>
-      <c r="V46" s="15">
+      <c r="U46" s="16">
+        <v>3</v>
+      </c>
+      <c r="V46" s="16">
         <v>4</v>
       </c>
       <c r="W46" s="6" t="s">
@@ -4478,31 +4481,31 @@
       </c>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A47" s="28" t="s">
+      <c r="A47" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="B47" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="P47" s="21" t="s">
+      <c r="P47" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="Q47" s="15">
+      <c r="Q47" s="16">
         <v>1764</v>
       </c>
-      <c r="R47" s="15">
+      <c r="R47" s="16">
         <v>55</v>
       </c>
-      <c r="S47" s="15">
+      <c r="S47" s="16">
         <v>16</v>
       </c>
-      <c r="T47" s="20">
+      <c r="T47" s="21">
         <v>50</v>
       </c>
-      <c r="U47" s="15">
-        <v>3</v>
-      </c>
-      <c r="V47" s="15">
+      <c r="U47" s="16">
+        <v>3</v>
+      </c>
+      <c r="V47" s="16">
         <v>4</v>
       </c>
       <c r="W47" s="6" t="s">
@@ -4510,31 +4513,31 @@
       </c>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A48" s="27" t="s">
+      <c r="A48" s="28" t="s">
         <v>169</v>
       </c>
-      <c r="B48" s="15" t="s">
+      <c r="B48" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="P48" s="21" t="s">
+      <c r="P48" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="Q48" s="15">
+      <c r="Q48" s="16">
         <v>1770</v>
       </c>
-      <c r="R48" s="15">
+      <c r="R48" s="16">
         <v>55</v>
       </c>
-      <c r="S48" s="15">
+      <c r="S48" s="16">
         <v>16</v>
       </c>
-      <c r="T48" s="20">
+      <c r="T48" s="21">
         <v>60</v>
       </c>
-      <c r="U48" s="15">
-        <v>3</v>
-      </c>
-      <c r="V48" s="15">
+      <c r="U48" s="16">
+        <v>3</v>
+      </c>
+      <c r="V48" s="16">
         <v>4</v>
       </c>
       <c r="W48" s="6" t="s">
@@ -4542,31 +4545,31 @@
       </c>
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A49" s="15" t="s">
+      <c r="A49" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="B49" s="15" t="s">
+      <c r="B49" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="P49" s="21" t="s">
+      <c r="P49" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="Q49" s="15">
+      <c r="Q49" s="16">
         <v>1770</v>
       </c>
-      <c r="R49" s="15">
+      <c r="R49" s="16">
         <v>60</v>
       </c>
-      <c r="S49" s="15">
+      <c r="S49" s="16">
         <v>18</v>
       </c>
-      <c r="T49" s="20">
+      <c r="T49" s="21">
         <v>75</v>
       </c>
-      <c r="U49" s="15">
-        <v>3</v>
-      </c>
-      <c r="V49" s="15">
+      <c r="U49" s="16">
+        <v>3</v>
+      </c>
+      <c r="V49" s="16">
         <v>4</v>
       </c>
       <c r="W49" s="6" t="s">
@@ -4574,31 +4577,31 @@
       </c>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A50" s="15" t="s">
+      <c r="A50" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="B50" s="15" t="s">
+      <c r="B50" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="P50" s="21" t="s">
+      <c r="P50" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="Q50" s="15">
+      <c r="Q50" s="16">
         <v>1776</v>
       </c>
-      <c r="R50" s="15">
+      <c r="R50" s="16">
         <v>75</v>
       </c>
-      <c r="S50" s="15">
+      <c r="S50" s="16">
         <v>20</v>
       </c>
-      <c r="T50" s="20">
+      <c r="T50" s="21">
         <v>100</v>
       </c>
-      <c r="U50" s="15">
-        <v>3</v>
-      </c>
-      <c r="V50" s="15">
+      <c r="U50" s="16">
+        <v>3</v>
+      </c>
+      <c r="V50" s="16">
         <v>4</v>
       </c>
       <c r="W50" s="6" t="s">
@@ -4606,31 +4609,31 @@
       </c>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A51" s="15" t="s">
+      <c r="A51" s="16" t="s">
         <v>175</v>
       </c>
-      <c r="B51" s="15" t="s">
+      <c r="B51" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="P51" s="21" t="s">
+      <c r="P51" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="Q51" s="15">
+      <c r="Q51" s="16">
         <v>1776</v>
       </c>
-      <c r="R51" s="15">
+      <c r="R51" s="16">
         <v>75</v>
       </c>
-      <c r="S51" s="15">
+      <c r="S51" s="16">
         <v>20</v>
       </c>
-      <c r="T51" s="20">
+      <c r="T51" s="21">
         <v>125</v>
       </c>
-      <c r="U51" s="15">
-        <v>3</v>
-      </c>
-      <c r="V51" s="15">
+      <c r="U51" s="16">
+        <v>3</v>
+      </c>
+      <c r="V51" s="16">
         <v>4</v>
       </c>
       <c r="W51" s="6" t="s">
@@ -4638,31 +4641,31 @@
       </c>
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A52" s="15" t="s">
+      <c r="A52" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="B52" s="15" t="s">
+      <c r="B52" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="P52" s="21" t="s">
+      <c r="P52" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="Q52" s="15">
+      <c r="Q52" s="16">
         <v>1776</v>
       </c>
-      <c r="R52" s="15">
+      <c r="R52" s="16">
         <v>80</v>
       </c>
-      <c r="S52" s="15">
+      <c r="S52" s="16">
         <v>22</v>
       </c>
-      <c r="T52" s="20">
+      <c r="T52" s="21">
         <v>150</v>
       </c>
-      <c r="U52" s="15">
-        <v>3</v>
-      </c>
-      <c r="V52" s="15">
+      <c r="U52" s="16">
+        <v>3</v>
+      </c>
+      <c r="V52" s="16">
         <v>4</v>
       </c>
       <c r="W52" s="6" t="s">
@@ -4670,31 +4673,31 @@
       </c>
     </row>
     <row r="53" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A53" s="15" t="s">
+      <c r="A53" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="B53" s="15" t="s">
+      <c r="B53" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="P53" s="21" t="s">
+      <c r="P53" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="Q53" s="15">
+      <c r="Q53" s="16">
         <v>1776</v>
       </c>
-      <c r="R53" s="15">
+      <c r="R53" s="16">
         <v>80</v>
       </c>
-      <c r="S53" s="15">
+      <c r="S53" s="16">
         <v>22</v>
       </c>
-      <c r="T53" s="20">
+      <c r="T53" s="21">
         <v>180</v>
       </c>
-      <c r="U53" s="15">
-        <v>3</v>
-      </c>
-      <c r="V53" s="15">
+      <c r="U53" s="16">
+        <v>3</v>
+      </c>
+      <c r="V53" s="16">
         <v>4</v>
       </c>
       <c r="W53" s="6" t="s">
@@ -4702,28 +4705,28 @@
       </c>
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A54" s="15" t="s">
+      <c r="A54" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="P54" s="21" t="s">
+      <c r="P54" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="Q54" s="15">
+      <c r="Q54" s="16">
         <v>1776</v>
       </c>
-      <c r="R54" s="15">
+      <c r="R54" s="16">
         <v>80</v>
       </c>
-      <c r="S54" s="15">
+      <c r="S54" s="16">
         <v>22</v>
       </c>
-      <c r="T54" s="20">
+      <c r="T54" s="21">
         <v>200</v>
       </c>
-      <c r="U54" s="15">
-        <v>3</v>
-      </c>
-      <c r="V54" s="15">
+      <c r="U54" s="16">
+        <v>3</v>
+      </c>
+      <c r="V54" s="16">
         <v>4</v>
       </c>
       <c r="W54" s="6" t="s">
@@ -4731,28 +4734,28 @@
       </c>
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A55" s="15" t="s">
+      <c r="A55" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="P55" s="21" t="s">
+      <c r="P55" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="Q55" s="15">
+      <c r="Q55" s="16">
         <v>1776</v>
       </c>
-      <c r="R55" s="15">
+      <c r="R55" s="16">
         <v>80</v>
       </c>
-      <c r="S55" s="15">
+      <c r="S55" s="16">
         <v>22</v>
       </c>
-      <c r="T55" s="20">
+      <c r="T55" s="21">
         <v>270</v>
       </c>
-      <c r="U55" s="15">
-        <v>3</v>
-      </c>
-      <c r="V55" s="15">
+      <c r="U55" s="16">
+        <v>3</v>
+      </c>
+      <c r="V55" s="16">
         <v>4</v>
       </c>
       <c r="W55" s="6" t="s">
@@ -4760,28 +4763,28 @@
       </c>
     </row>
     <row r="56" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A56" s="15" t="s">
+      <c r="A56" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="P56" s="21" t="s">
+      <c r="P56" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="Q56" s="15">
+      <c r="Q56" s="16">
         <v>1788</v>
       </c>
-      <c r="R56" s="15">
+      <c r="R56" s="16">
         <v>95</v>
       </c>
-      <c r="S56" s="15">
+      <c r="S56" s="16">
         <v>25</v>
       </c>
-      <c r="T56" s="20">
+      <c r="T56" s="21">
         <v>340</v>
       </c>
-      <c r="U56" s="15">
-        <v>3</v>
-      </c>
-      <c r="V56" s="15">
+      <c r="U56" s="16">
+        <v>3</v>
+      </c>
+      <c r="V56" s="16">
         <v>4</v>
       </c>
       <c r="W56" s="6" t="s">
@@ -4789,435 +4792,435 @@
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" s="17" t="s">
+      <c r="A59" s="18" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" s="15" t="s">
+      <c r="A60" s="16" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" s="15" t="s">
+      <c r="A61" s="16" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" s="15" t="s">
+      <c r="A62" s="16" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A63" s="29"/>
-      <c r="B63" s="29"/>
-      <c r="C63" s="30"/>
-      <c r="D63" s="30"/>
-      <c r="E63" s="30"/>
-      <c r="F63" s="31"/>
-      <c r="G63" s="31"/>
-      <c r="H63" s="31"/>
-      <c r="I63" s="31"/>
-      <c r="J63" s="31"/>
-      <c r="K63" s="31"/>
-      <c r="L63" s="31"/>
-      <c r="M63" s="31"/>
-      <c r="N63" s="31"/>
-      <c r="O63" s="31"/>
-      <c r="P63" s="31"/>
-      <c r="Q63" s="31"/>
-      <c r="R63" s="31"/>
-      <c r="S63" s="31"/>
-      <c r="T63" s="32"/>
-      <c r="U63" s="32"/>
-      <c r="V63" s="31"/>
-      <c r="W63" s="32"/>
-      <c r="X63" s="31"/>
+      <c r="A63" s="30"/>
+      <c r="B63" s="30"/>
+      <c r="C63" s="31"/>
+      <c r="D63" s="31"/>
+      <c r="E63" s="31"/>
+      <c r="F63" s="32"/>
+      <c r="G63" s="32"/>
+      <c r="H63" s="32"/>
+      <c r="I63" s="32"/>
+      <c r="J63" s="32"/>
+      <c r="K63" s="32"/>
+      <c r="L63" s="32"/>
+      <c r="M63" s="32"/>
+      <c r="N63" s="32"/>
+      <c r="O63" s="32"/>
+      <c r="P63" s="32"/>
+      <c r="Q63" s="32"/>
+      <c r="R63" s="32"/>
+      <c r="S63" s="32"/>
+      <c r="T63" s="33"/>
+      <c r="U63" s="33"/>
+      <c r="V63" s="32"/>
+      <c r="W63" s="33"/>
+      <c r="X63" s="32"/>
     </row>
     <row r="64" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="33" t="s">
+      <c r="A64" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="B64" s="34"/>
-      <c r="C64" s="3" t="s">
+      <c r="B64" s="35"/>
+      <c r="C64" s="13" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="35" t="s">
-        <v>3</v>
-      </c>
-      <c r="B65" s="36">
+      <c r="A65" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B65" s="37">
         <v>46168</v>
       </c>
-      <c r="C65" s="37" t="s">
+      <c r="C65" s="38" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="38" t="s">
+      <c r="A66" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="B66" s="39" t="s">
+      <c r="B66" s="40" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="38" t="s">
+      <c r="A67" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="B67" s="40" t="s">
+      <c r="B67" s="41" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="38" t="s">
+      <c r="A68" s="39" t="s">
         <v>149</v>
       </c>
-      <c r="B68" s="40" t="s">
+      <c r="B68" s="41" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="38" t="s">
+      <c r="A69" s="39" t="s">
         <v>192</v>
       </c>
-      <c r="B69" s="41">
+      <c r="B69" s="42">
         <v>46179</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="38" t="s">
+      <c r="A70" s="39" t="s">
         <v>193</v>
       </c>
-      <c r="B70" s="40">
+      <c r="B70" s="41">
         <v>2</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="38" t="s">
+      <c r="A71" s="39" t="s">
         <v>194</v>
       </c>
-      <c r="B71" s="40" t="s">
+      <c r="B71" s="41" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="38" t="s">
+      <c r="A72" s="39" t="s">
         <v>196</v>
       </c>
-      <c r="B72" s="40">
+      <c r="B72" s="41">
         <v>14</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="42" t="s">
+      <c r="A73" s="43" t="s">
         <v>197</v>
       </c>
-      <c r="B73" s="43">
+      <c r="B73" s="44">
         <v>10</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="75" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="44" t="s">
+      <c r="A75" s="45" t="s">
         <v>198</v>
       </c>
-      <c r="B75" s="45"/>
-      <c r="C75" s="29" t="s">
+      <c r="B75" s="46"/>
+      <c r="C75" s="30" t="s">
         <v>199</v>
       </c>
-      <c r="D75" s="32"/>
+      <c r="D75" s="33"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="35" t="s">
+      <c r="A76" s="36" t="s">
         <v>200</v>
       </c>
-      <c r="B76" s="46" t="str">
+      <c r="B76" s="47" t="str">
         <f>VLOOKUP(B67,B67,1)</f>
         <v>CEB</v>
       </c>
-      <c r="C76" s="15" t="s">
+      <c r="C76" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="D76" s="15">
+      <c r="D76" s="16">
         <f>SUM(D89*B96)/B97</f>
         <v>598.1538461538462</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="47" t="s">
+      <c r="A77" s="48" t="s">
         <v>51</v>
       </c>
-      <c r="B77" s="48">
+      <c r="B77" s="49">
         <v>44.5</v>
       </c>
-      <c r="C77" s="27" t="s">
+      <c r="C77" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="D77" s="15" t="str">
+      <c r="D77" s="16" t="str">
         <f>VLOOKUP(B77,A4:E25,4)</f>
         <v>2 1/4”Ø x 1/2" keyway</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="47" t="s">
+      <c r="A78" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="B78" s="40" t="s">
+      <c r="B78" s="41" t="s">
         <v>169</v>
       </c>
-      <c r="C78" s="27" t="s">
+      <c r="C78" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="D78" s="15" t="str">
+      <c r="D78" s="16" t="str">
         <f>VLOOKUP(B77,A4:E25,5)</f>
         <v>UCP212</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="47" t="s">
+      <c r="A79" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="B79" s="40" t="s">
+      <c r="B79" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="C79" s="27" t="s">
+      <c r="C79" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="D79" s="15" t="str">
+      <c r="D79" s="16" t="str">
         <f>VLOOKUP(B77,A4:E25,3)</f>
         <v>4”Ø x 4”L x 2 1/4"Ø bore x 1/2” keyway</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="47" t="s">
+      <c r="A80" s="48" t="s">
         <v>202</v>
       </c>
-      <c r="B80" s="40" t="s">
+      <c r="B80" s="41" t="s">
         <v>150</v>
       </c>
-      <c r="C80" s="27" t="s">
+      <c r="C80" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="D80" s="15" t="str">
+      <c r="D80" s="16" t="str">
         <f>VLOOKUP(B77,A4:E25,2)</f>
         <v>2 1/4”Ø x 1/2" keyway</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="47" t="s">
+      <c r="A81" s="48" t="s">
         <v>203</v>
       </c>
-      <c r="B81" s="40" t="s">
+      <c r="B81" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="C81" s="27" t="s">
+      <c r="C81" s="28" t="s">
         <v>204</v>
       </c>
-      <c r="D81" s="15">
+      <c r="D81" s="16">
         <f>VLOOKUP(B77,A4:F25,6)</f>
         <v>2.25</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="38" t="s">
+      <c r="A82" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="B82" s="40" t="s">
+      <c r="B82" s="41" t="s">
         <v>205</v>
       </c>
-      <c r="D82" s="15"/>
+      <c r="D82" s="16"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="38" t="s">
+      <c r="A83" s="39" t="s">
         <v>206</v>
       </c>
-      <c r="B83" s="40" t="s">
+      <c r="B83" s="41" t="s">
         <v>207</v>
       </c>
-      <c r="D83" s="15"/>
+      <c r="D83" s="16"/>
     </row>
     <row r="84" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="42" t="s">
+      <c r="A84" s="43" t="s">
         <v>208</v>
       </c>
-      <c r="B84" s="43">
+      <c r="B84" s="44">
         <v>595</v>
       </c>
-      <c r="D84" s="15"/>
+      <c r="D84" s="16"/>
     </row>
     <row r="85" ht="15" customHeight="1" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D85" s="15"/>
+      <c r="D85" s="16"/>
     </row>
     <row r="86" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="44" t="s">
+      <c r="A86" s="45" t="s">
         <v>209</v>
       </c>
-      <c r="B86" s="45"/>
-      <c r="C86" s="29" t="s">
+      <c r="B86" s="46"/>
+      <c r="C86" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="D86" s="32"/>
+      <c r="D86" s="33"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="49" t="s">
+      <c r="A87" s="50" t="s">
         <v>211</v>
       </c>
-      <c r="B87" s="50" t="s">
+      <c r="B87" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="C87" s="27" t="s">
+      <c r="C87" s="28" t="s">
         <v>212</v>
       </c>
-      <c r="D87" s="51">
+      <c r="D87" s="52">
         <f>VLOOKUP(TRIM(B89),P3:W56,5,FALSE)</f>
         <v>15</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="47" t="s">
+      <c r="A88" s="48" t="s">
         <v>213</v>
       </c>
-      <c r="B88" s="40" t="s">
+      <c r="B88" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="C88" s="27" t="s">
+      <c r="C88" s="28" t="s">
         <v>214</v>
       </c>
-      <c r="D88" s="15">
+      <c r="D88" s="16">
         <f>VLOOKUP(TRIM(B89),P3:W56,6,FALSE)</f>
         <v>3</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="47" t="s">
+      <c r="A89" s="48" t="s">
         <v>212</v>
       </c>
-      <c r="B89" s="40" t="s">
+      <c r="B89" s="41" t="s">
         <v>91</v>
       </c>
-      <c r="C89" s="15" t="s">
+      <c r="C89" s="16" t="s">
         <v>215</v>
       </c>
-      <c r="D89" s="52">
+      <c r="D89" s="53">
         <f>VLOOKUP(TRIM(B89),P3:W56,2,FALSE)</f>
         <v>1728</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="47" t="s">
+      <c r="A90" s="48" t="s">
         <v>160</v>
       </c>
-      <c r="B90" s="40">
+      <c r="B90" s="41">
         <v>220</v>
       </c>
-      <c r="C90" s="15" t="s">
+      <c r="C90" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="D90" s="15">
+      <c r="D90" s="16">
         <f>VLOOKUP(TRIM(B89),P3:W56,7,FALSE)</f>
         <v>4</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="38" t="s">
+      <c r="A91" s="39" t="s">
         <v>161</v>
       </c>
-      <c r="B91" s="40">
+      <c r="B91" s="41">
         <v>60</v>
       </c>
-      <c r="C91" s="15" t="s">
+      <c r="C91" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="D91" s="15">
+      <c r="D91" s="16">
         <f>VLOOKUP(TRIM(B89),P3:W56,3,FALSE)</f>
         <v>42</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="38" t="s">
+      <c r="A92" s="39" t="s">
         <v>162</v>
       </c>
-      <c r="B92" s="40" t="s">
+      <c r="B92" s="41" t="s">
         <v>164</v>
       </c>
-      <c r="C92" s="15" t="s">
+      <c r="C92" s="16" t="s">
         <v>217</v>
       </c>
-      <c r="D92" s="15">
+      <c r="D92" s="16">
         <f>VLOOKUP(TRIM(B89),P3:W56,4,FALSE)</f>
         <v>12</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="38" t="s">
+      <c r="A93" s="39" t="s">
         <v>163</v>
       </c>
-      <c r="B93" s="40" t="s">
+      <c r="B93" s="41" t="s">
         <v>165</v>
       </c>
-      <c r="C93" s="27" t="s">
+      <c r="C93" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="D93" s="15" t="str">
+      <c r="D93" s="16" t="str">
         <f>VLOOKUP(TRIM(B89),P3:W56,8,FALSE)</f>
         <v>3B</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="38" t="s">
+      <c r="A94" s="39" t="s">
         <v>215</v>
       </c>
-      <c r="B94" s="53">
+      <c r="B94" s="54">
         <f>VLOOKUP(D89,D89,1)</f>
         <v>1728</v>
       </c>
-      <c r="C94" s="27" t="s">
+      <c r="C94" s="28" t="s">
         <v>218</v>
       </c>
-      <c r="D94" s="15">
+      <c r="D94" s="16">
         <f>SUM(D91)+36</f>
         <v>78</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="38" t="s">
+      <c r="A95" s="39" t="s">
         <v>208</v>
       </c>
-      <c r="B95" s="53">
+      <c r="B95" s="54">
         <f>VLOOKUP(B84,B84,1)</f>
         <v>595</v>
       </c>
-      <c r="C95" s="15" t="s">
+      <c r="C95" s="16" t="s">
         <v>219</v>
       </c>
-      <c r="D95" s="15">
+      <c r="D95" s="16">
         <f>ROUNDUP(SUM(D81*25.4)+36, 0)</f>
         <v>94</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96" s="38" t="s">
+      <c r="A96" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="B96" s="54">
+      <c r="B96" s="55">
         <v>4.5</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" s="38" t="s">
+      <c r="A97" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="B97" s="54">
+      <c r="B97" s="55">
         <v>13</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" s="42" t="s">
+      <c r="A98" s="43" t="s">
         <v>201</v>
       </c>
-      <c r="B98" s="55">
+      <c r="B98" s="56">
         <f>VLOOKUP(D76,D76,1)</f>
         <v>598.1538461538462</v>
       </c>

</xml_diff>

<commit_message>
JO: left-align Capacity, pulleys, Hub, Shafting, Bearing (Shafting starts at C too)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HNv2pt2j3pqxEC7sBHUC3k
</commit_message>
<xml_diff>
--- a/public/templates/fans-jo-template.xlsx
+++ b/public/templates/fans-jo-template.xlsx
@@ -856,7 +856,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -865,7 +865,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -893,10 +893,13 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="12" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2098,12 +2101,12 @@
       <c r="N50" s="3"/>
       <c r="O50" s="3"/>
       <c r="P50" s="3"/>
-      <c r="Q50" s="16"/>
-      <c r="R50" s="16"/>
-      <c r="S50" s="16"/>
-      <c r="T50" s="16"/>
-      <c r="U50" s="16"/>
-      <c r="V50" s="16"/>
+      <c r="Q50" s="3"/>
+      <c r="R50" s="3"/>
+      <c r="S50" s="3"/>
+      <c r="T50" s="3"/>
+      <c r="U50" s="3"/>
+      <c r="V50" s="3"/>
       <c r="W50" s="16"/>
       <c r="X50" s="13"/>
     </row>
@@ -2142,28 +2145,28 @@
       <c r="B52" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D52" s="3" t="str">
+      <c r="C52" s="17">
         <f>Source!D80</f>
-        <v>2 1/4”Ø x 1/2" keyway</v>
-      </c>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
-      <c r="H52" s="5"/>
-      <c r="I52" s="5"/>
-      <c r="J52" s="5"/>
-      <c r="K52" s="5"/>
-      <c r="L52" s="5"/>
-      <c r="M52" s="5"/>
-      <c r="N52" s="13"/>
-      <c r="O52" s="13"/>
-      <c r="P52" s="13"/>
-      <c r="Q52" s="13"/>
-      <c r="R52" s="13"/>
-      <c r="S52" s="13"/>
-      <c r="T52" s="13"/>
-      <c r="U52" s="13"/>
-      <c r="V52" s="13"/>
+      </c>
+      <c r="D52" s="17"/>
+      <c r="E52" s="17"/>
+      <c r="F52" s="17"/>
+      <c r="G52" s="17"/>
+      <c r="H52" s="17"/>
+      <c r="I52" s="17"/>
+      <c r="J52" s="17"/>
+      <c r="K52" s="17"/>
+      <c r="L52" s="17"/>
+      <c r="M52" s="17"/>
+      <c r="N52" s="17"/>
+      <c r="O52" s="17"/>
+      <c r="P52" s="17"/>
+      <c r="Q52" s="17"/>
+      <c r="R52" s="17"/>
+      <c r="S52" s="17"/>
+      <c r="T52" s="17"/>
+      <c r="U52" s="17"/>
+      <c r="V52" s="17"/>
       <c r="W52" s="13"/>
       <c r="X52" s="13"/>
     </row>
@@ -2314,13 +2317,13 @@
       <c r="X57" s="13"/>
     </row>
     <row r="58" spans="19:23" x14ac:dyDescent="0.25">
-      <c r="S58" s="17" t="s">
+      <c r="S58" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="T58" s="17"/>
-      <c r="U58" s="17"/>
-      <c r="V58" s="17"/>
-      <c r="W58" s="17"/>
+      <c r="T58" s="18"/>
+      <c r="U58" s="18"/>
+      <c r="V58" s="18"/>
+      <c r="W58" s="18"/>
     </row>
     <row r="59" spans="23:23" x14ac:dyDescent="0.25">
       <c r="W59" s="7"/>
@@ -2347,8 +2350,8 @@
     <mergeCell ref="C44:V44"/>
     <mergeCell ref="C46:V46"/>
     <mergeCell ref="C48:V48"/>
-    <mergeCell ref="C50:P50"/>
-    <mergeCell ref="D52:M52"/>
+    <mergeCell ref="C50:V50"/>
+    <mergeCell ref="C52:V52"/>
     <mergeCell ref="C54:I54"/>
     <mergeCell ref="C56:V56"/>
     <mergeCell ref="S58:W58"/>
@@ -2384,13 +2387,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
       <c r="H2" s="6" t="s">
         <v>36</v>
       </c>
@@ -2465,16 +2468,16 @@
       <c r="J3" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="K3" s="20" t="s">
+      <c r="K3" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="L3" s="20" t="s">
+      <c r="L3" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="M3" s="20" t="s">
+      <c r="M3" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="P3" s="20" t="s">
+      <c r="P3" s="21" t="s">
         <v>55</v>
       </c>
       <c r="Q3" s="16">
@@ -2486,7 +2489,7 @@
       <c r="S3" s="16">
         <v>5</v>
       </c>
-      <c r="T3" s="21">
+      <c r="T3" s="22">
         <v>0.25</v>
       </c>
       <c r="U3" s="16">
@@ -2525,16 +2528,16 @@
         <v>40</v>
       </c>
       <c r="J4" s="16"/>
-      <c r="K4" s="22" t="s">
+      <c r="K4" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="L4" s="22" t="s">
+      <c r="L4" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="M4" s="22" t="s">
+      <c r="M4" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="P4" s="22" t="s">
+      <c r="P4" s="23" t="s">
         <v>63</v>
       </c>
       <c r="Q4" s="16">
@@ -2546,7 +2549,7 @@
       <c r="S4" s="16">
         <v>6</v>
       </c>
-      <c r="T4" s="21">
+      <c r="T4" s="22">
         <v>0.5</v>
       </c>
       <c r="U4" s="16">
@@ -2581,16 +2584,16 @@
       <c r="H5" s="16"/>
       <c r="I5" s="16"/>
       <c r="J5" s="16"/>
-      <c r="K5" s="22" t="s">
+      <c r="K5" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="L5" s="22" t="s">
+      <c r="L5" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="M5" s="22" t="s">
+      <c r="M5" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="P5" s="22" t="s">
+      <c r="P5" s="23" t="s">
         <v>66</v>
       </c>
       <c r="Q5" s="16">
@@ -2602,7 +2605,7 @@
       <c r="S5" s="16">
         <v>6</v>
       </c>
-      <c r="T5" s="21">
+      <c r="T5" s="22">
         <v>0.75</v>
       </c>
       <c r="U5" s="16">
@@ -2619,10 +2622,10 @@
       <c r="A6" s="16">
         <v>12.25</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="25" t="s">
         <v>70</v>
       </c>
       <c r="D6" s="13" t="s">
@@ -2631,22 +2634,22 @@
       <c r="E6" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="25">
+      <c r="F6" s="26">
         <v>1.25</v>
       </c>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
       <c r="J6" s="16"/>
-      <c r="K6" s="22" t="s">
+      <c r="K6" s="23" t="s">
         <v>73</v>
       </c>
-      <c r="L6" s="22" t="s">
+      <c r="L6" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="M6" s="22" t="s">
+      <c r="M6" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="P6" s="22" t="s">
+      <c r="P6" s="23" t="s">
         <v>73</v>
       </c>
       <c r="Q6" s="16">
@@ -2658,7 +2661,7 @@
       <c r="S6" s="16">
         <v>8</v>
       </c>
-      <c r="T6" s="26">
+      <c r="T6" s="27">
         <v>1</v>
       </c>
       <c r="U6" s="16">
@@ -2675,10 +2678,10 @@
       <c r="A7" s="16">
         <v>13.5</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="25" t="s">
         <v>70</v>
       </c>
       <c r="D7" s="13" t="s">
@@ -2687,22 +2690,22 @@
       <c r="E7" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F7" s="25">
+      <c r="F7" s="26">
         <v>1.25</v>
       </c>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
       <c r="J7" s="16"/>
-      <c r="K7" s="22" t="s">
+      <c r="K7" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="L7" s="22" t="s">
+      <c r="L7" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="M7" s="22" t="s">
+      <c r="M7" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="P7" s="22" t="s">
+      <c r="P7" s="23" t="s">
         <v>77</v>
       </c>
       <c r="Q7" s="16">
@@ -2714,7 +2717,7 @@
       <c r="S7" s="16">
         <v>8</v>
       </c>
-      <c r="T7" s="21">
+      <c r="T7" s="22">
         <v>1.5</v>
       </c>
       <c r="U7" s="16">
@@ -2731,10 +2734,10 @@
       <c r="A8" s="16">
         <v>15</v>
       </c>
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="25" t="s">
         <v>70</v>
       </c>
       <c r="D8" s="13" t="s">
@@ -2743,22 +2746,22 @@
       <c r="E8" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F8" s="25">
+      <c r="F8" s="26">
         <v>1.25</v>
       </c>
       <c r="H8" s="16"/>
       <c r="I8" s="16"/>
       <c r="J8" s="16"/>
-      <c r="K8" s="22" t="s">
+      <c r="K8" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="L8" s="22" t="s">
+      <c r="L8" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="M8" s="22" t="s">
+      <c r="M8" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="P8" s="22" t="s">
+      <c r="P8" s="23" t="s">
         <v>81</v>
       </c>
       <c r="Q8" s="16">
@@ -2770,7 +2773,7 @@
       <c r="S8" s="16">
         <v>8</v>
       </c>
-      <c r="T8" s="21">
+      <c r="T8" s="22">
         <v>2</v>
       </c>
       <c r="U8" s="16">
@@ -2787,10 +2790,10 @@
       <c r="A9" s="16">
         <v>16.5</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="25" t="s">
         <v>70</v>
       </c>
       <c r="D9" s="13" t="s">
@@ -2799,22 +2802,22 @@
       <c r="E9" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="25">
+      <c r="F9" s="26">
         <v>1.25</v>
       </c>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
       <c r="J9" s="16"/>
-      <c r="K9" s="22" t="s">
+      <c r="K9" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="L9" s="22" t="s">
+      <c r="L9" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="M9" s="22" t="s">
+      <c r="M9" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="P9" s="22" t="s">
+      <c r="P9" s="23" t="s">
         <v>84</v>
       </c>
       <c r="Q9" s="16">
@@ -2826,7 +2829,7 @@
       <c r="S9" s="16">
         <v>8</v>
       </c>
-      <c r="T9" s="21">
+      <c r="T9" s="22">
         <v>3</v>
       </c>
       <c r="U9" s="16">
@@ -2843,10 +2846,10 @@
       <c r="A10" s="16">
         <v>18.25</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="25" t="s">
         <v>70</v>
       </c>
       <c r="D10" s="13" t="s">
@@ -2855,22 +2858,22 @@
       <c r="E10" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="26">
         <v>1.25</v>
       </c>
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
       <c r="J10" s="16"/>
-      <c r="K10" s="22" t="s">
+      <c r="K10" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="L10" s="22" t="s">
+      <c r="L10" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="M10" s="22" t="s">
+      <c r="M10" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="P10" s="22" t="s">
+      <c r="P10" s="23" t="s">
         <v>87</v>
       </c>
       <c r="Q10" s="16">
@@ -2882,7 +2885,7 @@
       <c r="S10" s="16">
         <v>8</v>
       </c>
-      <c r="T10" s="21">
+      <c r="T10" s="22">
         <v>5</v>
       </c>
       <c r="U10" s="16">
@@ -2899,10 +2902,10 @@
       <c r="A11" s="16">
         <v>20</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="25" t="s">
         <v>70</v>
       </c>
       <c r="D11" s="13" t="s">
@@ -2911,23 +2914,23 @@
       <c r="E11" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="25">
+      <c r="F11" s="26">
         <v>1.25</v>
       </c>
       <c r="H11" s="16"/>
       <c r="I11" s="16"/>
       <c r="J11" s="16"/>
       <c r="K11" s="16"/>
-      <c r="L11" s="22" t="s">
+      <c r="L11" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="M11" s="22" t="s">
+      <c r="M11" s="23" t="s">
         <v>91</v>
       </c>
       <c r="O11" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="P11" s="20" t="s">
+      <c r="P11" s="21" t="s">
         <v>56</v>
       </c>
       <c r="Q11" s="16">
@@ -2939,7 +2942,7 @@
       <c r="S11" s="16">
         <v>5</v>
       </c>
-      <c r="T11" s="21">
+      <c r="T11" s="22">
         <v>0.5</v>
       </c>
       <c r="U11" s="16">
@@ -2956,10 +2959,10 @@
       <c r="A12" s="16">
         <v>22.25</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="25" t="s">
         <v>70</v>
       </c>
       <c r="D12" s="13" t="s">
@@ -2968,20 +2971,20 @@
       <c r="E12" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="26">
         <v>1.25</v>
       </c>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
       <c r="J12" s="16"/>
       <c r="K12" s="16"/>
-      <c r="L12" s="22" t="s">
+      <c r="L12" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="M12" s="22" t="s">
+      <c r="M12" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="P12" s="22" t="s">
+      <c r="P12" s="23" t="s">
         <v>64</v>
       </c>
       <c r="Q12" s="16">
@@ -2993,7 +2996,7 @@
       <c r="S12" s="16">
         <v>6</v>
       </c>
-      <c r="T12" s="21">
+      <c r="T12" s="22">
         <v>1</v>
       </c>
       <c r="U12" s="16">
@@ -3010,7 +3013,7 @@
       <c r="A13" s="16">
         <v>24.5</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="24" t="s">
         <v>95</v>
       </c>
       <c r="C13" s="13" t="s">
@@ -3022,20 +3025,20 @@
       <c r="E13" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="F13" s="25">
+      <c r="F13" s="26">
         <v>1.5</v>
       </c>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
       <c r="J13" s="16"/>
       <c r="K13" s="16"/>
-      <c r="L13" s="22" t="s">
+      <c r="L13" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="M13" s="22" t="s">
+      <c r="M13" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="P13" s="22" t="s">
+      <c r="P13" s="23" t="s">
         <v>67</v>
       </c>
       <c r="Q13" s="16">
@@ -3047,7 +3050,7 @@
       <c r="S13" s="16">
         <v>8</v>
       </c>
-      <c r="T13" s="21">
+      <c r="T13" s="22">
         <v>1.5</v>
       </c>
       <c r="U13" s="16">
@@ -3064,7 +3067,7 @@
       <c r="A14" s="16">
         <v>27</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="24" t="s">
         <v>95</v>
       </c>
       <c r="C14" s="13" t="s">
@@ -3076,20 +3079,20 @@
       <c r="E14" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="F14" s="25">
+      <c r="F14" s="26">
         <v>1.5</v>
       </c>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
       <c r="J14" s="16"/>
       <c r="K14" s="16"/>
-      <c r="L14" s="22" t="s">
+      <c r="L14" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="M14" s="22" t="s">
+      <c r="M14" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="P14" s="22" t="s">
+      <c r="P14" s="23" t="s">
         <v>74</v>
       </c>
       <c r="Q14" s="16">
@@ -3101,7 +3104,7 @@
       <c r="S14" s="16">
         <v>8</v>
       </c>
-      <c r="T14" s="21">
+      <c r="T14" s="22">
         <v>2</v>
       </c>
       <c r="U14" s="16">
@@ -3118,7 +3121,7 @@
       <c r="A15" s="16">
         <v>30</v>
       </c>
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="24" t="s">
         <v>103</v>
       </c>
       <c r="C15" s="13" t="s">
@@ -3130,20 +3133,20 @@
       <c r="E15" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="F15" s="25">
+      <c r="F15" s="26">
         <v>1.75</v>
       </c>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
       <c r="J15" s="16"/>
       <c r="K15" s="16"/>
-      <c r="L15" s="22" t="s">
+      <c r="L15" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="M15" s="22" t="s">
+      <c r="M15" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="P15" s="22" t="s">
+      <c r="P15" s="23" t="s">
         <v>78</v>
       </c>
       <c r="Q15" s="16">
@@ -3155,7 +3158,7 @@
       <c r="S15" s="16">
         <v>8</v>
       </c>
-      <c r="T15" s="21">
+      <c r="T15" s="22">
         <v>3</v>
       </c>
       <c r="U15" s="16">
@@ -3172,7 +3175,7 @@
       <c r="A16" s="16">
         <v>33</v>
       </c>
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="24" t="s">
         <v>109</v>
       </c>
       <c r="C16" s="13" t="s">
@@ -3184,20 +3187,20 @@
       <c r="E16" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="F16" s="25">
+      <c r="F16" s="26">
         <v>2</v>
       </c>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
       <c r="J16" s="16"/>
       <c r="K16" s="16"/>
-      <c r="L16" s="22" t="s">
+      <c r="L16" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="M16" s="22" t="s">
+      <c r="M16" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="P16" s="22" t="s">
+      <c r="P16" s="23" t="s">
         <v>82</v>
       </c>
       <c r="Q16" s="16">
@@ -3209,7 +3212,7 @@
       <c r="S16" s="16">
         <v>8</v>
       </c>
-      <c r="T16" s="21">
+      <c r="T16" s="22">
         <v>5</v>
       </c>
       <c r="U16" s="16">
@@ -3226,7 +3229,7 @@
       <c r="A17" s="16">
         <v>36.5</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="24" t="s">
         <v>109</v>
       </c>
       <c r="C17" s="13" t="s">
@@ -3238,20 +3241,20 @@
       <c r="E17" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="F17" s="25">
+      <c r="F17" s="26">
         <v>2</v>
       </c>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
       <c r="J17" s="16"/>
       <c r="K17" s="16"/>
-      <c r="L17" s="22" t="s">
+      <c r="L17" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="M17" s="22" t="s">
+      <c r="M17" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="P17" s="22" t="s">
+      <c r="P17" s="23" t="s">
         <v>85</v>
       </c>
       <c r="Q17" s="16">
@@ -3263,7 +3266,7 @@
       <c r="S17" s="16">
         <v>10</v>
       </c>
-      <c r="T17" s="21">
+      <c r="T17" s="22">
         <v>7.5</v>
       </c>
       <c r="U17" s="16">
@@ -3280,32 +3283,32 @@
       <c r="A18" s="16">
         <v>40.25</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="24" t="s">
         <v>117</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D18" s="28" t="s">
         <v>117</v>
       </c>
       <c r="E18" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="F18" s="25">
+      <c r="F18" s="26">
         <v>2.25</v>
       </c>
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
       <c r="J18" s="16"/>
       <c r="K18" s="16"/>
-      <c r="L18" s="22" t="s">
+      <c r="L18" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="M18" s="22" t="s">
+      <c r="M18" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="P18" s="22" t="s">
+      <c r="P18" s="23" t="s">
         <v>88</v>
       </c>
       <c r="Q18" s="16">
@@ -3317,7 +3320,7 @@
       <c r="S18" s="16">
         <v>10</v>
       </c>
-      <c r="T18" s="21">
+      <c r="T18" s="22">
         <v>10</v>
       </c>
       <c r="U18" s="16">
@@ -3334,32 +3337,32 @@
       <c r="A19" s="16">
         <v>44.5</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="24" t="s">
         <v>117</v>
       </c>
       <c r="C19" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="D19" s="27" t="s">
+      <c r="D19" s="28" t="s">
         <v>117</v>
       </c>
       <c r="E19" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="F19" s="25">
+      <c r="F19" s="26">
         <v>2.25</v>
       </c>
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="16"/>
       <c r="K19" s="16"/>
-      <c r="L19" s="22" t="s">
+      <c r="L19" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="M19" s="22" t="s">
+      <c r="M19" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="P19" s="22" t="s">
+      <c r="P19" s="23" t="s">
         <v>90</v>
       </c>
       <c r="Q19" s="16">
@@ -3371,7 +3374,7 @@
       <c r="S19" s="16">
         <v>12</v>
       </c>
-      <c r="T19" s="21">
+      <c r="T19" s="22">
         <v>15</v>
       </c>
       <c r="U19" s="16">
@@ -3388,7 +3391,7 @@
       <c r="A20" s="16">
         <v>49</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="24" t="s">
         <v>125</v>
       </c>
       <c r="C20" s="13" t="s">
@@ -3400,20 +3403,20 @@
       <c r="E20" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F20" s="25">
+      <c r="F20" s="26">
         <v>2.5</v>
       </c>
       <c r="H20" s="16"/>
       <c r="I20" s="16"/>
       <c r="J20" s="16"/>
       <c r="K20" s="16"/>
-      <c r="L20" s="22" t="s">
+      <c r="L20" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="M20" s="22" t="s">
+      <c r="M20" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="P20" s="22" t="s">
+      <c r="P20" s="23" t="s">
         <v>93</v>
       </c>
       <c r="Q20" s="16">
@@ -3425,7 +3428,7 @@
       <c r="S20" s="16">
         <v>12</v>
       </c>
-      <c r="T20" s="21">
+      <c r="T20" s="22">
         <v>20</v>
       </c>
       <c r="U20" s="16">
@@ -3442,7 +3445,7 @@
       <c r="A21" s="16">
         <v>54.5</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="24" t="s">
         <v>125</v>
       </c>
       <c r="C21" s="13" t="s">
@@ -3454,20 +3457,20 @@
       <c r="E21" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F21" s="25">
+      <c r="F21" s="26">
         <v>2.5</v>
       </c>
       <c r="H21" s="16"/>
       <c r="I21" s="16"/>
       <c r="J21" s="16"/>
       <c r="K21" s="16"/>
-      <c r="L21" s="22" t="s">
+      <c r="L21" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="M21" s="22" t="s">
+      <c r="M21" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="P21" s="22" t="s">
+      <c r="P21" s="23" t="s">
         <v>99</v>
       </c>
       <c r="Q21" s="16">
@@ -3479,7 +3482,7 @@
       <c r="S21" s="16">
         <v>14</v>
       </c>
-      <c r="T21" s="21">
+      <c r="T21" s="22">
         <v>25</v>
       </c>
       <c r="U21" s="16">
@@ -3496,7 +3499,7 @@
       <c r="A22" s="16">
         <v>60</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="24" t="s">
         <v>134</v>
       </c>
       <c r="C22" s="13" t="s">
@@ -3508,20 +3511,20 @@
       <c r="E22" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F22" s="25">
+      <c r="F22" s="26">
         <v>3</v>
       </c>
       <c r="H22" s="16"/>
       <c r="I22" s="16"/>
       <c r="J22" s="16"/>
       <c r="K22" s="16"/>
-      <c r="L22" s="22" t="s">
+      <c r="L22" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="M22" s="22" t="s">
+      <c r="M22" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="P22" s="22" t="s">
+      <c r="P22" s="23" t="s">
         <v>101</v>
       </c>
       <c r="Q22" s="16">
@@ -3533,7 +3536,7 @@
       <c r="S22" s="16">
         <v>14</v>
       </c>
-      <c r="T22" s="21">
+      <c r="T22" s="22">
         <v>30</v>
       </c>
       <c r="U22" s="16">
@@ -3550,7 +3553,7 @@
       <c r="A23" s="16">
         <v>66</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="24" t="s">
         <v>134</v>
       </c>
       <c r="C23" s="13" t="s">
@@ -3562,20 +3565,20 @@
       <c r="E23" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F23" s="25">
+      <c r="F23" s="26">
         <v>3</v>
       </c>
       <c r="H23" s="16"/>
       <c r="I23" s="16"/>
       <c r="J23" s="16"/>
       <c r="K23" s="16"/>
-      <c r="L23" s="22" t="s">
+      <c r="L23" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="M23" s="22" t="s">
+      <c r="M23" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="P23" s="22" t="s">
+      <c r="P23" s="23" t="s">
         <v>107</v>
       </c>
       <c r="Q23" s="16">
@@ -3587,7 +3590,7 @@
       <c r="S23" s="16">
         <v>16</v>
       </c>
-      <c r="T23" s="21">
+      <c r="T23" s="22">
         <v>40</v>
       </c>
       <c r="U23" s="16">
@@ -3604,7 +3607,7 @@
       <c r="A24" s="16">
         <v>73</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="B24" s="24" t="s">
         <v>134</v>
       </c>
       <c r="C24" s="13" t="s">
@@ -3616,20 +3619,20 @@
       <c r="E24" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F24" s="25">
+      <c r="F24" s="26">
         <v>3</v>
       </c>
       <c r="H24" s="16"/>
       <c r="I24" s="16"/>
       <c r="J24" s="16"/>
       <c r="K24" s="16"/>
-      <c r="L24" s="22" t="s">
+      <c r="L24" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="M24" s="22" t="s">
+      <c r="M24" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="P24" s="22" t="s">
+      <c r="P24" s="23" t="s">
         <v>113</v>
       </c>
       <c r="Q24" s="16">
@@ -3641,7 +3644,7 @@
       <c r="S24" s="16">
         <v>18</v>
       </c>
-      <c r="T24" s="21">
+      <c r="T24" s="22">
         <v>50</v>
       </c>
       <c r="U24" s="16">
@@ -3658,7 +3661,7 @@
       <c r="A25" s="16">
         <v>83</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="24" t="s">
         <v>134</v>
       </c>
       <c r="C25" s="13" t="s">
@@ -3670,20 +3673,20 @@
       <c r="E25" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F25" s="25">
+      <c r="F25" s="26">
         <v>3</v>
       </c>
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
       <c r="J25" s="16"/>
       <c r="K25" s="16"/>
-      <c r="L25" s="22" t="s">
+      <c r="L25" s="23" t="s">
         <v>147</v>
       </c>
-      <c r="M25" s="22" t="s">
+      <c r="M25" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="P25" s="22" t="s">
+      <c r="P25" s="23" t="s">
         <v>115</v>
       </c>
       <c r="Q25" s="16">
@@ -3695,7 +3698,7 @@
       <c r="S25" s="16">
         <v>18</v>
       </c>
-      <c r="T25" s="21">
+      <c r="T25" s="22">
         <v>60</v>
       </c>
       <c r="U25" s="16">
@@ -3714,8 +3717,8 @@
       <c r="J26" s="16"/>
       <c r="K26" s="16"/>
       <c r="L26" s="16"/>
-      <c r="M26" s="22"/>
-      <c r="P26" s="22" t="s">
+      <c r="M26" s="23"/>
+      <c r="P26" s="23" t="s">
         <v>120</v>
       </c>
       <c r="Q26" s="16">
@@ -3727,7 +3730,7 @@
       <c r="S26" s="16">
         <v>18</v>
       </c>
-      <c r="T26" s="21">
+      <c r="T26" s="22">
         <v>75</v>
       </c>
       <c r="U26" s="16">
@@ -3747,7 +3750,7 @@
       <c r="K27" s="16"/>
       <c r="L27" s="16"/>
       <c r="M27" s="16"/>
-      <c r="P27" s="22" t="s">
+      <c r="P27" s="23" t="s">
         <v>123</v>
       </c>
       <c r="Q27" s="16">
@@ -3759,7 +3762,7 @@
       <c r="S27" s="16">
         <v>20</v>
       </c>
-      <c r="T27" s="21">
+      <c r="T27" s="22">
         <v>100</v>
       </c>
       <c r="U27" s="16">
@@ -3773,7 +3776,7 @@
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A28" s="18" t="s">
+      <c r="A28" s="19" t="s">
         <v>19</v>
       </c>
       <c r="B28" s="16" t="s">
@@ -3785,7 +3788,7 @@
       <c r="K28" s="16"/>
       <c r="L28" s="16"/>
       <c r="M28" s="16"/>
-      <c r="P28" s="22" t="s">
+      <c r="P28" s="23" t="s">
         <v>129</v>
       </c>
       <c r="Q28" s="16">
@@ -3797,7 +3800,7 @@
       <c r="S28" s="16">
         <v>20</v>
       </c>
-      <c r="T28" s="21">
+      <c r="T28" s="22">
         <v>125</v>
       </c>
       <c r="U28" s="16">
@@ -3823,7 +3826,7 @@
       <c r="K29" s="16"/>
       <c r="L29" s="16"/>
       <c r="M29" s="16"/>
-      <c r="P29" s="22" t="s">
+      <c r="P29" s="23" t="s">
         <v>132</v>
       </c>
       <c r="Q29" s="16">
@@ -3835,7 +3838,7 @@
       <c r="S29" s="16">
         <v>22</v>
       </c>
-      <c r="T29" s="21">
+      <c r="T29" s="22">
         <v>150</v>
       </c>
       <c r="U29" s="16">
@@ -3861,7 +3864,7 @@
       <c r="K30" s="16"/>
       <c r="L30" s="16"/>
       <c r="M30" s="16"/>
-      <c r="P30" s="22" t="s">
+      <c r="P30" s="23" t="s">
         <v>138</v>
       </c>
       <c r="Q30" s="16">
@@ -3873,7 +3876,7 @@
       <c r="S30" s="16">
         <v>22</v>
       </c>
-      <c r="T30" s="21">
+      <c r="T30" s="22">
         <v>175</v>
       </c>
       <c r="U30" s="16">
@@ -3899,7 +3902,7 @@
       <c r="K31" s="16"/>
       <c r="L31" s="16"/>
       <c r="M31" s="16"/>
-      <c r="P31" s="22" t="s">
+      <c r="P31" s="23" t="s">
         <v>141</v>
       </c>
       <c r="Q31" s="16">
@@ -3911,7 +3914,7 @@
       <c r="S31" s="16">
         <v>25</v>
       </c>
-      <c r="T31" s="21">
+      <c r="T31" s="22">
         <v>200</v>
       </c>
       <c r="U31" s="16">
@@ -3931,7 +3934,7 @@
       <c r="K32" s="16"/>
       <c r="L32" s="16"/>
       <c r="M32" s="16"/>
-      <c r="P32" s="22" t="s">
+      <c r="P32" s="23" t="s">
         <v>144</v>
       </c>
       <c r="Q32" s="16">
@@ -3943,7 +3946,7 @@
       <c r="S32" s="16">
         <v>25</v>
       </c>
-      <c r="T32" s="21">
+      <c r="T32" s="22">
         <v>250</v>
       </c>
       <c r="U32" s="16">
@@ -3963,7 +3966,7 @@
       <c r="K33" s="16"/>
       <c r="L33" s="16"/>
       <c r="M33" s="16"/>
-      <c r="P33" s="22" t="s">
+      <c r="P33" s="23" t="s">
         <v>147</v>
       </c>
       <c r="Q33" s="16">
@@ -3975,7 +3978,7 @@
       <c r="S33" s="16">
         <v>25</v>
       </c>
-      <c r="T33" s="21">
+      <c r="T33" s="22">
         <v>300</v>
       </c>
       <c r="U33" s="16">
@@ -3989,7 +3992,7 @@
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A34" s="18" t="s">
+      <c r="A34" s="19" t="s">
         <v>23</v>
       </c>
       <c r="H34" s="16"/>
@@ -4001,7 +4004,7 @@
       <c r="O34" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="P34" s="20" t="s">
+      <c r="P34" s="21" t="s">
         <v>57</v>
       </c>
       <c r="Q34" s="16">
@@ -4013,7 +4016,7 @@
       <c r="S34" s="16">
         <v>5</v>
       </c>
-      <c r="T34" s="21">
+      <c r="T34" s="22">
         <v>0.5</v>
       </c>
       <c r="U34" s="16">
@@ -4036,7 +4039,7 @@
       <c r="K35" s="16"/>
       <c r="L35" s="16"/>
       <c r="M35" s="16"/>
-      <c r="P35" s="22" t="s">
+      <c r="P35" s="23" t="s">
         <v>65</v>
       </c>
       <c r="Q35" s="16">
@@ -4048,7 +4051,7 @@
       <c r="S35" s="16">
         <v>6</v>
       </c>
-      <c r="T35" s="21">
+      <c r="T35" s="22">
         <v>1</v>
       </c>
       <c r="U35" s="16">
@@ -4071,7 +4074,7 @@
       <c r="K36" s="16"/>
       <c r="L36" s="16"/>
       <c r="M36" s="16"/>
-      <c r="P36" s="22" t="s">
+      <c r="P36" s="23" t="s">
         <v>68</v>
       </c>
       <c r="Q36" s="16">
@@ -4083,7 +4086,7 @@
       <c r="S36" s="16">
         <v>8</v>
       </c>
-      <c r="T36" s="21">
+      <c r="T36" s="22">
         <v>1.5</v>
       </c>
       <c r="U36" s="16">
@@ -4100,13 +4103,13 @@
       <c r="A37" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="H37" s="28"/>
-      <c r="I37" s="28"/>
-      <c r="J37" s="28"/>
-      <c r="K37" s="28"/>
-      <c r="L37" s="28"/>
-      <c r="M37" s="28"/>
-      <c r="P37" s="22" t="s">
+      <c r="H37" s="29"/>
+      <c r="I37" s="29"/>
+      <c r="J37" s="29"/>
+      <c r="K37" s="29"/>
+      <c r="L37" s="29"/>
+      <c r="M37" s="29"/>
+      <c r="P37" s="23" t="s">
         <v>75</v>
       </c>
       <c r="Q37" s="16">
@@ -4118,7 +4121,7 @@
       <c r="S37" s="16">
         <v>8</v>
       </c>
-      <c r="T37" s="21">
+      <c r="T37" s="22">
         <v>2</v>
       </c>
       <c r="U37" s="16">
@@ -4138,7 +4141,7 @@
       <c r="K38" s="16"/>
       <c r="L38" s="16"/>
       <c r="M38" s="16"/>
-      <c r="P38" s="22" t="s">
+      <c r="P38" s="23" t="s">
         <v>79</v>
       </c>
       <c r="Q38" s="16">
@@ -4150,7 +4153,7 @@
       <c r="S38" s="16">
         <v>8</v>
       </c>
-      <c r="T38" s="21">
+      <c r="T38" s="22">
         <v>3</v>
       </c>
       <c r="U38" s="16">
@@ -4170,7 +4173,7 @@
       <c r="K39" s="16"/>
       <c r="L39" s="16"/>
       <c r="M39" s="16"/>
-      <c r="P39" s="22" t="s">
+      <c r="P39" s="23" t="s">
         <v>83</v>
       </c>
       <c r="Q39" s="16">
@@ -4182,7 +4185,7 @@
       <c r="S39" s="16">
         <v>8</v>
       </c>
-      <c r="T39" s="21">
+      <c r="T39" s="22">
         <v>5.5</v>
       </c>
       <c r="U39" s="16">
@@ -4196,22 +4199,22 @@
       </c>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A40" s="18" t="s">
+      <c r="A40" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="B40" s="18" t="s">
+      <c r="B40" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="C40" s="18" t="s">
+      <c r="C40" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="D40" s="18" t="s">
+      <c r="D40" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E40" s="18" t="s">
+      <c r="E40" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="F40" s="18" t="s">
+      <c r="F40" s="19" t="s">
         <v>163</v>
       </c>
       <c r="H40" s="16"/>
@@ -4220,7 +4223,7 @@
       <c r="K40" s="16"/>
       <c r="L40" s="16"/>
       <c r="M40" s="16"/>
-      <c r="P40" s="22" t="s">
+      <c r="P40" s="23" t="s">
         <v>86</v>
       </c>
       <c r="Q40" s="16">
@@ -4232,7 +4235,7 @@
       <c r="S40" s="16">
         <v>10</v>
       </c>
-      <c r="T40" s="21">
+      <c r="T40" s="22">
         <v>7.5</v>
       </c>
       <c r="U40" s="16">
@@ -4270,7 +4273,7 @@
       <c r="K41" s="16"/>
       <c r="L41" s="16"/>
       <c r="M41" s="16"/>
-      <c r="P41" s="22" t="s">
+      <c r="P41" s="23" t="s">
         <v>89</v>
       </c>
       <c r="Q41" s="16">
@@ -4282,7 +4285,7 @@
       <c r="S41" s="16">
         <v>10</v>
       </c>
-      <c r="T41" s="21">
+      <c r="T41" s="22">
         <v>10</v>
       </c>
       <c r="U41" s="16">
@@ -4320,7 +4323,7 @@
       <c r="K42" s="16"/>
       <c r="L42" s="16"/>
       <c r="M42" s="16"/>
-      <c r="P42" s="22" t="s">
+      <c r="P42" s="23" t="s">
         <v>91</v>
       </c>
       <c r="Q42" s="16">
@@ -4332,7 +4335,7 @@
       <c r="S42" s="16">
         <v>12</v>
       </c>
-      <c r="T42" s="21">
+      <c r="T42" s="22">
         <v>15</v>
       </c>
       <c r="U42" s="16">
@@ -4359,7 +4362,7 @@
       <c r="K43" s="16"/>
       <c r="L43" s="16"/>
       <c r="M43" s="16"/>
-      <c r="P43" s="22" t="s">
+      <c r="P43" s="23" t="s">
         <v>94</v>
       </c>
       <c r="Q43" s="16">
@@ -4371,7 +4374,7 @@
       <c r="S43" s="16">
         <v>12</v>
       </c>
-      <c r="T43" s="21">
+      <c r="T43" s="22">
         <v>20</v>
       </c>
       <c r="U43" s="16">
@@ -4395,7 +4398,7 @@
       <c r="K44" s="13"/>
       <c r="L44" s="13"/>
       <c r="M44" s="13"/>
-      <c r="P44" s="22" t="s">
+      <c r="P44" s="23" t="s">
         <v>100</v>
       </c>
       <c r="Q44" s="16">
@@ -4407,7 +4410,7 @@
       <c r="S44" s="16">
         <v>14</v>
       </c>
-      <c r="T44" s="21">
+      <c r="T44" s="22">
         <v>25</v>
       </c>
       <c r="U44" s="16">
@@ -4423,7 +4426,7 @@
     <row r="45" spans="4:23" x14ac:dyDescent="0.25">
       <c r="D45" s="16"/>
       <c r="F45" s="13"/>
-      <c r="P45" s="22" t="s">
+      <c r="P45" s="23" t="s">
         <v>102</v>
       </c>
       <c r="Q45" s="16">
@@ -4435,7 +4438,7 @@
       <c r="S45" s="16">
         <v>14</v>
       </c>
-      <c r="T45" s="21">
+      <c r="T45" s="22">
         <v>30</v>
       </c>
       <c r="U45" s="16">
@@ -4449,13 +4452,13 @@
       </c>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A46" s="28"/>
+      <c r="A46" s="29"/>
       <c r="B46" s="15"/>
       <c r="C46" s="16"/>
       <c r="D46" s="16"/>
       <c r="E46" s="16"/>
       <c r="F46" s="13"/>
-      <c r="P46" s="22" t="s">
+      <c r="P46" s="23" t="s">
         <v>108</v>
       </c>
       <c r="Q46" s="16">
@@ -4467,7 +4470,7 @@
       <c r="S46" s="16">
         <v>16</v>
       </c>
-      <c r="T46" s="21">
+      <c r="T46" s="22">
         <v>40</v>
       </c>
       <c r="U46" s="16">
@@ -4481,13 +4484,13 @@
       </c>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A47" s="29" t="s">
+      <c r="A47" s="30" t="s">
         <v>18</v>
       </c>
       <c r="B47" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="P47" s="22" t="s">
+      <c r="P47" s="23" t="s">
         <v>114</v>
       </c>
       <c r="Q47" s="16">
@@ -4499,7 +4502,7 @@
       <c r="S47" s="16">
         <v>16</v>
       </c>
-      <c r="T47" s="21">
+      <c r="T47" s="22">
         <v>50</v>
       </c>
       <c r="U47" s="16">
@@ -4513,13 +4516,13 @@
       </c>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A48" s="28" t="s">
+      <c r="A48" s="29" t="s">
         <v>169</v>
       </c>
       <c r="B48" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="P48" s="22" t="s">
+      <c r="P48" s="23" t="s">
         <v>116</v>
       </c>
       <c r="Q48" s="16">
@@ -4531,7 +4534,7 @@
       <c r="S48" s="16">
         <v>16</v>
       </c>
-      <c r="T48" s="21">
+      <c r="T48" s="22">
         <v>60</v>
       </c>
       <c r="U48" s="16">
@@ -4551,7 +4554,7 @@
       <c r="B49" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="P49" s="22" t="s">
+      <c r="P49" s="23" t="s">
         <v>121</v>
       </c>
       <c r="Q49" s="16">
@@ -4563,7 +4566,7 @@
       <c r="S49" s="16">
         <v>18</v>
       </c>
-      <c r="T49" s="21">
+      <c r="T49" s="22">
         <v>75</v>
       </c>
       <c r="U49" s="16">
@@ -4583,7 +4586,7 @@
       <c r="B50" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="P50" s="22" t="s">
+      <c r="P50" s="23" t="s">
         <v>124</v>
       </c>
       <c r="Q50" s="16">
@@ -4595,7 +4598,7 @@
       <c r="S50" s="16">
         <v>20</v>
       </c>
-      <c r="T50" s="21">
+      <c r="T50" s="22">
         <v>100</v>
       </c>
       <c r="U50" s="16">
@@ -4615,7 +4618,7 @@
       <c r="B51" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="P51" s="22" t="s">
+      <c r="P51" s="23" t="s">
         <v>130</v>
       </c>
       <c r="Q51" s="16">
@@ -4627,7 +4630,7 @@
       <c r="S51" s="16">
         <v>20</v>
       </c>
-      <c r="T51" s="21">
+      <c r="T51" s="22">
         <v>125</v>
       </c>
       <c r="U51" s="16">
@@ -4647,7 +4650,7 @@
       <c r="B52" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="P52" s="22" t="s">
+      <c r="P52" s="23" t="s">
         <v>133</v>
       </c>
       <c r="Q52" s="16">
@@ -4659,7 +4662,7 @@
       <c r="S52" s="16">
         <v>22</v>
       </c>
-      <c r="T52" s="21">
+      <c r="T52" s="22">
         <v>150</v>
       </c>
       <c r="U52" s="16">
@@ -4679,7 +4682,7 @@
       <c r="B53" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="P53" s="22" t="s">
+      <c r="P53" s="23" t="s">
         <v>139</v>
       </c>
       <c r="Q53" s="16">
@@ -4691,7 +4694,7 @@
       <c r="S53" s="16">
         <v>22</v>
       </c>
-      <c r="T53" s="21">
+      <c r="T53" s="22">
         <v>180</v>
       </c>
       <c r="U53" s="16">
@@ -4708,7 +4711,7 @@
       <c r="A54" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="P54" s="22" t="s">
+      <c r="P54" s="23" t="s">
         <v>142</v>
       </c>
       <c r="Q54" s="16">
@@ -4720,7 +4723,7 @@
       <c r="S54" s="16">
         <v>22</v>
       </c>
-      <c r="T54" s="21">
+      <c r="T54" s="22">
         <v>200</v>
       </c>
       <c r="U54" s="16">
@@ -4737,7 +4740,7 @@
       <c r="A55" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="P55" s="22" t="s">
+      <c r="P55" s="23" t="s">
         <v>145</v>
       </c>
       <c r="Q55" s="16">
@@ -4749,7 +4752,7 @@
       <c r="S55" s="16">
         <v>22</v>
       </c>
-      <c r="T55" s="21">
+      <c r="T55" s="22">
         <v>270</v>
       </c>
       <c r="U55" s="16">
@@ -4766,7 +4769,7 @@
       <c r="A56" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="P56" s="22" t="s">
+      <c r="P56" s="23" t="s">
         <v>148</v>
       </c>
       <c r="Q56" s="16">
@@ -4778,7 +4781,7 @@
       <c r="S56" s="16">
         <v>25</v>
       </c>
-      <c r="T56" s="21">
+      <c r="T56" s="22">
         <v>340</v>
       </c>
       <c r="U56" s="16">
@@ -4792,7 +4795,7 @@
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" s="18" t="s">
+      <c r="A59" s="19" t="s">
         <v>22</v>
       </c>
     </row>
@@ -4812,131 +4815,131 @@
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A63" s="30"/>
-      <c r="B63" s="30"/>
-      <c r="C63" s="31"/>
-      <c r="D63" s="31"/>
-      <c r="E63" s="31"/>
-      <c r="F63" s="32"/>
-      <c r="G63" s="32"/>
-      <c r="H63" s="32"/>
-      <c r="I63" s="32"/>
-      <c r="J63" s="32"/>
-      <c r="K63" s="32"/>
-      <c r="L63" s="32"/>
-      <c r="M63" s="32"/>
-      <c r="N63" s="32"/>
-      <c r="O63" s="32"/>
-      <c r="P63" s="32"/>
-      <c r="Q63" s="32"/>
-      <c r="R63" s="32"/>
-      <c r="S63" s="32"/>
-      <c r="T63" s="33"/>
-      <c r="U63" s="33"/>
-      <c r="V63" s="32"/>
-      <c r="W63" s="33"/>
-      <c r="X63" s="32"/>
+      <c r="A63" s="31"/>
+      <c r="B63" s="31"/>
+      <c r="C63" s="32"/>
+      <c r="D63" s="32"/>
+      <c r="E63" s="32"/>
+      <c r="F63" s="33"/>
+      <c r="G63" s="33"/>
+      <c r="H63" s="33"/>
+      <c r="I63" s="33"/>
+      <c r="J63" s="33"/>
+      <c r="K63" s="33"/>
+      <c r="L63" s="33"/>
+      <c r="M63" s="33"/>
+      <c r="N63" s="33"/>
+      <c r="O63" s="33"/>
+      <c r="P63" s="33"/>
+      <c r="Q63" s="33"/>
+      <c r="R63" s="33"/>
+      <c r="S63" s="33"/>
+      <c r="T63" s="34"/>
+      <c r="U63" s="34"/>
+      <c r="V63" s="33"/>
+      <c r="W63" s="34"/>
+      <c r="X63" s="33"/>
     </row>
     <row r="64" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="34" t="s">
+      <c r="A64" s="35" t="s">
         <v>187</v>
       </c>
-      <c r="B64" s="35"/>
+      <c r="B64" s="36"/>
       <c r="C64" s="13" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="36" t="s">
-        <v>3</v>
-      </c>
-      <c r="B65" s="37">
+      <c r="A65" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B65" s="38">
         <v>46168</v>
       </c>
-      <c r="C65" s="38" t="s">
+      <c r="C65" s="39" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="39" t="s">
+      <c r="A66" s="40" t="s">
         <v>190</v>
       </c>
-      <c r="B66" s="40" t="s">
+      <c r="B66" s="41" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="39" t="s">
+      <c r="A67" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="B67" s="41" t="s">
+      <c r="B67" s="42" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="39" t="s">
+      <c r="A68" s="40" t="s">
         <v>149</v>
       </c>
-      <c r="B68" s="41" t="s">
+      <c r="B68" s="42" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="39" t="s">
+      <c r="A69" s="40" t="s">
         <v>192</v>
       </c>
-      <c r="B69" s="42">
+      <c r="B69" s="43">
         <v>46179</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="39" t="s">
+      <c r="A70" s="40" t="s">
         <v>193</v>
       </c>
-      <c r="B70" s="41">
+      <c r="B70" s="42">
         <v>2</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="39" t="s">
+      <c r="A71" s="40" t="s">
         <v>194</v>
       </c>
-      <c r="B71" s="41" t="s">
+      <c r="B71" s="42" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="39" t="s">
+      <c r="A72" s="40" t="s">
         <v>196</v>
       </c>
-      <c r="B72" s="41">
+      <c r="B72" s="42">
         <v>14</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="43" t="s">
+      <c r="A73" s="44" t="s">
         <v>197</v>
       </c>
-      <c r="B73" s="44">
+      <c r="B73" s="45">
         <v>10</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="75" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="45" t="s">
+      <c r="A75" s="46" t="s">
         <v>198</v>
       </c>
-      <c r="B75" s="46"/>
-      <c r="C75" s="30" t="s">
+      <c r="B75" s="47"/>
+      <c r="C75" s="31" t="s">
         <v>199</v>
       </c>
-      <c r="D75" s="33"/>
+      <c r="D75" s="34"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="36" t="s">
+      <c r="A76" s="37" t="s">
         <v>200</v>
       </c>
-      <c r="B76" s="47" t="str">
+      <c r="B76" s="48" t="str">
         <f>VLOOKUP(B67,B67,1)</f>
         <v>CEB</v>
       </c>
@@ -4949,13 +4952,13 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="48" t="s">
+      <c r="A77" s="49" t="s">
         <v>51</v>
       </c>
-      <c r="B77" s="49">
+      <c r="B77" s="50">
         <v>44.5</v>
       </c>
-      <c r="C77" s="28" t="s">
+      <c r="C77" s="29" t="s">
         <v>31</v>
       </c>
       <c r="D77" s="16" t="str">
@@ -4964,13 +4967,13 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="48" t="s">
+      <c r="A78" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="B78" s="41" t="s">
+      <c r="B78" s="42" t="s">
         <v>169</v>
       </c>
-      <c r="C78" s="28" t="s">
+      <c r="C78" s="29" t="s">
         <v>33</v>
       </c>
       <c r="D78" s="16" t="str">
@@ -4979,13 +4982,13 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="48" t="s">
+      <c r="A79" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="B79" s="41" t="s">
+      <c r="B79" s="42" t="s">
         <v>184</v>
       </c>
-      <c r="C79" s="28" t="s">
+      <c r="C79" s="29" t="s">
         <v>30</v>
       </c>
       <c r="D79" s="16" t="str">
@@ -4994,13 +4997,13 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="48" t="s">
+      <c r="A80" s="49" t="s">
         <v>202</v>
       </c>
-      <c r="B80" s="41" t="s">
+      <c r="B80" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="C80" s="28" t="s">
+      <c r="C80" s="29" t="s">
         <v>31</v>
       </c>
       <c r="D80" s="16" t="str">
@@ -5009,13 +5012,13 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="48" t="s">
+      <c r="A81" s="49" t="s">
         <v>203</v>
       </c>
-      <c r="B81" s="41" t="s">
+      <c r="B81" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="C81" s="28" t="s">
+      <c r="C81" s="29" t="s">
         <v>204</v>
       </c>
       <c r="D81" s="16">
@@ -5024,28 +5027,28 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="39" t="s">
+      <c r="A82" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="B82" s="41" t="s">
+      <c r="B82" s="42" t="s">
         <v>205</v>
       </c>
       <c r="D82" s="16"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="39" t="s">
+      <c r="A83" s="40" t="s">
         <v>206</v>
       </c>
-      <c r="B83" s="41" t="s">
+      <c r="B83" s="42" t="s">
         <v>207</v>
       </c>
       <c r="D83" s="16"/>
     </row>
     <row r="84" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="43" t="s">
+      <c r="A84" s="44" t="s">
         <v>208</v>
       </c>
-      <c r="B84" s="44">
+      <c r="B84" s="45">
         <v>595</v>
       </c>
       <c r="D84" s="16"/>
@@ -5054,38 +5057,38 @@
       <c r="D85" s="16"/>
     </row>
     <row r="86" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="45" t="s">
+      <c r="A86" s="46" t="s">
         <v>209</v>
       </c>
-      <c r="B86" s="46"/>
-      <c r="C86" s="30" t="s">
+      <c r="B86" s="47"/>
+      <c r="C86" s="31" t="s">
         <v>210</v>
       </c>
-      <c r="D86" s="33"/>
+      <c r="D86" s="34"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="50" t="s">
+      <c r="A87" s="51" t="s">
         <v>211</v>
       </c>
-      <c r="B87" s="51" t="s">
+      <c r="B87" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="C87" s="28" t="s">
+      <c r="C87" s="29" t="s">
         <v>212</v>
       </c>
-      <c r="D87" s="52">
+      <c r="D87" s="53">
         <f>VLOOKUP(TRIM(B89),P3:W56,5,FALSE)</f>
         <v>15</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="48" t="s">
+      <c r="A88" s="49" t="s">
         <v>213</v>
       </c>
-      <c r="B88" s="41" t="s">
+      <c r="B88" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="C88" s="28" t="s">
+      <c r="C88" s="29" t="s">
         <v>214</v>
       </c>
       <c r="D88" s="16">
@@ -5094,25 +5097,25 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="48" t="s">
+      <c r="A89" s="49" t="s">
         <v>212</v>
       </c>
-      <c r="B89" s="41" t="s">
+      <c r="B89" s="42" t="s">
         <v>91</v>
       </c>
       <c r="C89" s="16" t="s">
         <v>215</v>
       </c>
-      <c r="D89" s="53">
+      <c r="D89" s="54">
         <f>VLOOKUP(TRIM(B89),P3:W56,2,FALSE)</f>
         <v>1728</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="48" t="s">
+      <c r="A90" s="49" t="s">
         <v>160</v>
       </c>
-      <c r="B90" s="41">
+      <c r="B90" s="42">
         <v>220</v>
       </c>
       <c r="C90" s="16" t="s">
@@ -5124,10 +5127,10 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="39" t="s">
+      <c r="A91" s="40" t="s">
         <v>161</v>
       </c>
-      <c r="B91" s="41">
+      <c r="B91" s="42">
         <v>60</v>
       </c>
       <c r="C91" s="16" t="s">
@@ -5139,10 +5142,10 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="39" t="s">
+      <c r="A92" s="40" t="s">
         <v>162</v>
       </c>
-      <c r="B92" s="41" t="s">
+      <c r="B92" s="42" t="s">
         <v>164</v>
       </c>
       <c r="C92" s="16" t="s">
@@ -5154,13 +5157,13 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="39" t="s">
+      <c r="A93" s="40" t="s">
         <v>163</v>
       </c>
-      <c r="B93" s="41" t="s">
+      <c r="B93" s="42" t="s">
         <v>165</v>
       </c>
-      <c r="C93" s="28" t="s">
+      <c r="C93" s="29" t="s">
         <v>28</v>
       </c>
       <c r="D93" s="16" t="str">
@@ -5169,14 +5172,14 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="39" t="s">
+      <c r="A94" s="40" t="s">
         <v>215</v>
       </c>
-      <c r="B94" s="54">
+      <c r="B94" s="55">
         <f>VLOOKUP(D89,D89,1)</f>
         <v>1728</v>
       </c>
-      <c r="C94" s="28" t="s">
+      <c r="C94" s="29" t="s">
         <v>218</v>
       </c>
       <c r="D94" s="16">
@@ -5185,10 +5188,10 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="39" t="s">
+      <c r="A95" s="40" t="s">
         <v>208</v>
       </c>
-      <c r="B95" s="54">
+      <c r="B95" s="55">
         <f>VLOOKUP(B84,B84,1)</f>
         <v>595</v>
       </c>
@@ -5201,26 +5204,26 @@
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96" s="39" t="s">
+      <c r="A96" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="B96" s="55">
+      <c r="B96" s="56">
         <v>4.5</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" s="39" t="s">
+      <c r="A97" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="B97" s="55">
+      <c r="B97" s="56">
         <v>13</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" s="43" t="s">
+      <c r="A98" s="44" t="s">
         <v>201</v>
       </c>
-      <c r="B98" s="56">
+      <c r="B98" s="57">
         <f>VLOOKUP(D76,D76,1)</f>
         <v>598.1538461538462</v>
       </c>

</xml_diff>

<commit_message>
JO: revert template to previous (centered) layout
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HNv2pt2j3pqxEC7sBHUC3k
</commit_message>
<xml_diff>
--- a/public/templates/fans-jo-template.xlsx
+++ b/public/templates/fans-jo-template.xlsx
@@ -856,7 +856,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -865,7 +865,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -893,13 +893,10 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="12" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2101,12 +2098,12 @@
       <c r="N50" s="3"/>
       <c r="O50" s="3"/>
       <c r="P50" s="3"/>
-      <c r="Q50" s="3"/>
-      <c r="R50" s="3"/>
-      <c r="S50" s="3"/>
-      <c r="T50" s="3"/>
-      <c r="U50" s="3"/>
-      <c r="V50" s="3"/>
+      <c r="Q50" s="16"/>
+      <c r="R50" s="16"/>
+      <c r="S50" s="16"/>
+      <c r="T50" s="16"/>
+      <c r="U50" s="16"/>
+      <c r="V50" s="16"/>
       <c r="W50" s="16"/>
       <c r="X50" s="13"/>
     </row>
@@ -2145,28 +2142,28 @@
       <c r="B52" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C52" s="17">
+      <c r="D52" s="3" t="str">
         <f>Source!D80</f>
-      </c>
-      <c r="D52" s="17"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
-      <c r="G52" s="17"/>
-      <c r="H52" s="17"/>
-      <c r="I52" s="17"/>
-      <c r="J52" s="17"/>
-      <c r="K52" s="17"/>
-      <c r="L52" s="17"/>
-      <c r="M52" s="17"/>
-      <c r="N52" s="17"/>
-      <c r="O52" s="17"/>
-      <c r="P52" s="17"/>
-      <c r="Q52" s="17"/>
-      <c r="R52" s="17"/>
-      <c r="S52" s="17"/>
-      <c r="T52" s="17"/>
-      <c r="U52" s="17"/>
-      <c r="V52" s="17"/>
+        <v>2 1/4”Ø x 1/2" keyway</v>
+      </c>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="5"/>
+      <c r="L52" s="5"/>
+      <c r="M52" s="5"/>
+      <c r="N52" s="13"/>
+      <c r="O52" s="13"/>
+      <c r="P52" s="13"/>
+      <c r="Q52" s="13"/>
+      <c r="R52" s="13"/>
+      <c r="S52" s="13"/>
+      <c r="T52" s="13"/>
+      <c r="U52" s="13"/>
+      <c r="V52" s="13"/>
       <c r="W52" s="13"/>
       <c r="X52" s="13"/>
     </row>
@@ -2317,13 +2314,13 @@
       <c r="X57" s="13"/>
     </row>
     <row r="58" spans="19:23" x14ac:dyDescent="0.25">
-      <c r="S58" s="18" t="s">
+      <c r="S58" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="T58" s="18"/>
-      <c r="U58" s="18"/>
-      <c r="V58" s="18"/>
-      <c r="W58" s="18"/>
+      <c r="T58" s="17"/>
+      <c r="U58" s="17"/>
+      <c r="V58" s="17"/>
+      <c r="W58" s="17"/>
     </row>
     <row r="59" spans="23:23" x14ac:dyDescent="0.25">
       <c r="W59" s="7"/>
@@ -2350,8 +2347,8 @@
     <mergeCell ref="C44:V44"/>
     <mergeCell ref="C46:V46"/>
     <mergeCell ref="C48:V48"/>
-    <mergeCell ref="C50:V50"/>
-    <mergeCell ref="C52:V52"/>
+    <mergeCell ref="C50:P50"/>
+    <mergeCell ref="D52:M52"/>
     <mergeCell ref="C54:I54"/>
     <mergeCell ref="C56:V56"/>
     <mergeCell ref="S58:W58"/>
@@ -2387,13 +2384,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
       <c r="H2" s="6" t="s">
         <v>36</v>
       </c>
@@ -2468,16 +2465,16 @@
       <c r="J3" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="K3" s="21" t="s">
+      <c r="K3" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="L3" s="21" t="s">
+      <c r="L3" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="M3" s="21" t="s">
+      <c r="M3" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="P3" s="21" t="s">
+      <c r="P3" s="20" t="s">
         <v>55</v>
       </c>
       <c r="Q3" s="16">
@@ -2489,7 +2486,7 @@
       <c r="S3" s="16">
         <v>5</v>
       </c>
-      <c r="T3" s="22">
+      <c r="T3" s="21">
         <v>0.25</v>
       </c>
       <c r="U3" s="16">
@@ -2528,16 +2525,16 @@
         <v>40</v>
       </c>
       <c r="J4" s="16"/>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="L4" s="23" t="s">
+      <c r="L4" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="M4" s="23" t="s">
+      <c r="M4" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="P4" s="23" t="s">
+      <c r="P4" s="22" t="s">
         <v>63</v>
       </c>
       <c r="Q4" s="16">
@@ -2549,7 +2546,7 @@
       <c r="S4" s="16">
         <v>6</v>
       </c>
-      <c r="T4" s="22">
+      <c r="T4" s="21">
         <v>0.5</v>
       </c>
       <c r="U4" s="16">
@@ -2584,16 +2581,16 @@
       <c r="H5" s="16"/>
       <c r="I5" s="16"/>
       <c r="J5" s="16"/>
-      <c r="K5" s="23" t="s">
+      <c r="K5" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="L5" s="23" t="s">
+      <c r="L5" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="M5" s="23" t="s">
+      <c r="M5" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="P5" s="23" t="s">
+      <c r="P5" s="22" t="s">
         <v>66</v>
       </c>
       <c r="Q5" s="16">
@@ -2605,7 +2602,7 @@
       <c r="S5" s="16">
         <v>6</v>
       </c>
-      <c r="T5" s="22">
+      <c r="T5" s="21">
         <v>0.75</v>
       </c>
       <c r="U5" s="16">
@@ -2622,10 +2619,10 @@
       <c r="A6" s="16">
         <v>12.25</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="24" t="s">
         <v>70</v>
       </c>
       <c r="D6" s="13" t="s">
@@ -2634,22 +2631,22 @@
       <c r="E6" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="25">
         <v>1.25</v>
       </c>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
       <c r="J6" s="16"/>
-      <c r="K6" s="23" t="s">
+      <c r="K6" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="L6" s="23" t="s">
+      <c r="L6" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="M6" s="23" t="s">
+      <c r="M6" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="P6" s="23" t="s">
+      <c r="P6" s="22" t="s">
         <v>73</v>
       </c>
       <c r="Q6" s="16">
@@ -2661,7 +2658,7 @@
       <c r="S6" s="16">
         <v>8</v>
       </c>
-      <c r="T6" s="27">
+      <c r="T6" s="26">
         <v>1</v>
       </c>
       <c r="U6" s="16">
@@ -2678,10 +2675,10 @@
       <c r="A7" s="16">
         <v>13.5</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="24" t="s">
         <v>70</v>
       </c>
       <c r="D7" s="13" t="s">
@@ -2690,22 +2687,22 @@
       <c r="E7" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="25">
         <v>1.25</v>
       </c>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
       <c r="J7" s="16"/>
-      <c r="K7" s="23" t="s">
+      <c r="K7" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="L7" s="23" t="s">
+      <c r="L7" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="M7" s="23" t="s">
+      <c r="M7" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="P7" s="23" t="s">
+      <c r="P7" s="22" t="s">
         <v>77</v>
       </c>
       <c r="Q7" s="16">
@@ -2717,7 +2714,7 @@
       <c r="S7" s="16">
         <v>8</v>
       </c>
-      <c r="T7" s="22">
+      <c r="T7" s="21">
         <v>1.5</v>
       </c>
       <c r="U7" s="16">
@@ -2734,10 +2731,10 @@
       <c r="A8" s="16">
         <v>15</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="24" t="s">
         <v>70</v>
       </c>
       <c r="D8" s="13" t="s">
@@ -2746,22 +2743,22 @@
       <c r="E8" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="25">
         <v>1.25</v>
       </c>
       <c r="H8" s="16"/>
       <c r="I8" s="16"/>
       <c r="J8" s="16"/>
-      <c r="K8" s="23" t="s">
+      <c r="K8" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="L8" s="23" t="s">
+      <c r="L8" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="M8" s="23" t="s">
+      <c r="M8" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="P8" s="23" t="s">
+      <c r="P8" s="22" t="s">
         <v>81</v>
       </c>
       <c r="Q8" s="16">
@@ -2773,7 +2770,7 @@
       <c r="S8" s="16">
         <v>8</v>
       </c>
-      <c r="T8" s="22">
+      <c r="T8" s="21">
         <v>2</v>
       </c>
       <c r="U8" s="16">
@@ -2790,10 +2787,10 @@
       <c r="A9" s="16">
         <v>16.5</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="24" t="s">
         <v>70</v>
       </c>
       <c r="D9" s="13" t="s">
@@ -2802,22 +2799,22 @@
       <c r="E9" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="25">
         <v>1.25</v>
       </c>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
       <c r="J9" s="16"/>
-      <c r="K9" s="23" t="s">
+      <c r="K9" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="L9" s="23" t="s">
+      <c r="L9" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="M9" s="23" t="s">
+      <c r="M9" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="P9" s="23" t="s">
+      <c r="P9" s="22" t="s">
         <v>84</v>
       </c>
       <c r="Q9" s="16">
@@ -2829,7 +2826,7 @@
       <c r="S9" s="16">
         <v>8</v>
       </c>
-      <c r="T9" s="22">
+      <c r="T9" s="21">
         <v>3</v>
       </c>
       <c r="U9" s="16">
@@ -2846,10 +2843,10 @@
       <c r="A10" s="16">
         <v>18.25</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="24" t="s">
         <v>70</v>
       </c>
       <c r="D10" s="13" t="s">
@@ -2858,22 +2855,22 @@
       <c r="E10" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="25">
         <v>1.25</v>
       </c>
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
       <c r="J10" s="16"/>
-      <c r="K10" s="23" t="s">
+      <c r="K10" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="L10" s="23" t="s">
+      <c r="L10" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="M10" s="23" t="s">
+      <c r="M10" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="P10" s="23" t="s">
+      <c r="P10" s="22" t="s">
         <v>87</v>
       </c>
       <c r="Q10" s="16">
@@ -2885,7 +2882,7 @@
       <c r="S10" s="16">
         <v>8</v>
       </c>
-      <c r="T10" s="22">
+      <c r="T10" s="21">
         <v>5</v>
       </c>
       <c r="U10" s="16">
@@ -2902,10 +2899,10 @@
       <c r="A11" s="16">
         <v>20</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="24" t="s">
         <v>70</v>
       </c>
       <c r="D11" s="13" t="s">
@@ -2914,23 +2911,23 @@
       <c r="E11" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="25">
         <v>1.25</v>
       </c>
       <c r="H11" s="16"/>
       <c r="I11" s="16"/>
       <c r="J11" s="16"/>
       <c r="K11" s="16"/>
-      <c r="L11" s="23" t="s">
+      <c r="L11" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="M11" s="23" t="s">
+      <c r="M11" s="22" t="s">
         <v>91</v>
       </c>
       <c r="O11" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="P11" s="21" t="s">
+      <c r="P11" s="20" t="s">
         <v>56</v>
       </c>
       <c r="Q11" s="16">
@@ -2942,7 +2939,7 @@
       <c r="S11" s="16">
         <v>5</v>
       </c>
-      <c r="T11" s="22">
+      <c r="T11" s="21">
         <v>0.5</v>
       </c>
       <c r="U11" s="16">
@@ -2959,10 +2956,10 @@
       <c r="A12" s="16">
         <v>22.25</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="24" t="s">
         <v>70</v>
       </c>
       <c r="D12" s="13" t="s">
@@ -2971,20 +2968,20 @@
       <c r="E12" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="25">
         <v>1.25</v>
       </c>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
       <c r="J12" s="16"/>
       <c r="K12" s="16"/>
-      <c r="L12" s="23" t="s">
+      <c r="L12" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="M12" s="23" t="s">
+      <c r="M12" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="P12" s="23" t="s">
+      <c r="P12" s="22" t="s">
         <v>64</v>
       </c>
       <c r="Q12" s="16">
@@ -2996,7 +2993,7 @@
       <c r="S12" s="16">
         <v>6</v>
       </c>
-      <c r="T12" s="22">
+      <c r="T12" s="21">
         <v>1</v>
       </c>
       <c r="U12" s="16">
@@ -3013,7 +3010,7 @@
       <c r="A13" s="16">
         <v>24.5</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="23" t="s">
         <v>95</v>
       </c>
       <c r="C13" s="13" t="s">
@@ -3025,20 +3022,20 @@
       <c r="E13" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="F13" s="26">
+      <c r="F13" s="25">
         <v>1.5</v>
       </c>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
       <c r="J13" s="16"/>
       <c r="K13" s="16"/>
-      <c r="L13" s="23" t="s">
+      <c r="L13" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="M13" s="23" t="s">
+      <c r="M13" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="P13" s="23" t="s">
+      <c r="P13" s="22" t="s">
         <v>67</v>
       </c>
       <c r="Q13" s="16">
@@ -3050,7 +3047,7 @@
       <c r="S13" s="16">
         <v>8</v>
       </c>
-      <c r="T13" s="22">
+      <c r="T13" s="21">
         <v>1.5</v>
       </c>
       <c r="U13" s="16">
@@ -3067,7 +3064,7 @@
       <c r="A14" s="16">
         <v>27</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="23" t="s">
         <v>95</v>
       </c>
       <c r="C14" s="13" t="s">
@@ -3079,20 +3076,20 @@
       <c r="E14" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="25">
         <v>1.5</v>
       </c>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
       <c r="J14" s="16"/>
       <c r="K14" s="16"/>
-      <c r="L14" s="23" t="s">
+      <c r="L14" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="M14" s="23" t="s">
+      <c r="M14" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="P14" s="23" t="s">
+      <c r="P14" s="22" t="s">
         <v>74</v>
       </c>
       <c r="Q14" s="16">
@@ -3104,7 +3101,7 @@
       <c r="S14" s="16">
         <v>8</v>
       </c>
-      <c r="T14" s="22">
+      <c r="T14" s="21">
         <v>2</v>
       </c>
       <c r="U14" s="16">
@@ -3121,7 +3118,7 @@
       <c r="A15" s="16">
         <v>30</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="23" t="s">
         <v>103</v>
       </c>
       <c r="C15" s="13" t="s">
@@ -3133,20 +3130,20 @@
       <c r="E15" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="F15" s="26">
+      <c r="F15" s="25">
         <v>1.75</v>
       </c>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
       <c r="J15" s="16"/>
       <c r="K15" s="16"/>
-      <c r="L15" s="23" t="s">
+      <c r="L15" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="M15" s="23" t="s">
+      <c r="M15" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="P15" s="23" t="s">
+      <c r="P15" s="22" t="s">
         <v>78</v>
       </c>
       <c r="Q15" s="16">
@@ -3158,7 +3155,7 @@
       <c r="S15" s="16">
         <v>8</v>
       </c>
-      <c r="T15" s="22">
+      <c r="T15" s="21">
         <v>3</v>
       </c>
       <c r="U15" s="16">
@@ -3175,7 +3172,7 @@
       <c r="A16" s="16">
         <v>33</v>
       </c>
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C16" s="13" t="s">
@@ -3187,20 +3184,20 @@
       <c r="E16" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="F16" s="26">
+      <c r="F16" s="25">
         <v>2</v>
       </c>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
       <c r="J16" s="16"/>
       <c r="K16" s="16"/>
-      <c r="L16" s="23" t="s">
+      <c r="L16" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="M16" s="23" t="s">
+      <c r="M16" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="P16" s="23" t="s">
+      <c r="P16" s="22" t="s">
         <v>82</v>
       </c>
       <c r="Q16" s="16">
@@ -3212,7 +3209,7 @@
       <c r="S16" s="16">
         <v>8</v>
       </c>
-      <c r="T16" s="22">
+      <c r="T16" s="21">
         <v>5</v>
       </c>
       <c r="U16" s="16">
@@ -3229,7 +3226,7 @@
       <c r="A17" s="16">
         <v>36.5</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C17" s="13" t="s">
@@ -3241,20 +3238,20 @@
       <c r="E17" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="F17" s="26">
+      <c r="F17" s="25">
         <v>2</v>
       </c>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
       <c r="J17" s="16"/>
       <c r="K17" s="16"/>
-      <c r="L17" s="23" t="s">
+      <c r="L17" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="M17" s="23" t="s">
+      <c r="M17" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="P17" s="23" t="s">
+      <c r="P17" s="22" t="s">
         <v>85</v>
       </c>
       <c r="Q17" s="16">
@@ -3266,7 +3263,7 @@
       <c r="S17" s="16">
         <v>10</v>
       </c>
-      <c r="T17" s="22">
+      <c r="T17" s="21">
         <v>7.5</v>
       </c>
       <c r="U17" s="16">
@@ -3283,32 +3280,32 @@
       <c r="A18" s="16">
         <v>40.25</v>
       </c>
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="23" t="s">
         <v>117</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="27" t="s">
         <v>117</v>
       </c>
       <c r="E18" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="F18" s="26">
+      <c r="F18" s="25">
         <v>2.25</v>
       </c>
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
       <c r="J18" s="16"/>
       <c r="K18" s="16"/>
-      <c r="L18" s="23" t="s">
+      <c r="L18" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="M18" s="23" t="s">
+      <c r="M18" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="P18" s="23" t="s">
+      <c r="P18" s="22" t="s">
         <v>88</v>
       </c>
       <c r="Q18" s="16">
@@ -3320,7 +3317,7 @@
       <c r="S18" s="16">
         <v>10</v>
       </c>
-      <c r="T18" s="22">
+      <c r="T18" s="21">
         <v>10</v>
       </c>
       <c r="U18" s="16">
@@ -3337,32 +3334,32 @@
       <c r="A19" s="16">
         <v>44.5</v>
       </c>
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="23" t="s">
         <v>117</v>
       </c>
       <c r="C19" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="D19" s="28" t="s">
+      <c r="D19" s="27" t="s">
         <v>117</v>
       </c>
       <c r="E19" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="F19" s="26">
+      <c r="F19" s="25">
         <v>2.25</v>
       </c>
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="16"/>
       <c r="K19" s="16"/>
-      <c r="L19" s="23" t="s">
+      <c r="L19" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="M19" s="23" t="s">
+      <c r="M19" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="P19" s="23" t="s">
+      <c r="P19" s="22" t="s">
         <v>90</v>
       </c>
       <c r="Q19" s="16">
@@ -3374,7 +3371,7 @@
       <c r="S19" s="16">
         <v>12</v>
       </c>
-      <c r="T19" s="22">
+      <c r="T19" s="21">
         <v>15</v>
       </c>
       <c r="U19" s="16">
@@ -3391,7 +3388,7 @@
       <c r="A20" s="16">
         <v>49</v>
       </c>
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="23" t="s">
         <v>125</v>
       </c>
       <c r="C20" s="13" t="s">
@@ -3403,20 +3400,20 @@
       <c r="E20" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F20" s="26">
+      <c r="F20" s="25">
         <v>2.5</v>
       </c>
       <c r="H20" s="16"/>
       <c r="I20" s="16"/>
       <c r="J20" s="16"/>
       <c r="K20" s="16"/>
-      <c r="L20" s="23" t="s">
+      <c r="L20" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="M20" s="23" t="s">
+      <c r="M20" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="P20" s="23" t="s">
+      <c r="P20" s="22" t="s">
         <v>93</v>
       </c>
       <c r="Q20" s="16">
@@ -3428,7 +3425,7 @@
       <c r="S20" s="16">
         <v>12</v>
       </c>
-      <c r="T20" s="22">
+      <c r="T20" s="21">
         <v>20</v>
       </c>
       <c r="U20" s="16">
@@ -3445,7 +3442,7 @@
       <c r="A21" s="16">
         <v>54.5</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="23" t="s">
         <v>125</v>
       </c>
       <c r="C21" s="13" t="s">
@@ -3457,20 +3454,20 @@
       <c r="E21" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F21" s="26">
+      <c r="F21" s="25">
         <v>2.5</v>
       </c>
       <c r="H21" s="16"/>
       <c r="I21" s="16"/>
       <c r="J21" s="16"/>
       <c r="K21" s="16"/>
-      <c r="L21" s="23" t="s">
+      <c r="L21" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="M21" s="23" t="s">
+      <c r="M21" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="P21" s="23" t="s">
+      <c r="P21" s="22" t="s">
         <v>99</v>
       </c>
       <c r="Q21" s="16">
@@ -3482,7 +3479,7 @@
       <c r="S21" s="16">
         <v>14</v>
       </c>
-      <c r="T21" s="22">
+      <c r="T21" s="21">
         <v>25</v>
       </c>
       <c r="U21" s="16">
@@ -3499,7 +3496,7 @@
       <c r="A22" s="16">
         <v>60</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="23" t="s">
         <v>134</v>
       </c>
       <c r="C22" s="13" t="s">
@@ -3511,20 +3508,20 @@
       <c r="E22" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F22" s="26">
+      <c r="F22" s="25">
         <v>3</v>
       </c>
       <c r="H22" s="16"/>
       <c r="I22" s="16"/>
       <c r="J22" s="16"/>
       <c r="K22" s="16"/>
-      <c r="L22" s="23" t="s">
+      <c r="L22" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="M22" s="23" t="s">
+      <c r="M22" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="P22" s="23" t="s">
+      <c r="P22" s="22" t="s">
         <v>101</v>
       </c>
       <c r="Q22" s="16">
@@ -3536,7 +3533,7 @@
       <c r="S22" s="16">
         <v>14</v>
       </c>
-      <c r="T22" s="22">
+      <c r="T22" s="21">
         <v>30</v>
       </c>
       <c r="U22" s="16">
@@ -3553,7 +3550,7 @@
       <c r="A23" s="16">
         <v>66</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="23" t="s">
         <v>134</v>
       </c>
       <c r="C23" s="13" t="s">
@@ -3565,20 +3562,20 @@
       <c r="E23" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F23" s="26">
+      <c r="F23" s="25">
         <v>3</v>
       </c>
       <c r="H23" s="16"/>
       <c r="I23" s="16"/>
       <c r="J23" s="16"/>
       <c r="K23" s="16"/>
-      <c r="L23" s="23" t="s">
+      <c r="L23" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="M23" s="23" t="s">
+      <c r="M23" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="P23" s="23" t="s">
+      <c r="P23" s="22" t="s">
         <v>107</v>
       </c>
       <c r="Q23" s="16">
@@ -3590,7 +3587,7 @@
       <c r="S23" s="16">
         <v>16</v>
       </c>
-      <c r="T23" s="22">
+      <c r="T23" s="21">
         <v>40</v>
       </c>
       <c r="U23" s="16">
@@ -3607,7 +3604,7 @@
       <c r="A24" s="16">
         <v>73</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="23" t="s">
         <v>134</v>
       </c>
       <c r="C24" s="13" t="s">
@@ -3619,20 +3616,20 @@
       <c r="E24" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F24" s="26">
+      <c r="F24" s="25">
         <v>3</v>
       </c>
       <c r="H24" s="16"/>
       <c r="I24" s="16"/>
       <c r="J24" s="16"/>
       <c r="K24" s="16"/>
-      <c r="L24" s="23" t="s">
+      <c r="L24" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="M24" s="23" t="s">
+      <c r="M24" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="P24" s="23" t="s">
+      <c r="P24" s="22" t="s">
         <v>113</v>
       </c>
       <c r="Q24" s="16">
@@ -3644,7 +3641,7 @@
       <c r="S24" s="16">
         <v>18</v>
       </c>
-      <c r="T24" s="22">
+      <c r="T24" s="21">
         <v>50</v>
       </c>
       <c r="U24" s="16">
@@ -3661,7 +3658,7 @@
       <c r="A25" s="16">
         <v>83</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="23" t="s">
         <v>134</v>
       </c>
       <c r="C25" s="13" t="s">
@@ -3673,20 +3670,20 @@
       <c r="E25" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="F25" s="26">
+      <c r="F25" s="25">
         <v>3</v>
       </c>
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
       <c r="J25" s="16"/>
       <c r="K25" s="16"/>
-      <c r="L25" s="23" t="s">
+      <c r="L25" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="M25" s="23" t="s">
+      <c r="M25" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="P25" s="23" t="s">
+      <c r="P25" s="22" t="s">
         <v>115</v>
       </c>
       <c r="Q25" s="16">
@@ -3698,7 +3695,7 @@
       <c r="S25" s="16">
         <v>18</v>
       </c>
-      <c r="T25" s="22">
+      <c r="T25" s="21">
         <v>60</v>
       </c>
       <c r="U25" s="16">
@@ -3717,8 +3714,8 @@
       <c r="J26" s="16"/>
       <c r="K26" s="16"/>
       <c r="L26" s="16"/>
-      <c r="M26" s="23"/>
-      <c r="P26" s="23" t="s">
+      <c r="M26" s="22"/>
+      <c r="P26" s="22" t="s">
         <v>120</v>
       </c>
       <c r="Q26" s="16">
@@ -3730,7 +3727,7 @@
       <c r="S26" s="16">
         <v>18</v>
       </c>
-      <c r="T26" s="22">
+      <c r="T26" s="21">
         <v>75</v>
       </c>
       <c r="U26" s="16">
@@ -3750,7 +3747,7 @@
       <c r="K27" s="16"/>
       <c r="L27" s="16"/>
       <c r="M27" s="16"/>
-      <c r="P27" s="23" t="s">
+      <c r="P27" s="22" t="s">
         <v>123</v>
       </c>
       <c r="Q27" s="16">
@@ -3762,7 +3759,7 @@
       <c r="S27" s="16">
         <v>20</v>
       </c>
-      <c r="T27" s="22">
+      <c r="T27" s="21">
         <v>100</v>
       </c>
       <c r="U27" s="16">
@@ -3776,7 +3773,7 @@
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="18" t="s">
         <v>19</v>
       </c>
       <c r="B28" s="16" t="s">
@@ -3788,7 +3785,7 @@
       <c r="K28" s="16"/>
       <c r="L28" s="16"/>
       <c r="M28" s="16"/>
-      <c r="P28" s="23" t="s">
+      <c r="P28" s="22" t="s">
         <v>129</v>
       </c>
       <c r="Q28" s="16">
@@ -3800,7 +3797,7 @@
       <c r="S28" s="16">
         <v>20</v>
       </c>
-      <c r="T28" s="22">
+      <c r="T28" s="21">
         <v>125</v>
       </c>
       <c r="U28" s="16">
@@ -3826,7 +3823,7 @@
       <c r="K29" s="16"/>
       <c r="L29" s="16"/>
       <c r="M29" s="16"/>
-      <c r="P29" s="23" t="s">
+      <c r="P29" s="22" t="s">
         <v>132</v>
       </c>
       <c r="Q29" s="16">
@@ -3838,7 +3835,7 @@
       <c r="S29" s="16">
         <v>22</v>
       </c>
-      <c r="T29" s="22">
+      <c r="T29" s="21">
         <v>150</v>
       </c>
       <c r="U29" s="16">
@@ -3864,7 +3861,7 @@
       <c r="K30" s="16"/>
       <c r="L30" s="16"/>
       <c r="M30" s="16"/>
-      <c r="P30" s="23" t="s">
+      <c r="P30" s="22" t="s">
         <v>138</v>
       </c>
       <c r="Q30" s="16">
@@ -3876,7 +3873,7 @@
       <c r="S30" s="16">
         <v>22</v>
       </c>
-      <c r="T30" s="22">
+      <c r="T30" s="21">
         <v>175</v>
       </c>
       <c r="U30" s="16">
@@ -3902,7 +3899,7 @@
       <c r="K31" s="16"/>
       <c r="L31" s="16"/>
       <c r="M31" s="16"/>
-      <c r="P31" s="23" t="s">
+      <c r="P31" s="22" t="s">
         <v>141</v>
       </c>
       <c r="Q31" s="16">
@@ -3914,7 +3911,7 @@
       <c r="S31" s="16">
         <v>25</v>
       </c>
-      <c r="T31" s="22">
+      <c r="T31" s="21">
         <v>200</v>
       </c>
       <c r="U31" s="16">
@@ -3934,7 +3931,7 @@
       <c r="K32" s="16"/>
       <c r="L32" s="16"/>
       <c r="M32" s="16"/>
-      <c r="P32" s="23" t="s">
+      <c r="P32" s="22" t="s">
         <v>144</v>
       </c>
       <c r="Q32" s="16">
@@ -3946,7 +3943,7 @@
       <c r="S32" s="16">
         <v>25</v>
       </c>
-      <c r="T32" s="22">
+      <c r="T32" s="21">
         <v>250</v>
       </c>
       <c r="U32" s="16">
@@ -3966,7 +3963,7 @@
       <c r="K33" s="16"/>
       <c r="L33" s="16"/>
       <c r="M33" s="16"/>
-      <c r="P33" s="23" t="s">
+      <c r="P33" s="22" t="s">
         <v>147</v>
       </c>
       <c r="Q33" s="16">
@@ -3978,7 +3975,7 @@
       <c r="S33" s="16">
         <v>25</v>
       </c>
-      <c r="T33" s="22">
+      <c r="T33" s="21">
         <v>300</v>
       </c>
       <c r="U33" s="16">
@@ -3992,7 +3989,7 @@
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A34" s="19" t="s">
+      <c r="A34" s="18" t="s">
         <v>23</v>
       </c>
       <c r="H34" s="16"/>
@@ -4004,7 +4001,7 @@
       <c r="O34" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="P34" s="21" t="s">
+      <c r="P34" s="20" t="s">
         <v>57</v>
       </c>
       <c r="Q34" s="16">
@@ -4016,7 +4013,7 @@
       <c r="S34" s="16">
         <v>5</v>
       </c>
-      <c r="T34" s="22">
+      <c r="T34" s="21">
         <v>0.5</v>
       </c>
       <c r="U34" s="16">
@@ -4039,7 +4036,7 @@
       <c r="K35" s="16"/>
       <c r="L35" s="16"/>
       <c r="M35" s="16"/>
-      <c r="P35" s="23" t="s">
+      <c r="P35" s="22" t="s">
         <v>65</v>
       </c>
       <c r="Q35" s="16">
@@ -4051,7 +4048,7 @@
       <c r="S35" s="16">
         <v>6</v>
       </c>
-      <c r="T35" s="22">
+      <c r="T35" s="21">
         <v>1</v>
       </c>
       <c r="U35" s="16">
@@ -4074,7 +4071,7 @@
       <c r="K36" s="16"/>
       <c r="L36" s="16"/>
       <c r="M36" s="16"/>
-      <c r="P36" s="23" t="s">
+      <c r="P36" s="22" t="s">
         <v>68</v>
       </c>
       <c r="Q36" s="16">
@@ -4086,7 +4083,7 @@
       <c r="S36" s="16">
         <v>8</v>
       </c>
-      <c r="T36" s="22">
+      <c r="T36" s="21">
         <v>1.5</v>
       </c>
       <c r="U36" s="16">
@@ -4103,13 +4100,13 @@
       <c r="A37" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="H37" s="29"/>
-      <c r="I37" s="29"/>
-      <c r="J37" s="29"/>
-      <c r="K37" s="29"/>
-      <c r="L37" s="29"/>
-      <c r="M37" s="29"/>
-      <c r="P37" s="23" t="s">
+      <c r="H37" s="28"/>
+      <c r="I37" s="28"/>
+      <c r="J37" s="28"/>
+      <c r="K37" s="28"/>
+      <c r="L37" s="28"/>
+      <c r="M37" s="28"/>
+      <c r="P37" s="22" t="s">
         <v>75</v>
       </c>
       <c r="Q37" s="16">
@@ -4121,7 +4118,7 @@
       <c r="S37" s="16">
         <v>8</v>
       </c>
-      <c r="T37" s="22">
+      <c r="T37" s="21">
         <v>2</v>
       </c>
       <c r="U37" s="16">
@@ -4141,7 +4138,7 @@
       <c r="K38" s="16"/>
       <c r="L38" s="16"/>
       <c r="M38" s="16"/>
-      <c r="P38" s="23" t="s">
+      <c r="P38" s="22" t="s">
         <v>79</v>
       </c>
       <c r="Q38" s="16">
@@ -4153,7 +4150,7 @@
       <c r="S38" s="16">
         <v>8</v>
       </c>
-      <c r="T38" s="22">
+      <c r="T38" s="21">
         <v>3</v>
       </c>
       <c r="U38" s="16">
@@ -4173,7 +4170,7 @@
       <c r="K39" s="16"/>
       <c r="L39" s="16"/>
       <c r="M39" s="16"/>
-      <c r="P39" s="23" t="s">
+      <c r="P39" s="22" t="s">
         <v>83</v>
       </c>
       <c r="Q39" s="16">
@@ -4185,7 +4182,7 @@
       <c r="S39" s="16">
         <v>8</v>
       </c>
-      <c r="T39" s="22">
+      <c r="T39" s="21">
         <v>5.5</v>
       </c>
       <c r="U39" s="16">
@@ -4199,22 +4196,22 @@
       </c>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A40" s="19" t="s">
+      <c r="A40" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="B40" s="19" t="s">
+      <c r="B40" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="C40" s="19" t="s">
+      <c r="C40" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="D40" s="19" t="s">
+      <c r="D40" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E40" s="19" t="s">
+      <c r="E40" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="F40" s="19" t="s">
+      <c r="F40" s="18" t="s">
         <v>163</v>
       </c>
       <c r="H40" s="16"/>
@@ -4223,7 +4220,7 @@
       <c r="K40" s="16"/>
       <c r="L40" s="16"/>
       <c r="M40" s="16"/>
-      <c r="P40" s="23" t="s">
+      <c r="P40" s="22" t="s">
         <v>86</v>
       </c>
       <c r="Q40" s="16">
@@ -4235,7 +4232,7 @@
       <c r="S40" s="16">
         <v>10</v>
       </c>
-      <c r="T40" s="22">
+      <c r="T40" s="21">
         <v>7.5</v>
       </c>
       <c r="U40" s="16">
@@ -4273,7 +4270,7 @@
       <c r="K41" s="16"/>
       <c r="L41" s="16"/>
       <c r="M41" s="16"/>
-      <c r="P41" s="23" t="s">
+      <c r="P41" s="22" t="s">
         <v>89</v>
       </c>
       <c r="Q41" s="16">
@@ -4285,7 +4282,7 @@
       <c r="S41" s="16">
         <v>10</v>
       </c>
-      <c r="T41" s="22">
+      <c r="T41" s="21">
         <v>10</v>
       </c>
       <c r="U41" s="16">
@@ -4323,7 +4320,7 @@
       <c r="K42" s="16"/>
       <c r="L42" s="16"/>
       <c r="M42" s="16"/>
-      <c r="P42" s="23" t="s">
+      <c r="P42" s="22" t="s">
         <v>91</v>
       </c>
       <c r="Q42" s="16">
@@ -4335,7 +4332,7 @@
       <c r="S42" s="16">
         <v>12</v>
       </c>
-      <c r="T42" s="22">
+      <c r="T42" s="21">
         <v>15</v>
       </c>
       <c r="U42" s="16">
@@ -4362,7 +4359,7 @@
       <c r="K43" s="16"/>
       <c r="L43" s="16"/>
       <c r="M43" s="16"/>
-      <c r="P43" s="23" t="s">
+      <c r="P43" s="22" t="s">
         <v>94</v>
       </c>
       <c r="Q43" s="16">
@@ -4374,7 +4371,7 @@
       <c r="S43" s="16">
         <v>12</v>
       </c>
-      <c r="T43" s="22">
+      <c r="T43" s="21">
         <v>20</v>
       </c>
       <c r="U43" s="16">
@@ -4398,7 +4395,7 @@
       <c r="K44" s="13"/>
       <c r="L44" s="13"/>
       <c r="M44" s="13"/>
-      <c r="P44" s="23" t="s">
+      <c r="P44" s="22" t="s">
         <v>100</v>
       </c>
       <c r="Q44" s="16">
@@ -4410,7 +4407,7 @@
       <c r="S44" s="16">
         <v>14</v>
       </c>
-      <c r="T44" s="22">
+      <c r="T44" s="21">
         <v>25</v>
       </c>
       <c r="U44" s="16">
@@ -4426,7 +4423,7 @@
     <row r="45" spans="4:23" x14ac:dyDescent="0.25">
       <c r="D45" s="16"/>
       <c r="F45" s="13"/>
-      <c r="P45" s="23" t="s">
+      <c r="P45" s="22" t="s">
         <v>102</v>
       </c>
       <c r="Q45" s="16">
@@ -4438,7 +4435,7 @@
       <c r="S45" s="16">
         <v>14</v>
       </c>
-      <c r="T45" s="22">
+      <c r="T45" s="21">
         <v>30</v>
       </c>
       <c r="U45" s="16">
@@ -4452,13 +4449,13 @@
       </c>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A46" s="29"/>
+      <c r="A46" s="28"/>
       <c r="B46" s="15"/>
       <c r="C46" s="16"/>
       <c r="D46" s="16"/>
       <c r="E46" s="16"/>
       <c r="F46" s="13"/>
-      <c r="P46" s="23" t="s">
+      <c r="P46" s="22" t="s">
         <v>108</v>
       </c>
       <c r="Q46" s="16">
@@ -4470,7 +4467,7 @@
       <c r="S46" s="16">
         <v>16</v>
       </c>
-      <c r="T46" s="22">
+      <c r="T46" s="21">
         <v>40</v>
       </c>
       <c r="U46" s="16">
@@ -4484,13 +4481,13 @@
       </c>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A47" s="30" t="s">
+      <c r="A47" s="29" t="s">
         <v>18</v>
       </c>
       <c r="B47" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="P47" s="23" t="s">
+      <c r="P47" s="22" t="s">
         <v>114</v>
       </c>
       <c r="Q47" s="16">
@@ -4502,7 +4499,7 @@
       <c r="S47" s="16">
         <v>16</v>
       </c>
-      <c r="T47" s="22">
+      <c r="T47" s="21">
         <v>50</v>
       </c>
       <c r="U47" s="16">
@@ -4516,13 +4513,13 @@
       </c>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A48" s="29" t="s">
+      <c r="A48" s="28" t="s">
         <v>169</v>
       </c>
       <c r="B48" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="P48" s="23" t="s">
+      <c r="P48" s="22" t="s">
         <v>116</v>
       </c>
       <c r="Q48" s="16">
@@ -4534,7 +4531,7 @@
       <c r="S48" s="16">
         <v>16</v>
       </c>
-      <c r="T48" s="22">
+      <c r="T48" s="21">
         <v>60</v>
       </c>
       <c r="U48" s="16">
@@ -4554,7 +4551,7 @@
       <c r="B49" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="P49" s="23" t="s">
+      <c r="P49" s="22" t="s">
         <v>121</v>
       </c>
       <c r="Q49" s="16">
@@ -4566,7 +4563,7 @@
       <c r="S49" s="16">
         <v>18</v>
       </c>
-      <c r="T49" s="22">
+      <c r="T49" s="21">
         <v>75</v>
       </c>
       <c r="U49" s="16">
@@ -4586,7 +4583,7 @@
       <c r="B50" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="P50" s="23" t="s">
+      <c r="P50" s="22" t="s">
         <v>124</v>
       </c>
       <c r="Q50" s="16">
@@ -4598,7 +4595,7 @@
       <c r="S50" s="16">
         <v>20</v>
       </c>
-      <c r="T50" s="22">
+      <c r="T50" s="21">
         <v>100</v>
       </c>
       <c r="U50" s="16">
@@ -4618,7 +4615,7 @@
       <c r="B51" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="P51" s="23" t="s">
+      <c r="P51" s="22" t="s">
         <v>130</v>
       </c>
       <c r="Q51" s="16">
@@ -4630,7 +4627,7 @@
       <c r="S51" s="16">
         <v>20</v>
       </c>
-      <c r="T51" s="22">
+      <c r="T51" s="21">
         <v>125</v>
       </c>
       <c r="U51" s="16">
@@ -4650,7 +4647,7 @@
       <c r="B52" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="P52" s="23" t="s">
+      <c r="P52" s="22" t="s">
         <v>133</v>
       </c>
       <c r="Q52" s="16">
@@ -4662,7 +4659,7 @@
       <c r="S52" s="16">
         <v>22</v>
       </c>
-      <c r="T52" s="22">
+      <c r="T52" s="21">
         <v>150</v>
       </c>
       <c r="U52" s="16">
@@ -4682,7 +4679,7 @@
       <c r="B53" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="P53" s="23" t="s">
+      <c r="P53" s="22" t="s">
         <v>139</v>
       </c>
       <c r="Q53" s="16">
@@ -4694,7 +4691,7 @@
       <c r="S53" s="16">
         <v>22</v>
       </c>
-      <c r="T53" s="22">
+      <c r="T53" s="21">
         <v>180</v>
       </c>
       <c r="U53" s="16">
@@ -4711,7 +4708,7 @@
       <c r="A54" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="P54" s="23" t="s">
+      <c r="P54" s="22" t="s">
         <v>142</v>
       </c>
       <c r="Q54" s="16">
@@ -4723,7 +4720,7 @@
       <c r="S54" s="16">
         <v>22</v>
       </c>
-      <c r="T54" s="22">
+      <c r="T54" s="21">
         <v>200</v>
       </c>
       <c r="U54" s="16">
@@ -4740,7 +4737,7 @@
       <c r="A55" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="P55" s="23" t="s">
+      <c r="P55" s="22" t="s">
         <v>145</v>
       </c>
       <c r="Q55" s="16">
@@ -4752,7 +4749,7 @@
       <c r="S55" s="16">
         <v>22</v>
       </c>
-      <c r="T55" s="22">
+      <c r="T55" s="21">
         <v>270</v>
       </c>
       <c r="U55" s="16">
@@ -4769,7 +4766,7 @@
       <c r="A56" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="P56" s="23" t="s">
+      <c r="P56" s="22" t="s">
         <v>148</v>
       </c>
       <c r="Q56" s="16">
@@ -4781,7 +4778,7 @@
       <c r="S56" s="16">
         <v>25</v>
       </c>
-      <c r="T56" s="22">
+      <c r="T56" s="21">
         <v>340</v>
       </c>
       <c r="U56" s="16">
@@ -4795,7 +4792,7 @@
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" s="19" t="s">
+      <c r="A59" s="18" t="s">
         <v>22</v>
       </c>
     </row>
@@ -4815,131 +4812,131 @@
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A63" s="31"/>
-      <c r="B63" s="31"/>
-      <c r="C63" s="32"/>
-      <c r="D63" s="32"/>
-      <c r="E63" s="32"/>
-      <c r="F63" s="33"/>
-      <c r="G63" s="33"/>
-      <c r="H63" s="33"/>
-      <c r="I63" s="33"/>
-      <c r="J63" s="33"/>
-      <c r="K63" s="33"/>
-      <c r="L63" s="33"/>
-      <c r="M63" s="33"/>
-      <c r="N63" s="33"/>
-      <c r="O63" s="33"/>
-      <c r="P63" s="33"/>
-      <c r="Q63" s="33"/>
-      <c r="R63" s="33"/>
-      <c r="S63" s="33"/>
-      <c r="T63" s="34"/>
-      <c r="U63" s="34"/>
-      <c r="V63" s="33"/>
-      <c r="W63" s="34"/>
-      <c r="X63" s="33"/>
+      <c r="A63" s="30"/>
+      <c r="B63" s="30"/>
+      <c r="C63" s="31"/>
+      <c r="D63" s="31"/>
+      <c r="E63" s="31"/>
+      <c r="F63" s="32"/>
+      <c r="G63" s="32"/>
+      <c r="H63" s="32"/>
+      <c r="I63" s="32"/>
+      <c r="J63" s="32"/>
+      <c r="K63" s="32"/>
+      <c r="L63" s="32"/>
+      <c r="M63" s="32"/>
+      <c r="N63" s="32"/>
+      <c r="O63" s="32"/>
+      <c r="P63" s="32"/>
+      <c r="Q63" s="32"/>
+      <c r="R63" s="32"/>
+      <c r="S63" s="32"/>
+      <c r="T63" s="33"/>
+      <c r="U63" s="33"/>
+      <c r="V63" s="32"/>
+      <c r="W63" s="33"/>
+      <c r="X63" s="32"/>
     </row>
     <row r="64" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="35" t="s">
+      <c r="A64" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="B64" s="36"/>
+      <c r="B64" s="35"/>
       <c r="C64" s="13" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B65" s="38">
+      <c r="A65" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B65" s="37">
         <v>46168</v>
       </c>
-      <c r="C65" s="39" t="s">
+      <c r="C65" s="38" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="40" t="s">
+      <c r="A66" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="B66" s="41" t="s">
+      <c r="B66" s="40" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="40" t="s">
+      <c r="A67" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="B67" s="42" t="s">
+      <c r="B67" s="41" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="40" t="s">
+      <c r="A68" s="39" t="s">
         <v>149</v>
       </c>
-      <c r="B68" s="42" t="s">
+      <c r="B68" s="41" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="40" t="s">
+      <c r="A69" s="39" t="s">
         <v>192</v>
       </c>
-      <c r="B69" s="43">
+      <c r="B69" s="42">
         <v>46179</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="40" t="s">
+      <c r="A70" s="39" t="s">
         <v>193</v>
       </c>
-      <c r="B70" s="42">
+      <c r="B70" s="41">
         <v>2</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="40" t="s">
+      <c r="A71" s="39" t="s">
         <v>194</v>
       </c>
-      <c r="B71" s="42" t="s">
+      <c r="B71" s="41" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="40" t="s">
+      <c r="A72" s="39" t="s">
         <v>196</v>
       </c>
-      <c r="B72" s="42">
+      <c r="B72" s="41">
         <v>14</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="44" t="s">
+      <c r="A73" s="43" t="s">
         <v>197</v>
       </c>
-      <c r="B73" s="45">
+      <c r="B73" s="44">
         <v>10</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="75" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="46" t="s">
+      <c r="A75" s="45" t="s">
         <v>198</v>
       </c>
-      <c r="B75" s="47"/>
-      <c r="C75" s="31" t="s">
+      <c r="B75" s="46"/>
+      <c r="C75" s="30" t="s">
         <v>199</v>
       </c>
-      <c r="D75" s="34"/>
+      <c r="D75" s="33"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="37" t="s">
+      <c r="A76" s="36" t="s">
         <v>200</v>
       </c>
-      <c r="B76" s="48" t="str">
+      <c r="B76" s="47" t="str">
         <f>VLOOKUP(B67,B67,1)</f>
         <v>CEB</v>
       </c>
@@ -4952,13 +4949,13 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="49" t="s">
+      <c r="A77" s="48" t="s">
         <v>51</v>
       </c>
-      <c r="B77" s="50">
+      <c r="B77" s="49">
         <v>44.5</v>
       </c>
-      <c r="C77" s="29" t="s">
+      <c r="C77" s="28" t="s">
         <v>31</v>
       </c>
       <c r="D77" s="16" t="str">
@@ -4967,13 +4964,13 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="49" t="s">
+      <c r="A78" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="B78" s="42" t="s">
+      <c r="B78" s="41" t="s">
         <v>169</v>
       </c>
-      <c r="C78" s="29" t="s">
+      <c r="C78" s="28" t="s">
         <v>33</v>
       </c>
       <c r="D78" s="16" t="str">
@@ -4982,13 +4979,13 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="49" t="s">
+      <c r="A79" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="B79" s="42" t="s">
+      <c r="B79" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="C79" s="29" t="s">
+      <c r="C79" s="28" t="s">
         <v>30</v>
       </c>
       <c r="D79" s="16" t="str">
@@ -4997,13 +4994,13 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="49" t="s">
+      <c r="A80" s="48" t="s">
         <v>202</v>
       </c>
-      <c r="B80" s="42" t="s">
+      <c r="B80" s="41" t="s">
         <v>150</v>
       </c>
-      <c r="C80" s="29" t="s">
+      <c r="C80" s="28" t="s">
         <v>31</v>
       </c>
       <c r="D80" s="16" t="str">
@@ -5012,13 +5009,13 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="49" t="s">
+      <c r="A81" s="48" t="s">
         <v>203</v>
       </c>
-      <c r="B81" s="42" t="s">
+      <c r="B81" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="C81" s="29" t="s">
+      <c r="C81" s="28" t="s">
         <v>204</v>
       </c>
       <c r="D81" s="16">
@@ -5027,28 +5024,28 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="40" t="s">
+      <c r="A82" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="B82" s="42" t="s">
+      <c r="B82" s="41" t="s">
         <v>205</v>
       </c>
       <c r="D82" s="16"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="40" t="s">
+      <c r="A83" s="39" t="s">
         <v>206</v>
       </c>
-      <c r="B83" s="42" t="s">
+      <c r="B83" s="41" t="s">
         <v>207</v>
       </c>
       <c r="D83" s="16"/>
     </row>
     <row r="84" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="44" t="s">
+      <c r="A84" s="43" t="s">
         <v>208</v>
       </c>
-      <c r="B84" s="45">
+      <c r="B84" s="44">
         <v>595</v>
       </c>
       <c r="D84" s="16"/>
@@ -5057,38 +5054,38 @@
       <c r="D85" s="16"/>
     </row>
     <row r="86" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="46" t="s">
+      <c r="A86" s="45" t="s">
         <v>209</v>
       </c>
-      <c r="B86" s="47"/>
-      <c r="C86" s="31" t="s">
+      <c r="B86" s="46"/>
+      <c r="C86" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="D86" s="34"/>
+      <c r="D86" s="33"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="51" t="s">
+      <c r="A87" s="50" t="s">
         <v>211</v>
       </c>
-      <c r="B87" s="52" t="s">
+      <c r="B87" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="C87" s="29" t="s">
+      <c r="C87" s="28" t="s">
         <v>212</v>
       </c>
-      <c r="D87" s="53">
+      <c r="D87" s="52">
         <f>VLOOKUP(TRIM(B89),P3:W56,5,FALSE)</f>
         <v>15</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="49" t="s">
+      <c r="A88" s="48" t="s">
         <v>213</v>
       </c>
-      <c r="B88" s="42" t="s">
+      <c r="B88" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="C88" s="29" t="s">
+      <c r="C88" s="28" t="s">
         <v>214</v>
       </c>
       <c r="D88" s="16">
@@ -5097,25 +5094,25 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="49" t="s">
+      <c r="A89" s="48" t="s">
         <v>212</v>
       </c>
-      <c r="B89" s="42" t="s">
+      <c r="B89" s="41" t="s">
         <v>91</v>
       </c>
       <c r="C89" s="16" t="s">
         <v>215</v>
       </c>
-      <c r="D89" s="54">
+      <c r="D89" s="53">
         <f>VLOOKUP(TRIM(B89),P3:W56,2,FALSE)</f>
         <v>1728</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="49" t="s">
+      <c r="A90" s="48" t="s">
         <v>160</v>
       </c>
-      <c r="B90" s="42">
+      <c r="B90" s="41">
         <v>220</v>
       </c>
       <c r="C90" s="16" t="s">
@@ -5127,10 +5124,10 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="40" t="s">
+      <c r="A91" s="39" t="s">
         <v>161</v>
       </c>
-      <c r="B91" s="42">
+      <c r="B91" s="41">
         <v>60</v>
       </c>
       <c r="C91" s="16" t="s">
@@ -5142,10 +5139,10 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="40" t="s">
+      <c r="A92" s="39" t="s">
         <v>162</v>
       </c>
-      <c r="B92" s="42" t="s">
+      <c r="B92" s="41" t="s">
         <v>164</v>
       </c>
       <c r="C92" s="16" t="s">
@@ -5157,13 +5154,13 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="40" t="s">
+      <c r="A93" s="39" t="s">
         <v>163</v>
       </c>
-      <c r="B93" s="42" t="s">
+      <c r="B93" s="41" t="s">
         <v>165</v>
       </c>
-      <c r="C93" s="29" t="s">
+      <c r="C93" s="28" t="s">
         <v>28</v>
       </c>
       <c r="D93" s="16" t="str">
@@ -5172,14 +5169,14 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="40" t="s">
+      <c r="A94" s="39" t="s">
         <v>215</v>
       </c>
-      <c r="B94" s="55">
+      <c r="B94" s="54">
         <f>VLOOKUP(D89,D89,1)</f>
         <v>1728</v>
       </c>
-      <c r="C94" s="29" t="s">
+      <c r="C94" s="28" t="s">
         <v>218</v>
       </c>
       <c r="D94" s="16">
@@ -5188,10 +5185,10 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="40" t="s">
+      <c r="A95" s="39" t="s">
         <v>208</v>
       </c>
-      <c r="B95" s="55">
+      <c r="B95" s="54">
         <f>VLOOKUP(B84,B84,1)</f>
         <v>595</v>
       </c>
@@ -5204,26 +5201,26 @@
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96" s="40" t="s">
+      <c r="A96" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="B96" s="56">
+      <c r="B96" s="55">
         <v>4.5</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" s="40" t="s">
+      <c r="A97" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="B97" s="56">
+      <c r="B97" s="55">
         <v>13</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" s="44" t="s">
+      <c r="A98" s="43" t="s">
         <v>201</v>
       </c>
-      <c r="B98" s="57">
+      <c r="B98" s="56">
         <f>VLOOKUP(D76,D76,1)</f>
         <v>598.1538461538462</v>
       </c>

</xml_diff>

<commit_message>
JO: left-align only the Capacity line (C40), nothing else touched
Add one left-aligned cell style and point C40 at it via zip-surgery; the
other 113 cells sharing the old style, the drawing, and all else are unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HNv2pt2j3pqxEC7sBHUC3k
</commit_message>
<xml_diff>
--- a/public/templates/fans-jo-template.xlsx
+++ b/public/templates/fans-jo-template.xlsx
@@ -856,7 +856,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1014,6 +1014,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1784,7 +1787,7 @@
       <c r="B40" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C40" s="3">
+      <c r="C40" s="57">
         <f>Source!B82&amp;"        "&amp;Source!B83</f>
       </c>
       <c r="D40" s="3"/>

</xml_diff>

<commit_message>
JO: revert C40 back to centered
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HNv2pt2j3pqxEC7sBHUC3k
</commit_message>
<xml_diff>
--- a/public/templates/fans-jo-template.xlsx
+++ b/public/templates/fans-jo-template.xlsx
@@ -856,7 +856,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1014,9 +1014,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1787,7 +1784,7 @@
       <c r="B40" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C40" s="57">
+      <c r="C40" s="3">
         <f>Source!B82&amp;"        "&amp;Source!B83</f>
       </c>
       <c r="D40" s="3"/>

</xml_diff>

<commit_message>
JO: color the five secondary values red (split each concat line into black + red cells)
</commit_message>
<xml_diff>
--- a/public/templates/fans-jo-template.xlsx
+++ b/public/templates/fans-jo-template.xlsx
@@ -856,7 +856,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1014,6 +1014,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="12" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1784,8 +1793,8 @@
       <c r="B40" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C40" s="3">
-        <f>Source!B82&amp;"        "&amp;Source!B83</f>
+      <c r="C40" s="57">
+        <f>Source!B82</f>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
@@ -1796,7 +1805,9 @@
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
-      <c r="M40" s="3"/>
+      <c r="M40" s="59">
+        <f>" "&amp;Source!B83</f>
+      </c>
       <c r="N40" s="3"/>
       <c r="O40" s="3"/>
       <c r="P40" s="3"/>
@@ -1844,8 +1855,8 @@
       <c r="B42" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C42" s="3">
-        <f>Source!B84&amp;" rpm        "&amp;ROUNDUP(Source!D76,0)&amp;" rpm"</f>
+      <c r="C42" s="57">
+        <f>Source!B84&amp;" rpm"</f>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
@@ -1856,7 +1867,9 @@
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
-      <c r="M42" s="3"/>
+      <c r="M42" s="59">
+        <f>" "&amp;ROUNDUP(Source!D76,0)&amp;" rpm"</f>
+      </c>
       <c r="N42" s="3"/>
       <c r="O42" s="3"/>
       <c r="P42" s="3"/>
@@ -1962,8 +1975,8 @@
       <c r="B46" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C46" s="15">
-        <f>TRIM(TEXT(Source!B96,"# ?/?"))&amp;""" Ø x "&amp;Source!D93&amp;" x "&amp;Source!D91&amp;" mm Ø bore x "&amp;Source!D92&amp;" mm keyway        "&amp;Source!D94&amp;" mm Ø Hub"</f>
+      <c r="C46" s="58">
+        <f>TRIM(TEXT(Source!B96,"# ?/?"))&amp;""" Ø x "&amp;Source!D93&amp;" x "&amp;Source!D91&amp;" mm Ø bore x "&amp;Source!D92&amp;" mm keyway"</f>
       </c>
       <c r="D46" s="15"/>
       <c r="E46" s="15"/>
@@ -1978,7 +1991,9 @@
       <c r="N46" s="15"/>
       <c r="O46" s="15"/>
       <c r="P46" s="15"/>
-      <c r="Q46" s="15"/>
+      <c r="Q46" s="59">
+        <f>" "&amp;Source!D94&amp;" mm Ø Hub"</f>
+      </c>
       <c r="R46" s="15"/>
       <c r="S46" s="15"/>
       <c r="T46" s="15"/>
@@ -2021,8 +2036,8 @@
       <c r="B48" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C48" s="15">
-        <f>TRIM(TEXT(Source!B97,"# ?/?"))&amp;""" Ø x "&amp;Source!D93&amp;" x "&amp;Source!D80&amp;"        "&amp;Source!D95&amp;" mm Ø Hub"</f>
+      <c r="C48" s="58">
+        <f>TRIM(TEXT(Source!B97,"# ?/?"))&amp;""" Ø x "&amp;Source!D93&amp;" x "&amp;Source!D80</f>
       </c>
       <c r="D48" s="15"/>
       <c r="E48" s="15"/>
@@ -2037,7 +2052,9 @@
       <c r="N48" s="15"/>
       <c r="O48" s="15"/>
       <c r="P48" s="15"/>
-      <c r="Q48" s="15"/>
+      <c r="Q48" s="59">
+        <f>" "&amp;Source!D95&amp;" mm Ø Hub"</f>
+      </c>
       <c r="R48" s="15"/>
       <c r="S48" s="15"/>
       <c r="T48" s="15"/>
@@ -2260,8 +2277,8 @@
       <c r="B56" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C56" s="3">
-        <f>Source!D78&amp;"     --     "&amp;SUM(Source!B70)*2&amp;" pcs"</f>
+      <c r="C56" s="57">
+        <f>Source!D78&amp;"  --"</f>
       </c>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
@@ -2272,7 +2289,9 @@
       <c r="J56" s="3"/>
       <c r="K56" s="3"/>
       <c r="L56" s="3"/>
-      <c r="M56" s="3"/>
+      <c r="M56" s="59">
+        <f>" "&amp;SUM(Source!B70)*2&amp;" pcs"</f>
+      </c>
       <c r="N56" s="3"/>
       <c r="O56" s="3"/>
       <c r="P56" s="3"/>
@@ -2327,7 +2346,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <mergeCells count="24">
+  <mergeCells count="29">
     <mergeCell ref="A12:W12"/>
     <mergeCell ref="D13:K13"/>
     <mergeCell ref="S13:V13"/>
@@ -2342,15 +2361,20 @@
     <mergeCell ref="C38:N38"/>
     <mergeCell ref="O38:P38"/>
     <mergeCell ref="R38:V38"/>
-    <mergeCell ref="C40:V40"/>
-    <mergeCell ref="C42:V42"/>
+    <mergeCell ref="C40:L40"/>
+    <mergeCell ref="M40:V40"/>
+    <mergeCell ref="C42:L42"/>
+    <mergeCell ref="M42:V42"/>
     <mergeCell ref="C44:V44"/>
-    <mergeCell ref="C46:V46"/>
-    <mergeCell ref="C48:V48"/>
+    <mergeCell ref="C46:P46"/>
+    <mergeCell ref="Q46:V46"/>
+    <mergeCell ref="C48:P48"/>
+    <mergeCell ref="Q48:V48"/>
     <mergeCell ref="C50:P50"/>
     <mergeCell ref="D52:M52"/>
     <mergeCell ref="C54:I54"/>
-    <mergeCell ref="C56:V56"/>
+    <mergeCell ref="C56:L56"/>
+    <mergeCell ref="M56:V56"/>
     <mergeCell ref="S58:W58"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
JO: center-align the five split value lines; make (make) parenthetical red in header
</commit_message>
<xml_diff>
--- a/public/templates/fans-jo-template.xlsx
+++ b/public/templates/fans-jo-template.xlsx
@@ -766,6 +766,12 @@
       <family val="2"/>
       <sz val="11"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -856,7 +862,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1022,6 +1028,12 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1540,8 +1552,8 @@
       <c r="B15" t="s">
         <v>2</v>
       </c>
-      <c r="C15" s="7">
-        <f>Source!B70&amp;" "&amp;Source!B71&amp;"   "&amp;Source!B77&amp;""" Ø   "&amp;Source!B67&amp;"   ("&amp;Source!B68&amp;")"</f>
+      <c r="C15" s="60">
+        <f>Source!B70&amp;" "&amp;Source!B71&amp;"   "&amp;Source!B77&amp;""" Ø   "&amp;Source!B67</f>
       </c>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
@@ -1556,7 +1568,9 @@
       <c r="N15" s="7"/>
       <c r="O15" s="7"/>
       <c r="P15" s="7"/>
-      <c r="Q15" s="7"/>
+      <c r="Q15" s="61">
+        <f>"   ("&amp;Source!B68&amp;")"</f>
+      </c>
       <c r="R15" s="7"/>
       <c r="S15" s="7"/>
       <c r="T15" s="7"/>
@@ -1793,7 +1807,7 @@
       <c r="B40" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C40" s="57">
+      <c r="C40" s="3">
         <f>Source!B82</f>
       </c>
       <c r="D40" s="3"/>
@@ -1855,7 +1869,7 @@
       <c r="B42" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C42" s="57">
+      <c r="C42" s="3">
         <f>Source!B84&amp;" rpm"</f>
       </c>
       <c r="D42" s="3"/>
@@ -1975,7 +1989,7 @@
       <c r="B46" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C46" s="58">
+      <c r="C46" s="15">
         <f>TRIM(TEXT(Source!B96,"# ?/?"))&amp;""" Ø x "&amp;Source!D93&amp;" x "&amp;Source!D91&amp;" mm Ø bore x "&amp;Source!D92&amp;" mm keyway"</f>
       </c>
       <c r="D46" s="15"/>
@@ -2036,7 +2050,7 @@
       <c r="B48" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C48" s="58">
+      <c r="C48" s="15">
         <f>TRIM(TEXT(Source!B97,"# ?/?"))&amp;""" Ø x "&amp;Source!D93&amp;" x "&amp;Source!D80</f>
       </c>
       <c r="D48" s="15"/>
@@ -2277,7 +2291,7 @@
       <c r="B56" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C56" s="57">
+      <c r="C56" s="3">
         <f>Source!D78&amp;"  --"</f>
       </c>
       <c r="D56" s="3"/>
@@ -2346,11 +2360,12 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <mergeCells count="29">
+  <mergeCells count="30">
     <mergeCell ref="A12:W12"/>
     <mergeCell ref="D13:K13"/>
     <mergeCell ref="S13:V13"/>
-    <mergeCell ref="C15:V15"/>
+    <mergeCell ref="C15:P15"/>
+    <mergeCell ref="Q15:V15"/>
     <mergeCell ref="C17:G17"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="H20:I20"/>

</xml_diff>

<commit_message>
JO: set header cells C15/Q15 to Arial 11
</commit_message>
<xml_diff>
--- a/public/templates/fans-jo-template.xlsx
+++ b/public/templates/fans-jo-template.xlsx
@@ -1552,7 +1552,7 @@
       <c r="B15" t="s">
         <v>2</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="3">
         <f>Source!B70&amp;" "&amp;Source!B71&amp;"   "&amp;Source!B77&amp;""" Ø   "&amp;Source!B67</f>
       </c>
       <c r="D15" s="7"/>
@@ -1568,7 +1568,7 @@
       <c r="N15" s="7"/>
       <c r="O15" s="7"/>
       <c r="P15" s="7"/>
-      <c r="Q15" s="61">
+      <c r="Q15" s="59">
         <f>"   ("&amp;Source!B68&amp;")"</f>
       </c>
       <c r="R15" s="7"/>

</xml_diff>